<commit_message>
initial commit for SG3600UD-MV Safety quiz
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8886BF74-5E12-504A-BB70-FD9B30E12318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEE2AD7-9716-8248-9AA0-A6ECE0F18547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-39820" yWindow="780" windowWidth="36880" windowHeight="21600" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="-39820" yWindow="800" windowWidth="36880" windowHeight="21600" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="92">
   <si>
     <t>Question Text</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Multi</t>
   </si>
   <si>
-    <t>Text</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
@@ -71,166 +68,6 @@
     <t>D</t>
   </si>
   <si>
-    <t>What is the minimum category of FR PPE needed to perform the LOTO on SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>Where do you configure the open loop mode on the SG3600UD-MV HMI?</t>
-  </si>
-  <si>
-    <t>Overview -&gt; Management -&gt; Device Operation</t>
-  </si>
-  <si>
-    <t>Function -&gt; Set - Parameter -&gt; Password 1111 -&gt; run-parameter</t>
-  </si>
-  <si>
-    <t>Function -&gt; Set-Parameter-&gt;Password 4040</t>
-  </si>
-  <si>
-    <t>Function -&gt; Run info -&gt; Inv Unit</t>
-  </si>
-  <si>
-    <t>What is the correct password to log on SG3600UD-MV inverter web portal?</t>
-  </si>
-  <si>
-    <t>pw1111</t>
-  </si>
-  <si>
-    <t>dp@ems200</t>
-  </si>
-  <si>
-    <t>adamg1</t>
-  </si>
-  <si>
-    <t>What is the maximum DC input voltage of SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>630V</t>
-  </si>
-  <si>
-    <t>800V</t>
-  </si>
-  <si>
-    <t>955V</t>
-  </si>
-  <si>
-    <t>1500V</t>
-  </si>
-  <si>
-    <t>Which of the following is the default IP address of the NET1 port of SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>192.168.13.100</t>
-  </si>
-  <si>
-    <t>192.168.0.100</t>
-  </si>
-  <si>
-    <t>14.14.14.14</t>
-  </si>
-  <si>
-    <t>12.12.12.12</t>
-  </si>
-  <si>
-    <t>What communication interface does the SG3600UD-MV inverter use to communicate with the IGBT Coolign fans?</t>
-  </si>
-  <si>
-    <t>CAN</t>
-  </si>
-  <si>
-    <t>Ethernet</t>
-  </si>
-  <si>
-    <t>MPLC</t>
-  </si>
-  <si>
-    <t>RS485</t>
-  </si>
-  <si>
-    <t>What is the proper path to access and change values for the protection parameters in the SG3600UD-MV UMCG web portal?</t>
-  </si>
-  <si>
-    <t>Monitoring -&gt; Param. Setting -&gt; Pro-param</t>
-  </si>
-  <si>
-    <t>Monitoring -&gt; Param. Setting -&gt; Pro-param. -&gt; Setting -&gt; Confirm</t>
-  </si>
-  <si>
-    <t>Function -&gt; Set-Param. -&gt; Password 1111 -&gt; Pro-parameter</t>
-  </si>
-  <si>
-    <t>Management -&gt; Param. Setting -&gt; Pro-param. -&gt; Setting -&gt; Confirm</t>
-  </si>
-  <si>
-    <t>What is the proper path to export historical data in the SG3600UD-MV UMCG web portal?</t>
-  </si>
-  <si>
-    <t>Monitoring -&gt; Data Display -&gt; Historical Data -&gt; Export</t>
-  </si>
-  <si>
-    <t>Management -&gt; Device Operation -&gt; Historical Data -&gt; Export</t>
-  </si>
-  <si>
-    <t>Maintenance -&gt; Historical Data -&gt; Export</t>
-  </si>
-  <si>
-    <t>Function -&gt; History Information -&gt; His-Data -&gt; Export</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Before a firmware upgrade, which of the following </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">is not </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>a required screenshot?</t>
-    </r>
-  </si>
-  <si>
-    <t>Settings -&gt; DI Settings</t>
-  </si>
-  <si>
-    <t>Management -&gt; Device Operation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Settings -&gt; About </t>
-  </si>
-  <si>
-    <t>What are the potential causes of a power module fault?</t>
-  </si>
-  <si>
-    <t>Hardware overcurrent event</t>
-  </si>
-  <si>
-    <t>High transformer oil temperature</t>
-  </si>
-  <si>
-    <t>Fan communication error</t>
-  </si>
-  <si>
-    <t>Driver board fault signal</t>
-  </si>
-  <si>
-    <t>A, D</t>
-  </si>
-  <si>
-    <t>What are the possible energy/voltage sources for the SG3600UD-MV inverter?</t>
-  </si>
-  <si>
     <t>Wind Power</t>
   </si>
   <si>
@@ -252,80 +89,236 @@
     <t>BESS</t>
   </si>
   <si>
-    <t>AC and DC capacitors</t>
-  </si>
-  <si>
     <t>B, D, E, F</t>
   </si>
   <si>
-    <t>Which of the following components/locations need to be checked for oil leakage during MVT commissioning and routine maintenance?</t>
-  </si>
-  <si>
-    <t>HV Bushings</t>
-  </si>
-  <si>
-    <t>Tap Changer</t>
-  </si>
-  <si>
-    <t>Oil Thermostat</t>
-  </si>
-  <si>
-    <t>Pressure Relief Device</t>
-  </si>
-  <si>
-    <t>A, B, C, D</t>
-  </si>
-  <si>
-    <t>The SG3600UD-MV only contains one of which of the following boards (i.e. only one board for the entire inverter unit?)</t>
-  </si>
-  <si>
-    <t>PA</t>
-  </si>
-  <si>
-    <t>PE</t>
-  </si>
-  <si>
-    <t>PL</t>
-  </si>
-  <si>
-    <t>PG</t>
-  </si>
-  <si>
-    <t>PT</t>
-  </si>
-  <si>
-    <t>B, E</t>
-  </si>
-  <si>
-    <t>After the inverter is powered off, voltage measurement can be performed immediately.</t>
-  </si>
-  <si>
-    <t>In case of extreme weather conditions like sandstorms, thunderstorms, hgih winds, hail, inverter cabinet doors can still be opened.</t>
-  </si>
-  <si>
-    <t>The SG3600UD-MV inverter has a DC startup voltage of 955V.</t>
-  </si>
-  <si>
-    <t>If there is no incident energy sticker found on the power distribution/aux cabinet, I am permitted to acces it while the skid is energized, as long as I have on a CAT4 suit.</t>
-  </si>
-  <si>
-    <t>Summarize the power cycle procedure for the SG3600UD-MV inverter, including shutdown and power up. Be sure to include all the steps and voltage measurement points.</t>
-  </si>
-  <si>
-    <t>Describe the process of connecting to the SG3600UD-MV UMCG (web portal). Please make note of the IP address(es)</t>
-  </si>
-  <si>
-    <t>Summarize the proces of replacing a specific power stack for the fault message "Power Module Fault" from the HMI. Please include the details for the identification process and the general procedure to replace the physical power stack.</t>
-  </si>
-  <si>
-    <t>Describe the E-stop functionality and describe a recommended procedure to safely test the functionality of the E-STOP without damaging the inverter.</t>
+    <t>On a customer site, what is the LOTO document that should ultimatly be implemented?</t>
+  </si>
+  <si>
+    <t>The site's LOTO procedure document</t>
+  </si>
+  <si>
+    <t>Sungrow PV LOTO guidance document</t>
+  </si>
+  <si>
+    <t>Best judgement</t>
+  </si>
+  <si>
+    <t>SG3600UD Power Cycle MOP</t>
+  </si>
+  <si>
+    <t>There is no incident eenrgy label on the SG3600UD auxiliary cabinet. I can still access the auxiliary cabinet while it is energized, as long as I have on the appropriate PPE</t>
+  </si>
+  <si>
+    <t>Testing the DC Busbars in one inverter unit for de-energyzation is sufficient to prove DC busbar de-energization for both inverter units.</t>
+  </si>
+  <si>
+    <t>Which of the following people are permitted to operate MVT Load Switch of the SG3600UD-MV?</t>
+  </si>
+  <si>
+    <t>Sungrow Employees</t>
+  </si>
+  <si>
+    <t>Sungrow Vendors/Sub-contractors</t>
+  </si>
+  <si>
+    <t>Site Personnel</t>
+  </si>
+  <si>
+    <t>All of the above</t>
+  </si>
+  <si>
+    <t>The proper first step to de-energize the SG3600UD-MV is to….</t>
+  </si>
+  <si>
+    <t>Open the MVT Load Switch</t>
+  </si>
+  <si>
+    <t>Open the DC door knob switch</t>
+  </si>
+  <si>
+    <t>Send a key stop command for the inverter</t>
+  </si>
+  <si>
+    <t>Disconnect the combiner boxes</t>
+  </si>
+  <si>
+    <t>I have turned off all the appropriate switches in the power down procedure, and have waited 24 hours. I may work on the units with the assumption that they are now in a de-energized state.</t>
+  </si>
+  <si>
+    <t>Closing the DC knob switch on the SG3600UD inverter unit will automatically close the DC load break switches.</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>It depends</t>
+  </si>
+  <si>
+    <t>Is it required for someone on-site to open the combiner boxes, even at night, to safely perform de-energized work on the SG3600UD-MV?</t>
+  </si>
+  <si>
+    <t>AC Capacitor de-energization testing should include which of the following tests on a multimeter?</t>
+  </si>
+  <si>
+    <t>Capacitance</t>
+  </si>
+  <si>
+    <t>DC Voltage</t>
+  </si>
+  <si>
+    <t>DC Voltage and AC Voltage</t>
+  </si>
+  <si>
+    <t>DC Voltage and AC Voltage and Capacitance</t>
+  </si>
+  <si>
+    <t>Checking the AC Capacitors for just one unit on the SG3600UD-MV is sufficient to confirm all AC capacitors have discharged.</t>
+  </si>
+  <si>
+    <t>Sungrow employees and/or sub-contractors shall not operate DC Field Disconnects (DC Combiners or LBDs) on site.</t>
+  </si>
+  <si>
+    <t>What document should be referenced to safely power on the SG3600UD-MV?</t>
+  </si>
+  <si>
+    <t>SG3600UD-MV System Manual</t>
+  </si>
+  <si>
+    <t>SG3600UD-MV Power Cycle MOP</t>
+  </si>
+  <si>
+    <t>Common Sense</t>
+  </si>
+  <si>
+    <t>PV LOTO Guidance document</t>
+  </si>
+  <si>
+    <t>How many minutes, at a minimum, do I need to wait after turning off the appropriate swiches on the SG3600UD-MV skid to test for de-energization?</t>
+  </si>
+  <si>
+    <t>10 minutes</t>
+  </si>
+  <si>
+    <t>20 minutes</t>
+  </si>
+  <si>
+    <t>1 minute</t>
+  </si>
+  <si>
+    <t>5 minutes</t>
+  </si>
+  <si>
+    <t>How many qualified employees are needed to perform the shutdown and de-energization verification testing on the SG3600UD-MV?</t>
+  </si>
+  <si>
+    <t>What class of gloves are needed to perform de-energization verification testing on the SG3600UD-MV?</t>
+  </si>
+  <si>
+    <t>Testing for AC common bussing de-energization at one of the valid testing locations is sufficient to prove LV AC common bussing de-energization for the whole SG3600UD-MV skid.</t>
+  </si>
+  <si>
+    <t>How many main AC circuit breakers should open up in the SG3600UD-MV with a key stop command for the entire skid?</t>
+  </si>
+  <si>
+    <t>A safety second is required when working on voltages above which level?</t>
+  </si>
+  <si>
+    <t>Given that the unit is completely de-energized and LOTO'd according to the power-down procedure, what are the first two switches to turn on for the SG3600UD-MV power-on procedure?</t>
+  </si>
+  <si>
+    <t>QS5 and QS6</t>
+  </si>
+  <si>
+    <t>QS9 and QF1</t>
+  </si>
+  <si>
+    <t>QS2 and MVT Load Switch</t>
+  </si>
+  <si>
+    <t>None of the above</t>
+  </si>
+  <si>
+    <t>Sungrow does not require indicidual DC Load Switches and AC Breakers to be LOTO'd.</t>
+  </si>
+  <si>
+    <t>I need to replace a power stack/power module in Unit 2 of the SG3600UD-MV skid. As long as I test for de-energization of the AC common bussing and all the appropriate testing checks within Unit 2, I can proceed with the replacement procedure.</t>
+  </si>
+  <si>
+    <t>The best method to do a functional test of the E-stop button will be during a real-life operating circumstance, such as when the inverter is pushing 100% output power to the grid.</t>
+  </si>
+  <si>
+    <t>Under which of the below following conditions may the AC side fo the SG3600UD-MV inverter units be opened up to test for de-energization? The donned PPE matches the incident energy label requirement.</t>
+  </si>
+  <si>
+    <t>As long as the inverter is shutdown via the HMI or web portal</t>
+  </si>
+  <si>
+    <t>If the combiners and MVT load switch have been opened</t>
+  </si>
+  <si>
+    <t>if I have pressed the E-stop button and 20 minutes have elapsed afterwards</t>
+  </si>
+  <si>
+    <t>If all the appropriate switches in accordance with the power down procedure have been opened up, with 5 minutes having elapsed afterwards.</t>
+  </si>
+  <si>
+    <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, the inverter cabinet doors can still be opened.</t>
+  </si>
+  <si>
+    <t>QS1</t>
+  </si>
+  <si>
+    <t>QS2</t>
+  </si>
+  <si>
+    <t>QS3</t>
+  </si>
+  <si>
+    <t>QS4</t>
+  </si>
+  <si>
+    <t>Which of the following DC Load Switches are present on every single SG3600UD-MV inverter?</t>
+  </si>
+  <si>
+    <t>A, C</t>
+  </si>
+  <si>
+    <t>What are all the potential energy/voltage sources to isolate from / allow to discharge during de-energization of the SG3600UD-MV inverters?</t>
+  </si>
+  <si>
+    <t>AC and DC Capacitors</t>
+  </si>
+  <si>
+    <t>Which of the following testing locations need to be checked to confirm de-energization on the DC side of the SG3600UD-MV inverter?</t>
+  </si>
+  <si>
+    <t>FU29 and FU30</t>
+  </si>
+  <si>
+    <t>AC SPD circuit, before the fuses. Either in Aux cabinet or in Unit 1</t>
+  </si>
+  <si>
+    <t>DC busbars leading into the DC Load Switches</t>
+  </si>
+  <si>
+    <t>FU16, FU17, and FU18</t>
+  </si>
+  <si>
+    <t>DC Branch Fuses</t>
+  </si>
+  <si>
+    <t>A, C, E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -346,21 +339,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow (Body)"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -379,18 +357,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -723,15 +699,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="218.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="228.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="60.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="55.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="133.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -743,22 +719,22 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>1</v>
@@ -772,25 +748,25 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2">
-        <v>4</v>
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J2" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -798,22 +774,18 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
       <c r="I3" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J3" s="2">
         <v>3</v>
@@ -824,22 +796,16 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4">
-        <v>1111</v>
-      </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>10</v>
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -850,25 +816,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -876,25 +842,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="I6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -902,22 +868,16 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
         <v>35</v>
       </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
       <c r="I7" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J7">
         <v>3</v>
@@ -939,14 +899,11 @@
       <c r="E8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" t="s">
-        <v>40</v>
-      </c>
       <c r="I8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -954,22 +911,16 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J9">
         <v>3</v>
@@ -980,107 +931,89 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" t="s">
-        <v>54</v>
+        <v>46</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="J11">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" t="s">
-        <v>59</v>
-      </c>
-      <c r="F12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" t="s">
-        <v>64</v>
-      </c>
-      <c r="H12" t="s">
-        <v>63</v>
+        <v>47</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" t="s">
-        <v>71</v>
+        <v>6</v>
       </c>
       <c r="J13">
         <v>4</v>
@@ -1088,30 +1021,24 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D14" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" t="s">
-        <v>78</v>
-      </c>
       <c r="J14">
         <v>4</v>
       </c>
@@ -1121,20 +1048,26 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" t="b">
+        <v>58</v>
+      </c>
+      <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" t="b">
-        <v>0</v>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>4</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1142,20 +1075,26 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" t="b">
+        <v>59</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
         <v>1</v>
       </c>
-      <c r="D16" t="b">
-        <v>0</v>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J16">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1163,7 +1102,7 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1184,107 +1123,285 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" t="b">
+        <v>61</v>
+      </c>
+      <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18" t="b">
-        <v>0</v>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
       </c>
       <c r="I18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19">
+        <v>750</v>
+      </c>
+      <c r="D19">
+        <v>600</v>
+      </c>
+      <c r="E19">
+        <v>480</v>
+      </c>
+      <c r="F19">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
         <v>6</v>
       </c>
-      <c r="B19" t="s">
-        <v>83</v>
-      </c>
       <c r="J19">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+        <v>63</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="G20" s="2"/>
+      <c r="I20" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="J20">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+        <v>68</v>
+      </c>
+      <c r="C21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
+      <c r="I21" t="s">
+        <v>7</v>
+      </c>
       <c r="J21">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="C22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
+      <c r="I22" t="s">
+        <v>6</v>
+      </c>
       <c r="J22">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
+      <c r="A23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="G23" s="2"/>
+      <c r="I23" t="s">
+        <v>6</v>
+      </c>
+      <c r="J23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+      <c r="A24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="G24" s="2"/>
+      <c r="I24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="A25" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
+      <c r="I25" t="s">
+        <v>6</v>
+      </c>
+      <c r="J25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" t="s">
+        <v>80</v>
+      </c>
+      <c r="I26" t="s">
+        <v>82</v>
+      </c>
+      <c r="J26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I28" t="s">
+        <v>91</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{AA8F7D75-AA91-5545-8D46-889BC9732FDE}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added one more question
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEE2AD7-9716-8248-9AA0-A6ECE0F18547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D26E237-B483-2B47-8872-9CBBC427DCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-39820" yWindow="800" windowWidth="36880" windowHeight="21600" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="-26480" yWindow="800" windowWidth="23540" windowHeight="21600" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="93">
   <si>
     <t>Question Text</t>
   </si>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>A, C, E</t>
+  </si>
+  <si>
+    <t>Sungrow mandatres that the DC knob switch on the SG3600UD-MV unit needs to have ONLY a tag applied.</t>
   </si>
 </sst>
 </file>
@@ -699,7 +702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1401,6 +1404,26 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="s">
+        <v>6</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update the question pool for SG4400UD-MV safety assessment and update the title of the assessment
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF54CC9C-D3E3-A34F-BD9C-62B70F473CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70268CF5-FA13-8E44-A7CF-D3E7990B8F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-40340" yWindow="1000" windowWidth="19440" windowHeight="20240" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20560" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="102">
   <si>
     <t>Question Text</t>
   </si>
@@ -86,36 +86,12 @@
     <t>F</t>
   </si>
   <si>
-    <t>BESS</t>
-  </si>
-  <si>
-    <t>B, D, E, F</t>
-  </si>
-  <si>
-    <t>On a customer site, what is the LOTO document that should ultimatly be implemented?</t>
-  </si>
-  <si>
     <t>The site's LOTO procedure document</t>
   </si>
   <si>
     <t>Sungrow PV LOTO guidance document</t>
   </si>
   <si>
-    <t>Best judgement</t>
-  </si>
-  <si>
-    <t>SG3600UD Power Cycle MOP</t>
-  </si>
-  <si>
-    <t>There is no incident eenrgy label on the SG3600UD auxiliary cabinet. I can still access the auxiliary cabinet while it is energized, as long as I have on the appropriate PPE</t>
-  </si>
-  <si>
-    <t>Testing the DC Busbars in one inverter unit for de-energyzation is sufficient to prove DC busbar de-energization for both inverter units.</t>
-  </si>
-  <si>
-    <t>Which of the following people are permitted to operate MVT Load Switch of the SG3600UD-MV?</t>
-  </si>
-  <si>
     <t>Sungrow Employees</t>
   </si>
   <si>
@@ -128,27 +104,12 @@
     <t>All of the above</t>
   </si>
   <si>
-    <t>The proper first step to de-energize the SG3600UD-MV is to….</t>
-  </si>
-  <si>
     <t>Open the MVT Load Switch</t>
   </si>
   <si>
-    <t>Open the DC door knob switch</t>
-  </si>
-  <si>
-    <t>Send a key stop command for the inverter</t>
-  </si>
-  <si>
     <t>Disconnect the combiner boxes</t>
   </si>
   <si>
-    <t>I have turned off all the appropriate switches in the power down procedure, and have waited 24 hours. I may work on the units with the assumption that they are now in a de-energized state.</t>
-  </si>
-  <si>
-    <t>Closing the DC knob switch on the SG3600UD inverter unit will automatically close the DC load break switches.</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -158,12 +119,6 @@
     <t>It depends</t>
   </si>
   <si>
-    <t>Is it required for someone on-site to open the combiner boxes, even at night, to safely perform de-energized work on the SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>AC Capacitor de-energization testing should include which of the following tests on a multimeter?</t>
-  </si>
-  <si>
     <t>Capacitance</t>
   </si>
   <si>
@@ -173,33 +128,9 @@
     <t>DC Voltage and AC Voltage</t>
   </si>
   <si>
-    <t>DC Voltage and AC Voltage and Capacitance</t>
-  </si>
-  <si>
-    <t>Checking the AC Capacitors for just one unit on the SG3600UD-MV is sufficient to confirm all AC capacitors have discharged.</t>
-  </si>
-  <si>
-    <t>Sungrow employees and/or sub-contractors shall not operate DC Field Disconnects (DC Combiners or LBDs) on site.</t>
-  </si>
-  <si>
-    <t>What document should be referenced to safely power on the SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>SG3600UD-MV System Manual</t>
-  </si>
-  <si>
-    <t>SG3600UD-MV Power Cycle MOP</t>
-  </si>
-  <si>
     <t>Common Sense</t>
   </si>
   <si>
-    <t>PV LOTO Guidance document</t>
-  </si>
-  <si>
-    <t>How many minutes, at a minimum, do I need to wait after turning off the appropriate swiches on the SG3600UD-MV skid to test for de-energization?</t>
-  </si>
-  <si>
     <t>10 minutes</t>
   </si>
   <si>
@@ -212,27 +143,6 @@
     <t>5 minutes</t>
   </si>
   <si>
-    <t>How many qualified employees are needed to perform the shutdown and de-energization verification testing on the SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>What class of gloves are needed to perform de-energization verification testing on the SG3600UD-MV?</t>
-  </si>
-  <si>
-    <t>Testing for AC common bussing de-energization at one of the valid testing locations is sufficient to prove LV AC common bussing de-energization for the whole SG3600UD-MV skid.</t>
-  </si>
-  <si>
-    <t>How many main AC circuit breakers should open up in the SG3600UD-MV with a key stop command for the entire skid?</t>
-  </si>
-  <si>
-    <t>A safety second is required when working on voltages above which level?</t>
-  </si>
-  <si>
-    <t>Given that the unit is completely de-energized and LOTO'd according to the power-down procedure, what are the first two switches to turn on for the SG3600UD-MV power-on procedure?</t>
-  </si>
-  <si>
-    <t>QS5 and QS6</t>
-  </si>
-  <si>
     <t>QS9 and QF1</t>
   </si>
   <si>
@@ -242,79 +152,196 @@
     <t>None of the above</t>
   </si>
   <si>
-    <t>Sungrow does not require indicidual DC Load Switches and AC Breakers to be LOTO'd.</t>
-  </si>
-  <si>
-    <t>I need to replace a power stack/power module in Unit 2 of the SG3600UD-MV skid. As long as I test for de-energization of the AC common bussing and all the appropriate testing checks within Unit 2, I can proceed with the replacement procedure.</t>
-  </si>
-  <si>
     <t>The best method to do a functional test of the E-stop button will be during a real-life operating circumstance, such as when the inverter is pushing 100% output power to the grid.</t>
   </si>
   <si>
-    <t>Under which of the below following conditions may the AC side fo the SG3600UD-MV inverter units be opened up to test for de-energization? The donned PPE matches the incident energy label requirement.</t>
-  </si>
-  <si>
-    <t>As long as the inverter is shutdown via the HMI or web portal</t>
-  </si>
-  <si>
-    <t>If the combiners and MVT load switch have been opened</t>
-  </si>
-  <si>
-    <t>if I have pressed the E-stop button and 20 minutes have elapsed afterwards</t>
-  </si>
-  <si>
     <t>If all the appropriate switches in accordance with the power down procedure have been opened up, with 5 minutes having elapsed afterwards.</t>
   </si>
   <si>
-    <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, the inverter cabinet doors can still be opened.</t>
-  </si>
-  <si>
-    <t>QS1</t>
-  </si>
-  <si>
-    <t>QS2</t>
-  </si>
-  <si>
-    <t>QS3</t>
-  </si>
-  <si>
-    <t>QS4</t>
-  </si>
-  <si>
-    <t>Which of the following DC Load Switches are present on every single SG3600UD-MV inverter?</t>
-  </si>
-  <si>
-    <t>A, C</t>
-  </si>
-  <si>
-    <t>What are all the potential energy/voltage sources to isolate from / allow to discharge during de-energization of the SG3600UD-MV inverters?</t>
-  </si>
-  <si>
     <t>AC and DC Capacitors</t>
   </si>
   <si>
-    <t>Which of the following testing locations need to be checked to confirm de-energization on the DC side of the SG3600UD-MV inverter?</t>
-  </si>
-  <si>
-    <t>FU29 and FU30</t>
-  </si>
-  <si>
     <t>AC SPD circuit, before the fuses. Either in Aux cabinet or in Unit 1</t>
   </si>
   <si>
-    <t>DC busbars leading into the DC Load Switches</t>
-  </si>
-  <si>
-    <t>FU16, FU17, and FU18</t>
-  </si>
-  <si>
-    <t>DC Branch Fuses</t>
-  </si>
-  <si>
-    <t>A, C, E</t>
-  </si>
-  <si>
-    <t>Sungrow mandatres that the DC knob switch on the SG3600UD-MV unit needs to have ONLY a tag applied.</t>
+    <t>What door LED indicator color proves that the SG4400UD is de-energized?</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>When the LEDs are off</t>
+  </si>
+  <si>
+    <t>LED indicator doesn't prove de-energization</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>In an emergency power-down situation, how many E-stop buttons on the SG4400UD should be pressed in?</t>
+  </si>
+  <si>
+    <t>There is no incident energy label on the SG4400UD auxiliary cabinet. I can still access the auxiliary cabinet while it is energized, as long as I have on the apppropriate PPE.</t>
+  </si>
+  <si>
+    <t>On a customer site, what is the LOTO document that should ultimately be implemented?</t>
+  </si>
+  <si>
+    <t>Best Judgement</t>
+  </si>
+  <si>
+    <t>SG4400UD Power Cycle MOP</t>
+  </si>
+  <si>
+    <t>Testing the DC Busbars in one inverter unit for de-energization is sufficient to prove DC busbar de-energization for all 3-4 inverter units.</t>
+  </si>
+  <si>
+    <t>Who can the MVT load switch of the SG4400UD be operated by?</t>
+  </si>
+  <si>
+    <t>What is the updated testing points used to confirm DC Capacitor de-energization in the SG1100UD units?</t>
+  </si>
+  <si>
+    <t>FU23 and FU24</t>
+  </si>
+  <si>
+    <t>On top of the DC Load Break Switch</t>
+  </si>
+  <si>
+    <t>FU40, FU41, &amp;FU42</t>
+  </si>
+  <si>
+    <t>FU31, FU32, FU33</t>
+  </si>
+  <si>
+    <t>The proper first step to de-energize the SG4400UD is to…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send a shutdown command in the web portal for the unit that maintenance will be performed on </t>
+  </si>
+  <si>
+    <t>Change the control mode to local and send a shutdown command for all inverter units/the entire skid</t>
+  </si>
+  <si>
+    <t>I have turned off all the appropriate switches in the power down procedure, and have waited for 24 hours. I may work on the units with the assumption that they are now in a de-energized state.</t>
+  </si>
+  <si>
+    <t>Closing the DC knob on the front of each SG1100UD inverter unit will close the DC load break switches.</t>
+  </si>
+  <si>
+    <t>In the 5kVA auxiliary cabinet, how many phases can I access for de-energization testing at FU104?</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Is it required for someone on-site to open the switches inside the combiner boxes, even at night, to safely perform de-energized work on the SG4400UD?</t>
+  </si>
+  <si>
+    <t>What SG4400UD Web Portal Setting Disables/Enables the use of the door switches</t>
+  </si>
+  <si>
+    <t>Manual Fan Speed Regulation</t>
+  </si>
+  <si>
+    <t>Access Protection Enabling</t>
+  </si>
+  <si>
+    <t>Active Power Limit Ratio</t>
+  </si>
+  <si>
+    <t>Shutdown</t>
+  </si>
+  <si>
+    <t>AC capacitor de-energization testing should include which of the following testing modes on a multi-meter?</t>
+  </si>
+  <si>
+    <t>AC Voltage and Capaciitance</t>
+  </si>
+  <si>
+    <t>Sungrow mandates the DC knobs on the front of each SG1100UD unit need to have ONLY a tag applied</t>
+  </si>
+  <si>
+    <t>What document should be used to safely power on the SG4400UD?</t>
+  </si>
+  <si>
+    <t>SG4400UD-MV System Manual</t>
+  </si>
+  <si>
+    <t>SG4400UD-MV Power Cycle MOP</t>
+  </si>
+  <si>
+    <t>1+X LOTO document</t>
+  </si>
+  <si>
+    <t>How many minutes, at a minimum, do I need to wait after turning off the appropriate switches on the SG4400UD skid to test for de-energization?</t>
+  </si>
+  <si>
+    <t>Testing for AC common bussing de-energization at one of the valid testing locations is sufficient to prove AC common bussing de-energization for the whole SG4400UD skid.</t>
+  </si>
+  <si>
+    <t>How many main AC Circuit Breakers should open up in the SG4400UD with a shutdown command for the entire skid?</t>
+  </si>
+  <si>
+    <t>What are the first two switches to turn on for the SG4400UD power-on procedure? Assume that the unit is completely de-energized according to the power-down procedure.</t>
+  </si>
+  <si>
+    <t>QS2 and QS9</t>
+  </si>
+  <si>
+    <t>Under which of the below following conditions may the AC side for the SG1100UD inverter units (back side) be immediately opened up to test for de-energization? The donned PPE matches the AC incident energy label requirement.</t>
+  </si>
+  <si>
+    <t>As long as the inverter is shutdown via the web portal</t>
+  </si>
+  <si>
+    <t>If the combiners and MVT load switch have been opened, with 5 minutes having elapsed afterwards.</t>
+  </si>
+  <si>
+    <t>If I have pressed the E-stop button and 20 minutes have elapsed afterwards</t>
+  </si>
+  <si>
+    <t>I need to replace a power stack/power module in Unit 2 of the SG4400UD. As long as I test for de-energization of the AC common bussing and all the appropriate testing checks within Unit 2, I can proceed with the replacement procedure.</t>
+  </si>
+  <si>
+    <t>What is the primary purpose of the QS2 maintenance switch? How many are on the SG4400UD-MV skid?</t>
+  </si>
+  <si>
+    <t>Provide power to auxiliary cabinet 1</t>
+  </si>
+  <si>
+    <t>Energize T2 transformer, 3</t>
+  </si>
+  <si>
+    <t>Energize T1 transformer, 4</t>
+  </si>
+  <si>
+    <t>Provide power to auxiliary cabinet, 4</t>
+  </si>
+  <si>
+    <t>B, D, E</t>
+  </si>
+  <si>
+    <t>Which of the following testing locations include DC voltage checks to confirm de-energization?</t>
+  </si>
+  <si>
+    <t>HV room voltage</t>
+  </si>
+  <si>
+    <t>PE board 24V output</t>
+  </si>
+  <si>
+    <t>FU31, FU32, and FU33</t>
+  </si>
+  <si>
+    <t>A, E</t>
+  </si>
+  <si>
+    <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, inverter cabinet doors can still be opened.</t>
+  </si>
+  <si>
+    <t>What are the energy/voltage sources to isolate from/allow to discharge during de-energization of the SG4400UD inverters?</t>
   </si>
 </sst>
 </file>
@@ -363,11 +390,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,10 +741,10 @@
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="228.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="60.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="71" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="88.6640625" customWidth="1"/>
+    <col min="5" max="5" width="83" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="133.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -752,22 +785,22 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J2" s="2">
         <v>4</v>
@@ -778,21 +811,25 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="2" t="b">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="D3" s="4">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4">
+        <v>3</v>
+      </c>
+      <c r="F3" s="4">
+        <v>4</v>
+      </c>
       <c r="I3" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J3" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -800,7 +837,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2" t="b">
         <v>1</v>
@@ -820,22 +857,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="I5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -846,25 +883,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>34</v>
+        <v>52</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -872,19 +903,25 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" t="b">
-        <v>0</v>
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
       </c>
       <c r="I7" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -892,19 +929,22 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
+        <v>57</v>
+      </c>
+      <c r="F8" t="s">
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -915,19 +955,25 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>23</v>
       </c>
       <c r="I9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -935,25 +981,19 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" t="s">
-        <v>45</v>
+        <v>62</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -961,19 +1001,22 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" t="b">
-        <v>0</v>
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
       </c>
       <c r="I11" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -981,19 +1024,25 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" t="b">
+        <v>64</v>
+      </c>
+      <c r="C12" s="5">
         <v>1</v>
       </c>
-      <c r="D12" t="b">
-        <v>0</v>
+      <c r="D12" s="5">
+        <v>2</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>65</v>
       </c>
       <c r="I12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1001,26 +1050,20 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" t="s">
-        <v>51</v>
-      </c>
-      <c r="F13" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J13">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1028,21 +1071,24 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="H14" s="2"/>
+      <c r="I14" t="s">
+        <v>6</v>
+      </c>
       <c r="J14">
         <v>4</v>
       </c>
@@ -1052,23 +1098,23 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
-        <v>2</v>
-      </c>
-      <c r="E15">
-        <v>3</v>
-      </c>
-      <c r="F15">
-        <v>4</v>
+        <v>72</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>73</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>4</v>
@@ -1079,26 +1125,20 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16">
+        <v>74</v>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" t="b">
         <v>0</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>2</v>
-      </c>
-      <c r="F16">
-        <v>3</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J16">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1106,20 +1146,26 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" t="b">
-        <v>1</v>
-      </c>
-      <c r="D17" t="b">
-        <v>0</v>
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" t="s">
+        <v>78</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -1127,25 +1173,25 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
-        <v>2</v>
-      </c>
-      <c r="E18">
-        <v>3</v>
-      </c>
-      <c r="F18">
-        <v>4</v>
+        <v>79</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" t="s">
+        <v>34</v>
       </c>
       <c r="I18" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -1153,25 +1199,25 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19">
-        <v>750</v>
-      </c>
-      <c r="D19">
-        <v>600</v>
-      </c>
-      <c r="E19">
-        <v>480</v>
-      </c>
-      <c r="F19">
-        <v>120</v>
+        <v>81</v>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5">
+        <v>2</v>
+      </c>
+      <c r="E19" s="5">
+        <v>3</v>
+      </c>
+      <c r="F19" s="5">
+        <v>4</v>
       </c>
       <c r="I19" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J19">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
@@ -1179,26 +1225,26 @@
         <v>4</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="G20" s="2"/>
       <c r="I20" s="2" t="s">
         <v>7</v>
       </c>
       <c r="J20">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -1206,22 +1252,26 @@
         <v>4</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="G21" s="2"/>
       <c r="I21" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J21">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -1229,7 +1279,7 @@
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C22" s="2" t="b">
         <v>1</v>
@@ -1252,7 +1302,7 @@
         <v>4</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="C23" s="2" t="b">
         <v>1</v>
@@ -1270,26 +1320,26 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="G24" s="2"/>
       <c r="I24" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>4</v>
@@ -1297,22 +1347,28 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="I25" t="s">
-        <v>6</v>
+        <v>95</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="J25">
         <v>3</v>
@@ -1320,60 +1376,42 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C26" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" t="s">
-        <v>80</v>
+        <v>100</v>
+      </c>
+      <c r="C26" t="b">
+        <v>1</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="J26">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C27" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" t="s">
-        <v>84</v>
-      </c>
-      <c r="H27" t="s">
-        <v>16</v>
+        <v>80</v>
+      </c>
+      <c r="C27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="I27" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="J27">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -1381,49 +1419,33 @@
         <v>5</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="C28" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="G28" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="I28" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J28">
         <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" t="b">
-        <v>1</v>
-      </c>
-      <c r="D29" t="b">
-        <v>0</v>
-      </c>
-      <c r="I29" t="s">
-        <v>6</v>
-      </c>
-      <c r="J29">
-        <v>3</v>
-      </c>
+      <c r="A29" s="1"/>
+      <c r="B29" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix the issue of button missing
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7011FE1C-0EAF-8340-9308-95DA6BDB567E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0149C5A-CC83-6B49-B285-800F54AD7759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-200" yWindow="520" windowWidth="36500" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="900" yWindow="500" windowWidth="18960" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Added gitignore to pretect credentials and updated the sample code
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28EEB283-88FD-E44F-A702-7DB785FF733B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9DFDAD-B24A-AA4B-9C83-898B6CD9A7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20660" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="-38580" yWindow="1900" windowWidth="34560" windowHeight="20640" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
change the name of answer sheet for SG3600UD_MV_CSP
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9DFDAD-B24A-AA4B-9C83-898B6CD9A7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC35728-CD18-4E4E-930B-AD14FD6FED84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38580" yWindow="1900" windowWidth="34560" windowHeight="20640" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20640" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix the code of True or False rendering function
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF54CC9C-D3E3-A34F-BD9C-62B70F473CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609136BF-B27C-7B4B-A6D2-CF6D689AFB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-40340" yWindow="1000" windowWidth="19440" windowHeight="20240" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20100" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
modify the question pool structure - adding columns G and H for
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{422EAF5C-C01F-3A44-B578-62BEF89F9D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491F9FB6-815E-1B40-9CEF-58CB7A7BF7BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="104">
   <si>
     <t>Question Text</t>
   </si>
@@ -342,6 +342,12 @@
   </si>
   <si>
     <t>What are the energy/voltage sources to isolate from/allow to discharge during de-energization of the SG4400UD inverters?</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
 </sst>
 </file>
@@ -735,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -745,10 +751,13 @@
     <col min="5" max="5" width="83" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="133.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="10" max="10" width="22.1640625" customWidth="1"/>
+    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -774,13 +783,19 @@
         <v>15</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -799,14 +814,14 @@
       <c r="F2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L2" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -825,14 +840,14 @@
       <c r="F3" s="4">
         <v>4</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L3" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -845,14 +860,14 @@
       <c r="D4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -871,14 +886,14 @@
       <c r="F5" t="s">
         <v>51</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>7</v>
       </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -891,14 +906,14 @@
       <c r="D6" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>6</v>
       </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -917,14 +932,14 @@
       <c r="F7" t="s">
         <v>21</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>8</v>
       </c>
-      <c r="J7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -943,14 +958,14 @@
       <c r="F8" t="s">
         <v>58</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>9</v>
       </c>
-      <c r="J8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -969,14 +984,14 @@
       <c r="F9" t="s">
         <v>23</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>8</v>
       </c>
-      <c r="J9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -989,14 +1004,14 @@
       <c r="D10" t="b">
         <v>0</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>6</v>
       </c>
-      <c r="J10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -1012,14 +1027,14 @@
       <c r="E11" t="s">
         <v>26</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>8</v>
       </c>
-      <c r="J11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1038,14 +1053,14 @@
       <c r="F12" t="s">
         <v>65</v>
       </c>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>6</v>
       </c>
-      <c r="J12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
@@ -1059,14 +1074,14 @@
         <v>25</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>7</v>
       </c>
-      <c r="J13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
@@ -1086,14 +1101,14 @@
         <v>71</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>6</v>
       </c>
-      <c r="J14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
@@ -1113,14 +1128,14 @@
         <v>73</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>8</v>
       </c>
-      <c r="J15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1134,14 +1149,14 @@
         <v>0</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>6</v>
       </c>
-      <c r="J16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1161,14 +1176,14 @@
         <v>78</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>6</v>
       </c>
-      <c r="J17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1187,14 +1202,14 @@
       <c r="F18" t="s">
         <v>34</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>9</v>
       </c>
-      <c r="J18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1213,14 +1228,14 @@
       <c r="F19" s="5">
         <v>4</v>
       </c>
-      <c r="I19" t="s">
+      <c r="K19" t="s">
         <v>9</v>
       </c>
-      <c r="J19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1240,14 +1255,14 @@
         <v>37</v>
       </c>
       <c r="G20" s="2"/>
-      <c r="I20" s="2" t="s">
+      <c r="K20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1267,14 +1282,14 @@
         <v>39</v>
       </c>
       <c r="G21" s="2"/>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>9</v>
       </c>
-      <c r="J21">
+      <c r="L21">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1290,14 +1305,14 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
-      <c r="I22" t="s">
+      <c r="K22" t="s">
         <v>6</v>
       </c>
-      <c r="J22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>4</v>
       </c>
@@ -1311,14 +1326,14 @@
         <v>0</v>
       </c>
       <c r="G23" s="2"/>
-      <c r="I23" t="s">
+      <c r="K23" t="s">
         <v>6</v>
       </c>
-      <c r="J23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>5</v>
       </c>
@@ -1338,14 +1353,14 @@
         <v>93</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="I24" s="2" t="s">
+      <c r="K24" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J24">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L24">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
@@ -1367,14 +1382,14 @@
       <c r="G25" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="K25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="J25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
@@ -1387,14 +1402,14 @@
       <c r="D26" t="b">
         <v>0</v>
       </c>
-      <c r="I26" t="s">
+      <c r="K26" t="s">
         <v>6</v>
       </c>
-      <c r="J26">
+      <c r="L26">
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
@@ -1407,14 +1422,14 @@
       <c r="D27" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I27" t="s">
+      <c r="K27" t="s">
         <v>7</v>
       </c>
-      <c r="J27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>5</v>
       </c>
@@ -1436,14 +1451,14 @@
       <c r="G28" t="s">
         <v>40</v>
       </c>
-      <c r="I28" t="s">
+      <c r="K28" t="s">
         <v>94</v>
       </c>
-      <c r="J28">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update the repository to connect to the Google Cloud Reponse Records Sheet
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DFB401-6075-EE4A-8A62-988EBB3E85EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB75E489-FA1B-0848-A5CE-4F8CCFF097E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-72960" yWindow="640" windowWidth="38380" windowHeight="20240" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
   <si>
     <t>Question Text</t>
   </si>
@@ -394,6 +394,15 @@
   </si>
   <si>
     <t>Describe the power up and down process of the SG3150U including the LOTO procedure. Be sure to mention all five of the energy sources that should be identified and tested for de-energization.</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
 </sst>
 </file>
@@ -810,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -820,12 +829,13 @@
     <col min="5" max="5" width="76.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="57.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -848,13 +858,22 @@
         <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
@@ -873,14 +892,14 @@
       <c r="F2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>9</v>
       </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -899,14 +918,14 @@
       <c r="F3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
         <v>8</v>
       </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -925,14 +944,14 @@
       <c r="F4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H4" t="s">
+      <c r="K4" t="s">
         <v>7</v>
       </c>
-      <c r="I4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -951,14 +970,14 @@
       <c r="F5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H5" t="s">
+      <c r="K5" t="s">
         <v>6</v>
       </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -977,14 +996,14 @@
       <c r="F6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H6" t="s">
+      <c r="K6" t="s">
         <v>9</v>
       </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
@@ -1003,14 +1022,14 @@
       <c r="F7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="H7" t="s">
+      <c r="K7" t="s">
         <v>8</v>
       </c>
-      <c r="I7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
@@ -1029,14 +1048,14 @@
       <c r="F8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H8" t="s">
+      <c r="K8" t="s">
         <v>9</v>
       </c>
-      <c r="I8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
@@ -1055,14 +1074,14 @@
       <c r="F9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H9" t="s">
+      <c r="K9" t="s">
         <v>6</v>
       </c>
-      <c r="I9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
@@ -1081,14 +1100,14 @@
       <c r="F10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H10" t="s">
+      <c r="K10" t="s">
         <v>7</v>
       </c>
-      <c r="I10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
@@ -1107,14 +1126,14 @@
       <c r="F11" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H11" t="s">
+      <c r="K11" t="s">
         <v>8</v>
       </c>
-      <c r="I11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
@@ -1133,14 +1152,14 @@
       <c r="F12" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H12" t="s">
+      <c r="K12" t="s">
         <v>6</v>
       </c>
-      <c r="I12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
@@ -1162,14 +1181,14 @@
       <c r="G13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H13" t="s">
+      <c r="K13" t="s">
         <v>73</v>
       </c>
-      <c r="I13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
@@ -1188,14 +1207,14 @@
       <c r="F14" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="H14" t="s">
+      <c r="K14" t="s">
         <v>78</v>
       </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>5</v>
       </c>
@@ -1217,14 +1236,14 @@
       <c r="G15" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="H15" t="s">
+      <c r="K15" t="s">
         <v>73</v>
       </c>
-      <c r="I15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>5</v>
       </c>
@@ -1243,14 +1262,14 @@
       <c r="F16" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H16" t="s">
+      <c r="K16" t="s">
         <v>14</v>
       </c>
-      <c r="I16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>5</v>
       </c>
@@ -1269,14 +1288,14 @@
       <c r="F17" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="H17" t="s">
+      <c r="K17" t="s">
         <v>95</v>
       </c>
-      <c r="I17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>5</v>
       </c>
@@ -1295,14 +1314,14 @@
       <c r="F18" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="H18" t="s">
+      <c r="K18" t="s">
         <v>101</v>
       </c>
-      <c r="I18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>4</v>
       </c>
@@ -1315,14 +1334,14 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H19" t="s">
+      <c r="K19" t="s">
         <v>6</v>
       </c>
-      <c r="I19">
+      <c r="L19">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>4</v>
       </c>
@@ -1335,14 +1354,14 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H20" t="s">
+      <c r="K20" t="s">
         <v>6</v>
       </c>
-      <c r="I20">
+      <c r="L20">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>4</v>
       </c>
@@ -1357,14 +1376,14 @@
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
-      <c r="H21" s="3" t="s">
+      <c r="K21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I21">
+      <c r="L21">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>4</v>
       </c>
@@ -1377,14 +1396,14 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H22" t="s">
+      <c r="K22" t="s">
         <v>6</v>
       </c>
-      <c r="I22">
+      <c r="L22">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>4</v>
       </c>
@@ -1397,14 +1416,14 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H23" t="s">
+      <c r="K23" t="s">
         <v>6</v>
       </c>
-      <c r="I23">
+      <c r="L23">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>4</v>
       </c>
@@ -1417,14 +1436,14 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H24" t="s">
+      <c r="K24" t="s">
         <v>7</v>
       </c>
-      <c r="I24">
+      <c r="L24">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>108</v>
       </c>
@@ -1435,12 +1454,12 @@
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25">
+      <c r="K25" s="3"/>
+      <c r="L25">
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>108</v>
       </c>
@@ -1449,11 +1468,11 @@
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
-      <c r="I26">
+      <c r="L26">
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>108</v>
       </c>
@@ -1464,17 +1483,17 @@
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27">
+      <c r="K27" s="3"/>
+      <c r="L27">
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="2"/>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
     </row>

</xml_diff>

<commit_message>
update the repository to connect to the Google Cloud Response Records Sheet
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B84C3BB-E02C-EE47-9196-A5A1908A6FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373D3110-694A-EE4C-ACF7-4A431A1BF659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-70360" yWindow="560" windowWidth="34740" windowHeight="20240" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="96">
   <si>
     <t>Question Text</t>
   </si>
@@ -321,6 +321,9 @@
   </si>
   <si>
     <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
 </sst>
 </file>
@@ -723,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -739,7 +742,7 @@
     <col min="11" max="11" width="7.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -768,13 +771,16 @@
         <v>94</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
@@ -793,14 +799,14 @@
       <c r="F2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>7</v>
       </c>
-      <c r="K2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -813,14 +819,14 @@
       <c r="D3" t="b">
         <v>0</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>6</v>
       </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -835,14 +841,14 @@
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>6</v>
       </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -861,14 +867,14 @@
       <c r="F5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>8</v>
       </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -887,14 +893,14 @@
       <c r="F6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>8</v>
       </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
@@ -907,14 +913,14 @@
       <c r="D7" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>6</v>
       </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
@@ -927,14 +933,14 @@
       <c r="D8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>7</v>
       </c>
-      <c r="K8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
@@ -950,14 +956,14 @@
       <c r="E9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>6</v>
       </c>
-      <c r="K9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
@@ -976,14 +982,14 @@
       <c r="F10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>8</v>
       </c>
-      <c r="K10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
@@ -996,14 +1002,14 @@
       <c r="D11" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>6</v>
       </c>
-      <c r="K11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
@@ -1016,14 +1022,14 @@
       <c r="D12" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>7</v>
       </c>
-      <c r="K12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>4</v>
       </c>
@@ -1036,14 +1042,14 @@
       <c r="D13" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>6</v>
       </c>
-      <c r="K13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>4</v>
       </c>
@@ -1062,14 +1068,14 @@
       <c r="F14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>6</v>
       </c>
-      <c r="K14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>4</v>
       </c>
@@ -1088,14 +1094,14 @@
       <c r="F15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>9</v>
       </c>
-      <c r="K15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>4</v>
       </c>
@@ -1114,14 +1120,14 @@
       <c r="F16">
         <v>4</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>6</v>
       </c>
-      <c r="K16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>4</v>
       </c>
@@ -1140,14 +1146,14 @@
       <c r="F17">
         <v>3</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>7</v>
       </c>
-      <c r="K17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>4</v>
       </c>
@@ -1160,14 +1166,14 @@
       <c r="D18" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>7</v>
       </c>
-      <c r="K18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>4</v>
       </c>
@@ -1186,14 +1192,14 @@
       <c r="F19">
         <v>3</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>7</v>
       </c>
-      <c r="K19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>4</v>
       </c>
@@ -1212,14 +1218,14 @@
       <c r="F20">
         <v>120</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>6</v>
       </c>
-      <c r="K20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>4</v>
       </c>
@@ -1238,14 +1244,14 @@
       <c r="F21" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J21" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>4</v>
       </c>
@@ -1258,14 +1264,14 @@
       <c r="D22" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>7</v>
       </c>
-      <c r="K22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>4</v>
       </c>
@@ -1278,14 +1284,14 @@
       <c r="D23" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>6</v>
       </c>
-      <c r="K23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>4</v>
       </c>
@@ -1298,14 +1304,14 @@
       <c r="D24" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>6</v>
       </c>
-      <c r="K24">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>4</v>
       </c>
@@ -1324,14 +1330,14 @@
       <c r="F25" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="K25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>4</v>
       </c>
@@ -1344,14 +1350,14 @@
       <c r="D26" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="J26" t="s">
+      <c r="K26" t="s">
         <v>6</v>
       </c>
-      <c r="K26">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>5</v>
       </c>
@@ -1370,14 +1376,14 @@
       <c r="F27" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="K27" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="K27">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>5</v>
       </c>
@@ -1405,14 +1411,14 @@
       <c r="I28" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="K28" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="K28">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>5</v>
       </c>
@@ -1434,10 +1440,10 @@
       <c r="G29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="J29" s="2" t="s">
+      <c r="K29" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update the question bank file
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0149C5A-CC83-6B49-B285-800F54AD7759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9ADBBCD-6AD9-A941-8319-18FEE1D18518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="500" windowWidth="18960" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="900" yWindow="760" windowWidth="30840" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
update the repository to connect to Goole Cloud repsonse record sheet
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5944137-C4A1-0B43-8222-4589C2B5A751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CF6380-0695-A24E-A148-A483E23954D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="500" windowWidth="36740" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="82">
   <si>
     <t>Question Text</t>
   </si>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t>Text</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
 </sst>
 </file>
@@ -684,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
@@ -696,11 +699,12 @@
     <col min="7" max="7" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -729,13 +733,16 @@
         <v>79</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -754,14 +761,14 @@
       <c r="F2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L2" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -780,14 +787,14 @@
       <c r="F3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L3" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -806,14 +813,14 @@
       <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>8</v>
       </c>
-      <c r="K4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -832,14 +839,14 @@
       <c r="F5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>8</v>
       </c>
-      <c r="K5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -852,14 +859,14 @@
       <c r="D6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>6</v>
       </c>
-      <c r="K6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -878,14 +885,14 @@
       <c r="F7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>7</v>
       </c>
-      <c r="K7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -904,14 +911,14 @@
       <c r="F8" s="6">
         <v>480</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>6</v>
       </c>
-      <c r="K8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -930,14 +937,14 @@
       <c r="F9" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>6</v>
       </c>
-      <c r="K9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -956,14 +963,14 @@
       <c r="F10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>7</v>
       </c>
-      <c r="K10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
@@ -985,14 +992,14 @@
       <c r="G11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>56</v>
       </c>
-      <c r="K11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -1020,14 +1027,14 @@
       <c r="I12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>65</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
@@ -1051,14 +1058,14 @@
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>72</v>
       </c>
-      <c r="K13">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
@@ -1073,14 +1080,14 @@
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>7</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
@@ -1095,14 +1102,14 @@
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>7</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1117,14 +1124,14 @@
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>6</v>
       </c>
-      <c r="K16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1139,14 +1146,14 @@
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>6</v>
       </c>
-      <c r="K17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1159,25 +1166,25 @@
       <c r="D18" t="b">
         <v>0</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>6</v>
       </c>
-      <c r="K18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>80</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1187,7 +1194,7 @@
       <c r="G20" s="2"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1196,7 +1203,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1205,14 +1212,14 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1222,7 +1229,7 @@
       <c r="G24" s="2"/>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
@@ -1231,20 +1238,20 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="2"/>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update the repository to connect to Google Cloud Response Answer Sheet
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C3618E-996B-9941-9F34-45B6A705D5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A460184-3BC5-ED49-BD64-53A6B9DF40D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="103">
   <si>
     <t>Question Text</t>
   </si>
@@ -339,6 +339,12 @@
   </si>
   <si>
     <t>A, B, D</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>H</t>
   </si>
 </sst>
 </file>
@@ -740,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -753,9 +759,10 @@
     <col min="8" max="8" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -781,13 +788,19 @@
         <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -806,14 +819,14 @@
       <c r="F2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L2" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -828,14 +841,14 @@
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="I3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L3" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -854,14 +867,14 @@
       <c r="F4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>9</v>
       </c>
-      <c r="J4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -880,14 +893,14 @@
       <c r="F5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>9</v>
       </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -906,14 +919,14 @@
       <c r="F6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>8</v>
       </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -932,14 +945,14 @@
       <c r="F7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>6</v>
       </c>
-      <c r="J7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -958,14 +971,14 @@
       <c r="F8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>6</v>
       </c>
-      <c r="J8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -980,14 +993,14 @@
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>6</v>
       </c>
-      <c r="J9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -1006,14 +1019,14 @@
       <c r="F10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>7</v>
       </c>
-      <c r="J10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1033,14 +1046,14 @@
         <v>50</v>
       </c>
       <c r="G11" s="4"/>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>97</v>
       </c>
-      <c r="J11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1057,14 +1070,14 @@
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>7</v>
       </c>
-      <c r="J12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
@@ -1085,14 +1098,14 @@
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="2"/>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>7</v>
       </c>
-      <c r="J13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
@@ -1117,14 +1130,14 @@
       <c r="H14" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>98</v>
       </c>
-      <c r="J14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
@@ -1144,14 +1157,14 @@
         <v>12</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>6</v>
       </c>
-      <c r="J15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
@@ -1165,14 +1178,14 @@
         <v>0</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>7</v>
       </c>
-      <c r="J16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1192,14 +1205,14 @@
         <v>69</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>8</v>
       </c>
-      <c r="J17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1212,14 +1225,14 @@
       <c r="D18" t="b">
         <v>0</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>6</v>
       </c>
-      <c r="J18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
@@ -1241,14 +1254,14 @@
       <c r="G19" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1261,14 +1274,14 @@
       <c r="D20" t="b">
         <v>0</v>
       </c>
-      <c r="I20" t="s">
+      <c r="K20" t="s">
         <v>7</v>
       </c>
-      <c r="J20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1287,14 +1300,14 @@
       <c r="F21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>7</v>
       </c>
-      <c r="J21">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1313,14 +1326,14 @@
       <c r="F22" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="I22" t="s">
+      <c r="K22" t="s">
         <v>100</v>
       </c>
-      <c r="J22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>4</v>
       </c>
@@ -1339,14 +1352,14 @@
       <c r="F23" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="I23" t="s">
+      <c r="K23" t="s">
         <v>8</v>
       </c>
-      <c r="J23">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="L23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
@@ -1368,14 +1381,14 @@
       <c r="G24" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="K24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J24">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L24">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
@@ -1384,20 +1397,20 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="2"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="2"/>
       <c r="D28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update PT1.0 CSP testing pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7104D4-7512-2840-9D29-A60D25F11953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60E0A06-9344-B044-8E4E-541783D48ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="500" windowWidth="35900" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="-37160" yWindow="500" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="147">
   <si>
     <t>Question Text</t>
   </si>
@@ -293,30 +293,12 @@
     <t>DC/DCs</t>
   </si>
   <si>
-    <t>Battery Collection Panel</t>
-  </si>
-  <si>
-    <t>PCS DC Side Fuses</t>
-  </si>
-  <si>
-    <t>PCS DC Capacitor Bank</t>
-  </si>
-  <si>
     <t>PCS Power Stacks</t>
   </si>
   <si>
-    <t>AC Filtering (AC Inductor -&gt; AC Capacitors)</t>
-  </si>
-  <si>
     <t>MVT Low Voltage Bushings</t>
   </si>
   <si>
-    <t xml:space="preserve">AC Circuir Breaker </t>
-  </si>
-  <si>
-    <t>PCS DC Load Swich</t>
-  </si>
-  <si>
     <t>G</t>
   </si>
   <si>
@@ -329,14 +311,179 @@
     <t>J</t>
   </si>
   <si>
-    <t>D, H, I, A, J, F, G, B, C, E</t>
+    <t>Battery Collection Panel </t>
+  </si>
+  <si>
+    <t>PCS DC Side Fuses </t>
+  </si>
+  <si>
+    <t> PCS DC Load Switch</t>
+  </si>
+  <si>
+    <t>PC DC Capacitor Bank</t>
+  </si>
+  <si>
+    <t>AC Filtering (AC Inductor-&gt;AC Capacitors)</t>
+  </si>
+  <si>
+    <t>AC Circuit Breaker</t>
+  </si>
+  <si>
+    <t>A, B, C, D, E, F, G, H, I, J</t>
+  </si>
+  <si>
+    <t>On PCS, the air flow inlet is located on top to prevent dust get inside the unit</t>
+  </si>
+  <si>
+    <t>The intelligent unit board that communicate with SCADA is __ board</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>PZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At  25 degree C, the pressure for the fuel tank should be set to 0 psig </t>
+  </si>
+  <si>
+    <t>What is needed to connect with a CMU</t>
+  </si>
+  <si>
+    <t>iConfig</t>
+  </si>
+  <si>
+    <t>USB CAN adapter</t>
+  </si>
+  <si>
+    <t>Cell temperature and voltage information could be accessed from BSC</t>
+  </si>
+  <si>
+    <t>Which type of fuses make troubleshooting easy?</t>
+  </si>
+  <si>
+    <t>Barral Fuses</t>
+  </si>
+  <si>
+    <t>Branch Fuses</t>
+  </si>
+  <si>
+    <t>There are _ circulation(s) of air cooling in the PCS</t>
+  </si>
+  <si>
+    <t>PCS air inlet is on top.</t>
+  </si>
+  <si>
+    <t>In the PCS, you can connect to your laptop to the _ board for PCS information.</t>
+  </si>
+  <si>
+    <t>PE</t>
+  </si>
+  <si>
+    <t>PX</t>
+  </si>
+  <si>
+    <t>What is the torque strengh for the M8 screws? (N.m)</t>
+  </si>
+  <si>
+    <t>7-8</t>
+  </si>
+  <si>
+    <t>60-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-23 </t>
+  </si>
+  <si>
+    <t>119-140</t>
+  </si>
+  <si>
+    <t>What do you need to connect to a CMU?</t>
+  </si>
+  <si>
+    <t>USBCAN</t>
+  </si>
+  <si>
+    <t>CMU monitor app</t>
+  </si>
+  <si>
+    <t>Generator</t>
+  </si>
+  <si>
+    <t>A, B</t>
+  </si>
+  <si>
+    <t>In BSC, what information can you see?</t>
+  </si>
+  <si>
+    <t>Rack information</t>
+  </si>
+  <si>
+    <t>Cell information</t>
+  </si>
+  <si>
+    <t>DCDC information</t>
+  </si>
+  <si>
+    <t>Transformer information</t>
+  </si>
+  <si>
+    <t>A, B, C</t>
+  </si>
+  <si>
+    <t>Which board(s) supply power to other boards?</t>
+  </si>
+  <si>
+    <t>PG</t>
+  </si>
+  <si>
+    <t>Where in the LC can you switch between Local mode, Remote mode and Local/Remote mode?</t>
+  </si>
+  <si>
+    <t>System info</t>
+  </si>
+  <si>
+    <t>Running info</t>
+  </si>
+  <si>
+    <t>Running Settings</t>
+  </si>
+  <si>
+    <t>Which sub-device parameters can you set on LC parameter settings?</t>
+  </si>
+  <si>
+    <t>PCS</t>
+  </si>
+  <si>
+    <t>BSC</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>Ammeter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local Controller can access the following equipments: </t>
+  </si>
+  <si>
+    <t>LCU</t>
+  </si>
+  <si>
+    <t>B, C, D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -385,21 +532,31 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -423,19 +580,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -771,7 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:AQ65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.1640625" customWidth="1"/>
@@ -785,46 +966,46 @@
     <col min="9" max="9" width="15.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="6" t="s">
         <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>1</v>
@@ -837,285 +1018,294 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="7" t="s">
         <v>16</v>
       </c>
+      <c r="G2" s="8"/>
       <c r="M2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="N2" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="9" t="s">
         <v>21</v>
       </c>
+      <c r="G3" s="8"/>
       <c r="M3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="N3" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="10">
         <v>0.1</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="10">
         <v>0.3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="10">
         <v>0.5</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="10">
         <v>1</v>
       </c>
+      <c r="G4" s="8"/>
       <c r="M4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="N4">
-        <v>3</v>
+      <c r="N4" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>27</v>
       </c>
+      <c r="G5" s="8"/>
       <c r="M5" t="s">
         <v>8</v>
       </c>
-      <c r="N5">
-        <v>3</v>
+      <c r="N5" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="7" t="s">
         <v>32</v>
       </c>
+      <c r="G6" s="8"/>
       <c r="M6" t="s">
         <v>7</v>
       </c>
-      <c r="N6">
-        <v>3</v>
+      <c r="N6" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="7" t="s">
         <v>37</v>
       </c>
+      <c r="G7" s="8"/>
       <c r="M7" t="s">
         <v>6</v>
       </c>
-      <c r="N7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+      <c r="N7" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="7" t="s">
         <v>42</v>
       </c>
+      <c r="G8" s="8"/>
       <c r="M8" t="s">
         <v>6</v>
       </c>
-      <c r="N8">
-        <v>3</v>
+      <c r="N8" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="7" t="s">
         <v>47</v>
       </c>
+      <c r="G9" s="8"/>
       <c r="M9" t="s">
         <v>9</v>
       </c>
-      <c r="N9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+      <c r="N9" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="7" t="s">
         <v>52</v>
       </c>
+      <c r="G10" s="8"/>
       <c r="M10" t="s">
         <v>6</v>
       </c>
-      <c r="N10">
-        <v>3</v>
+      <c r="N10" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="7" t="s">
         <v>58</v>
       </c>
       <c r="M11" t="s">
         <v>59</v>
       </c>
       <c r="N11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="34" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="12" t="s">
         <v>65</v>
       </c>
       <c r="M12" t="s">
@@ -1125,260 +1315,911 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="34" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="7" t="s">
         <v>71</v>
       </c>
+      <c r="G13" s="8"/>
       <c r="H13" s="2"/>
-      <c r="M13" s="4" t="s">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="3" t="s">
         <v>72</v>
       </c>
       <c r="N13">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="2" t="b">
+      <c r="C14" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="D14" s="2" t="b">
+      <c r="D14" s="9" t="b">
         <v>0</v>
       </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
       <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
       <c r="M14" t="s">
         <v>6</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="2" t="b">
+      <c r="C15" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="D15" s="2" t="b">
+      <c r="D15" s="9" t="b">
         <v>0</v>
       </c>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
       <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
       <c r="M15" t="s">
         <v>7</v>
       </c>
       <c r="N15">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="2" t="b">
+      <c r="C16" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="D16" s="2" t="b">
+      <c r="D16" s="9" t="b">
         <v>0</v>
       </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
       <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
       <c r="M16" t="s">
         <v>7</v>
       </c>
       <c r="N16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:43" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="2" t="b">
+      <c r="C17" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="D17" s="2" t="b">
+      <c r="D17" s="9" t="b">
         <v>0</v>
       </c>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
       <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
       <c r="M17" t="s">
         <v>7</v>
       </c>
       <c r="N17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" s="11" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:43" s="5" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="K18" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="L18" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D18" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="K18" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="M18" s="11" t="s">
+      <c r="M18" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="N18" s="11">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="N18">
+        <v>24</v>
+      </c>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+      <c r="W18"/>
+      <c r="X18"/>
+      <c r="Y18"/>
+      <c r="Z18"/>
+      <c r="AA18"/>
+      <c r="AB18"/>
+      <c r="AC18"/>
+      <c r="AD18"/>
+      <c r="AE18"/>
+      <c r="AF18"/>
+      <c r="AG18"/>
+      <c r="AH18"/>
+      <c r="AI18"/>
+      <c r="AJ18"/>
+      <c r="AK18"/>
+      <c r="AL18"/>
+      <c r="AM18"/>
+      <c r="AN18"/>
+      <c r="AO18"/>
+      <c r="AP18"/>
+      <c r="AQ18"/>
+    </row>
+    <row r="19" spans="1:43" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="7" t="s">
         <v>78</v>
       </c>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
       <c r="N19">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+    <row r="20" spans="1:43" ht="17" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
       <c r="M20" s="2"/>
       <c r="N20">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="17" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+    <row r="21" spans="1:43" ht="17" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
       <c r="N21">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
+    <row r="22" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="M22" t="s">
+        <v>7</v>
+      </c>
+      <c r="N22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="8"/>
+      <c r="M23" t="s">
+        <v>6</v>
+      </c>
+      <c r="N23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="M24" t="s">
+        <v>6</v>
+      </c>
+      <c r="N24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="M25" t="s">
+        <v>8</v>
+      </c>
+      <c r="N25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D26" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="M26" t="s">
+        <v>7</v>
+      </c>
+      <c r="N26">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="M27" t="s">
+        <v>6</v>
+      </c>
+      <c r="N27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28" s="8">
+        <v>4</v>
+      </c>
+      <c r="D28" s="8">
+        <v>3</v>
+      </c>
+      <c r="E28" s="8">
+        <v>2</v>
+      </c>
+      <c r="F28" s="8">
+        <v>1</v>
+      </c>
+      <c r="G28" s="8"/>
+      <c r="M28" t="s">
+        <v>8</v>
+      </c>
+      <c r="N28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="M29" t="s">
+        <v>7</v>
+      </c>
+      <c r="N29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G30" s="8"/>
+      <c r="M30" t="s">
+        <v>9</v>
+      </c>
+      <c r="N30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G31" s="8"/>
+      <c r="M31" t="s">
+        <v>8</v>
+      </c>
+      <c r="N31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:43" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G32" s="8"/>
+      <c r="M32" t="s">
+        <v>126</v>
+      </c>
+      <c r="N32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" s="8"/>
+      <c r="M33" t="s">
+        <v>132</v>
+      </c>
+      <c r="N33">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G34" s="8"/>
+      <c r="M34" t="s">
+        <v>7</v>
+      </c>
+      <c r="N34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G35" s="8"/>
+      <c r="M35" t="s">
+        <v>9</v>
+      </c>
+      <c r="N35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="G36" s="8"/>
+      <c r="M36" t="s">
+        <v>72</v>
+      </c>
+      <c r="N36">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="G37" s="8"/>
+      <c r="M37" t="s">
+        <v>146</v>
+      </c>
+      <c r="N37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
+      <c r="G55" s="8"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="8"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="8"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="8"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="8"/>
+      <c r="G61" s="8"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B62" s="8"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8"/>
+      <c r="G62" s="8"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B63" s="8"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="8"/>
+      <c r="G63" s="8"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B64" s="8"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="8"/>
+      <c r="G64" s="8"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B65" s="8"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1" xr:uid="{6B259FB3-67CD-2D46-80FA-4F1AF0636AEA}"/>
+    <hyperlink ref="E10" r:id="rId1" xr:uid="{AA4C6722-B2BD-E747-9576-5F96AC641EB9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update the PT2.0 Safety testing question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A460184-3BC5-ED49-BD64-53A6B9DF40D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2704692-7E97-3645-9AFF-A87B8E4129CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="164">
   <si>
     <t>Question Text</t>
   </si>
@@ -344,14 +344,197 @@
     <t>G</t>
   </si>
   <si>
-    <t>H</t>
+    <t>What Multimeter testing mode is needed when testing the busbars above QF1 and QF2 in the MVS?</t>
+  </si>
+  <si>
+    <t>What Multimeter testing mode is needed when testing the bubars below QF1 in the Battery Supply Panel?</t>
+  </si>
+  <si>
+    <t>How often should Class 0 gloves be inspected?</t>
+  </si>
+  <si>
+    <t>Before each use</t>
+  </si>
+  <si>
+    <t>After each use</t>
+  </si>
+  <si>
+    <t>Before and After each use</t>
+  </si>
+  <si>
+    <t>Every six months</t>
+  </si>
+  <si>
+    <t>The High Voltage room of the MVT is opened during the isolation procedure.</t>
+  </si>
+  <si>
+    <t>Which of the following are done in the LC during the LOTO process?</t>
+  </si>
+  <si>
+    <t>Switching the system to local mode</t>
+  </si>
+  <si>
+    <t>Key stopping the system</t>
+  </si>
+  <si>
+    <t>All of the above</t>
+  </si>
+  <si>
+    <t>What calorie rating is the bare minimum for CAT 4 PPE?</t>
+  </si>
+  <si>
+    <t>When a change in scope happens, work is immediately continued.</t>
+  </si>
+  <si>
+    <t>Which of the following is most effective for removing a hazard?</t>
+  </si>
+  <si>
+    <t>Elimination/Substitution</t>
+  </si>
+  <si>
+    <t>Engineering Controls</t>
+  </si>
+  <si>
+    <t>Administrative and Work Practice Controls</t>
+  </si>
+  <si>
+    <t>PPE</t>
+  </si>
+  <si>
+    <t>Prescription glasses are a valid replacement for protective eyeware.</t>
+  </si>
+  <si>
+    <t>Why is hearing protection recommended on site?</t>
+  </si>
+  <si>
+    <t>Our machines are very loud</t>
+  </si>
+  <si>
+    <t>Very loud music is played on site</t>
+  </si>
+  <si>
+    <t>Silence helps improve focus</t>
+  </si>
+  <si>
+    <t>Arc blasts can damage eardrums</t>
+  </si>
+  <si>
+    <t>How often do class 0 gloves need to be recertified?</t>
+  </si>
+  <si>
+    <t>Every 6 months</t>
+  </si>
+  <si>
+    <t>Every Year</t>
+  </si>
+  <si>
+    <t>Every 2 years</t>
+  </si>
+  <si>
+    <t>Every 10 years</t>
+  </si>
+  <si>
+    <t>Who is responsible for maintaining PPE?</t>
+  </si>
+  <si>
+    <t>Employer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sungrow </t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Safety Supervisor</t>
+  </si>
+  <si>
+    <t>CAT 4 suits are on size fits all.</t>
+  </si>
+  <si>
+    <t>Which of the following are potential slip hazards on a BESS site?</t>
+  </si>
+  <si>
+    <t>Transformer Oil</t>
+  </si>
+  <si>
+    <t>Coolant</t>
+  </si>
+  <si>
+    <t>Snow</t>
+  </si>
+  <si>
+    <t>Which type of hazard control is LOTO an example of?</t>
+  </si>
+  <si>
+    <t>Which type of hazard control are guardrails an example of?</t>
+  </si>
+  <si>
+    <t>Metal Ladders cannot be used on an energized work site.</t>
+  </si>
+  <si>
+    <t>Saving time is an adequate justification for energized work.</t>
+  </si>
+  <si>
+    <t>Insulators are always able to stop the flow of electricity.</t>
+  </si>
+  <si>
+    <t>Even if an electrical burn doesn't appear serious the victim should still be examined by a medical professional.</t>
+  </si>
+  <si>
+    <t>Which of the following can cause a fire.</t>
+  </si>
+  <si>
+    <t>Too little resistance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Too much resistance </t>
+  </si>
+  <si>
+    <t>Improper termination of a wire</t>
+  </si>
+  <si>
+    <t>If no battery removal tool is present it is acceptable to attempt to pull out a battery pack without a tool.</t>
+  </si>
+  <si>
+    <t>A zip tie is an adequate lock.</t>
+  </si>
+  <si>
+    <t>Which of the following must be written on a tag during LOTO. (Select all that apply)</t>
+  </si>
+  <si>
+    <t>The name of the person who placed the lock</t>
+  </si>
+  <si>
+    <t>A means to contact the person who placed the lock</t>
+  </si>
+  <si>
+    <t>The birthday of the person who placed the lock</t>
+  </si>
+  <si>
+    <t>The voltage the lock is preventing from being turned on</t>
+  </si>
+  <si>
+    <t>A,B</t>
+  </si>
+  <si>
+    <t>Can a lock be removed without contacting the person who placed the lock.</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>If you are standing outside the arc flash boundary you can stil receive a 2nd degree burn in the event of an arc.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -384,6 +567,14 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -409,9 +600,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -746,23 +937,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:L29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K50"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="129.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -791,360 +978,360 @@
         <v>101</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" s="2" t="s">
+      <c r="D3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="J3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" t="s">
+        <v>6</v>
+      </c>
+      <c r="K7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="J9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J10" t="s">
         <v>7</v>
       </c>
-      <c r="L2" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="4" t="b">
+      <c r="K10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="J11" t="s">
+        <v>97</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="D3" s="4" t="b">
+      <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="K3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" t="s">
-        <v>9</v>
-      </c>
-      <c r="L4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K5" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" t="s">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" t="s">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K8" t="s">
-        <v>6</v>
-      </c>
-      <c r="L8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="K9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" t="s">
         <v>7</v>
       </c>
-      <c r="L10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="K12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" t="s">
+        <v>7</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="K11" t="s">
-        <v>97</v>
-      </c>
-      <c r="L11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="K12" t="s">
-        <v>7</v>
-      </c>
-      <c r="L12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="2"/>
-      <c r="K13" t="s">
-        <v>7</v>
-      </c>
-      <c r="L13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="K14" t="s">
+      <c r="I14" s="2"/>
+      <c r="J14" t="s">
         <v>98</v>
       </c>
-      <c r="L14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>3</v>
       </c>
       <c r="D15">
@@ -1157,262 +1344,843 @@
         <v>12</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="K15" t="s">
+      <c r="I15" s="2"/>
+      <c r="J15" t="s">
         <v>6</v>
       </c>
-      <c r="L15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="4" t="b">
+      <c r="C16" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="D16" s="4" t="b">
+      <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="K16" t="s">
+      <c r="I16" s="2"/>
+      <c r="J16" t="s">
         <v>7</v>
       </c>
-      <c r="L16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="3" t="s">
         <v>69</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="K17" t="s">
+      <c r="I17" s="2"/>
+      <c r="J17" t="s">
         <v>8</v>
       </c>
-      <c r="L17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="4" t="b">
+      <c r="C18" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
       </c>
-      <c r="K18" t="s">
+      <c r="J18" t="s">
         <v>6</v>
       </c>
-      <c r="L18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="J19" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="L19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="4" t="b">
+      <c r="C20" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D20" t="b">
         <v>0</v>
       </c>
-      <c r="K20" t="s">
+      <c r="J20" t="s">
         <v>7</v>
       </c>
-      <c r="L20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="K21" t="s">
+      <c r="J21" t="s">
         <v>7</v>
       </c>
-      <c r="L21">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K22" t="s">
+      <c r="J22" t="s">
         <v>100</v>
       </c>
-      <c r="L22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="K23" t="s">
+      <c r="J23" t="s">
         <v>8</v>
       </c>
-      <c r="L23">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="J24" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L24">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
+      <c r="K24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="J25" t="s">
+        <v>7</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="J26" t="s">
+        <v>7</v>
+      </c>
+      <c r="K26">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J27" t="s">
+        <v>8</v>
+      </c>
+      <c r="K27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" t="s">
+        <v>6</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J29" t="s">
+        <v>9</v>
+      </c>
+      <c r="K29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30">
+        <v>30</v>
+      </c>
+      <c r="D30">
+        <v>40</v>
+      </c>
+      <c r="E30">
+        <v>50</v>
+      </c>
+      <c r="F30">
+        <v>60</v>
+      </c>
+      <c r="J30" t="s">
+        <v>6</v>
+      </c>
+      <c r="K30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" t="s">
+        <v>6</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C32" t="s">
+        <v>117</v>
+      </c>
+      <c r="D32" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" t="s">
+        <v>119</v>
+      </c>
+      <c r="F32" t="s">
+        <v>120</v>
+      </c>
+      <c r="J32" t="s">
+        <v>7</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" t="s">
+        <v>6</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C34" t="s">
+        <v>123</v>
+      </c>
+      <c r="D34" t="s">
+        <v>124</v>
+      </c>
+      <c r="E34" t="s">
+        <v>125</v>
+      </c>
+      <c r="F34" t="s">
+        <v>126</v>
+      </c>
+      <c r="J34" t="s">
+        <v>9</v>
+      </c>
+      <c r="K34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C35" t="s">
+        <v>128</v>
+      </c>
+      <c r="D35" t="s">
+        <v>129</v>
+      </c>
+      <c r="E35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F35" t="s">
+        <v>131</v>
+      </c>
+      <c r="J35" t="s">
+        <v>7</v>
+      </c>
+      <c r="K35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" t="s">
+        <v>133</v>
+      </c>
+      <c r="D36" t="s">
+        <v>134</v>
+      </c>
+      <c r="E36" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" t="s">
+        <v>136</v>
+      </c>
+      <c r="J36" t="s">
+        <v>8</v>
+      </c>
+      <c r="K36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C37" t="b">
+        <v>1</v>
+      </c>
+      <c r="D37" t="b">
+        <v>0</v>
+      </c>
+      <c r="J37" t="s">
+        <v>6</v>
+      </c>
+      <c r="K37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C38" t="s">
+        <v>139</v>
+      </c>
+      <c r="D38" t="s">
+        <v>140</v>
+      </c>
+      <c r="E38" t="s">
+        <v>141</v>
+      </c>
+      <c r="F38" t="s">
+        <v>113</v>
+      </c>
+      <c r="J38" t="s">
+        <v>9</v>
+      </c>
+      <c r="K38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C39" t="s">
+        <v>117</v>
+      </c>
+      <c r="D39" t="s">
+        <v>118</v>
+      </c>
+      <c r="E39" t="s">
+        <v>119</v>
+      </c>
+      <c r="F39" t="s">
+        <v>120</v>
+      </c>
+      <c r="J39" t="s">
+        <v>8</v>
+      </c>
+      <c r="K39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C40" t="s">
+        <v>117</v>
+      </c>
+      <c r="D40" t="s">
+        <v>118</v>
+      </c>
+      <c r="E40" t="s">
+        <v>119</v>
+      </c>
+      <c r="F40" t="s">
+        <v>120</v>
+      </c>
+      <c r="J40" t="s">
+        <v>6</v>
+      </c>
+      <c r="K40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C41" t="b">
+        <v>1</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" t="s">
+        <v>7</v>
+      </c>
+      <c r="K41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C42" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" t="s">
+        <v>6</v>
+      </c>
+      <c r="K42">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" t="b">
+        <v>1</v>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+      <c r="J43" t="s">
+        <v>6</v>
+      </c>
+      <c r="K43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C44" t="b">
+        <v>1</v>
+      </c>
+      <c r="D44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="s">
+        <v>7</v>
+      </c>
+      <c r="K44">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D45" t="s">
+        <v>150</v>
+      </c>
+      <c r="E45" t="s">
+        <v>151</v>
+      </c>
+      <c r="F45" t="s">
+        <v>113</v>
+      </c>
+      <c r="J45" t="s">
+        <v>9</v>
+      </c>
+      <c r="K45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C46" t="b">
+        <v>1</v>
+      </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" t="s">
+        <v>6</v>
+      </c>
+      <c r="K46">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C47" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47" t="b">
+        <v>0</v>
+      </c>
+      <c r="J47" t="s">
+        <v>6</v>
+      </c>
+      <c r="K47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C48" t="s">
+        <v>155</v>
+      </c>
+      <c r="D48" t="s">
+        <v>156</v>
+      </c>
+      <c r="E48" t="s">
+        <v>157</v>
+      </c>
+      <c r="F48" t="s">
+        <v>158</v>
+      </c>
+      <c r="J48" t="s">
+        <v>159</v>
+      </c>
+      <c r="K48">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C49" t="s">
+        <v>161</v>
+      </c>
+      <c r="D49" t="s">
+        <v>162</v>
+      </c>
+      <c r="J49" t="s">
+        <v>6</v>
+      </c>
+      <c r="K49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C50" t="b">
+        <v>1</v>
+      </c>
+      <c r="D50" t="b">
+        <v>0</v>
+      </c>
+      <c r="J50" t="s">
+        <v>7</v>
+      </c>
+      <c r="K50">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update the PT2.0 CSP testing question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CF6380-0695-A24E-A148-A483E23954D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98330A9B-BA95-CE49-B3D6-3B7DC49CA484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="153">
   <si>
     <t>Question Text</t>
   </si>
@@ -119,21 +119,6 @@
     <t>192.168.0.50</t>
   </si>
   <si>
-    <t>0.5C (2 hour) variants of the battery containers have __ load switches in the Battery Collection Panel and __ PCS units per rack.</t>
-  </si>
-  <si>
-    <t>6, 2</t>
-  </si>
-  <si>
-    <t>3, 2</t>
-  </si>
-  <si>
-    <t>6, 1</t>
-  </si>
-  <si>
-    <t>3, 1</t>
-  </si>
-  <si>
     <t>The Main AC Circuit Breakers (QF1 and QF2 of the SCC) automatically open upon pressing 'OFF' in the Local Controller Web Page.</t>
   </si>
   <si>
@@ -281,14 +266,242 @@
     <t>Text</t>
   </si>
   <si>
-    <t>H</t>
+    <t>0.5C (2 hour) variants of the battery containers have __ load switches.</t>
+  </si>
+  <si>
+    <t>What kind of password is needed to log into the LC300?</t>
+  </si>
+  <si>
+    <t>A universal password</t>
+  </si>
+  <si>
+    <t>A daily password generated by Sungrow</t>
+  </si>
+  <si>
+    <t>A daily password generated by site</t>
+  </si>
+  <si>
+    <t>No password is needed</t>
+  </si>
+  <si>
+    <t>In the 0.25C version of the PowerTitan 2.0 how many racks are connected to each PCS?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single </t>
+  </si>
+  <si>
+    <t>How do the BMU and CMU boards communicate to each other?</t>
+  </si>
+  <si>
+    <t>Ethernet</t>
+  </si>
+  <si>
+    <t>RS485</t>
+  </si>
+  <si>
+    <t>CANBus</t>
+  </si>
+  <si>
+    <t>What kind of information is stored in the CMU board?</t>
+  </si>
+  <si>
+    <t>Pack Information</t>
+  </si>
+  <si>
+    <t>Rack Information</t>
+  </si>
+  <si>
+    <t>Battery Container Information</t>
+  </si>
+  <si>
+    <t>System Block Information</t>
+  </si>
+  <si>
+    <t>What kind of information does the BMU board provide?</t>
+  </si>
+  <si>
+    <t>What kind of information does the BSC monitor?</t>
+  </si>
+  <si>
+    <t>What kind of information does the LC monitor?</t>
+  </si>
+  <si>
+    <t>How often should cell balancing be done?</t>
+  </si>
+  <si>
+    <t>Once a week</t>
+  </si>
+  <si>
+    <t>Once a month</t>
+  </si>
+  <si>
+    <t>Every six months</t>
+  </si>
+  <si>
+    <t>Once a year</t>
+  </si>
+  <si>
+    <t>What is the rated capacity of a battery pack?</t>
+  </si>
+  <si>
+    <t>230 aH</t>
+  </si>
+  <si>
+    <t>280 aH</t>
+  </si>
+  <si>
+    <t>314 aH</t>
+  </si>
+  <si>
+    <t>690 aH</t>
+  </si>
+  <si>
+    <t>How are packs within a rack connected?</t>
+  </si>
+  <si>
+    <t>Series</t>
+  </si>
+  <si>
+    <t>Parallel</t>
+  </si>
+  <si>
+    <t>How many BMU boards are in each pack?</t>
+  </si>
+  <si>
+    <t>How many battery racks are there in one battery container?</t>
+  </si>
+  <si>
+    <t>How many CMU boards are there per battery rack?</t>
+  </si>
+  <si>
+    <t>The transfer boxes in the battery container have the same self sealing coolant connectors as the battery packs.</t>
+  </si>
+  <si>
+    <t>Where is the CMU located?</t>
+  </si>
+  <si>
+    <t>Inside the battery pack</t>
+  </si>
+  <si>
+    <t>Inside a PCS</t>
+  </si>
+  <si>
+    <t>Inside the LCU</t>
+  </si>
+  <si>
+    <t>Inside the terminal box</t>
+  </si>
+  <si>
+    <t>Which types of power conversion are the PCS unites capable of?</t>
+  </si>
+  <si>
+    <t>AC to DC</t>
+  </si>
+  <si>
+    <t>DC to AC</t>
+  </si>
+  <si>
+    <t>All of the above</t>
+  </si>
+  <si>
+    <t>None of the above</t>
+  </si>
+  <si>
+    <t>How is information from the CMUs accessed?</t>
+  </si>
+  <si>
+    <t>Connection to the CMU board view CANbus</t>
+  </si>
+  <si>
+    <t>In the CMU Monitor section on the BSC webpage</t>
+  </si>
+  <si>
+    <t>In the CMU Monitor section on the LC webpage</t>
+  </si>
+  <si>
+    <t>Through SCADA</t>
+  </si>
+  <si>
+    <t>How many AC load switches will there be in the Battery Collection Panel for the .5C version of the PowerTitan 2.0?</t>
+  </si>
+  <si>
+    <t>How many AC load switches will there be in the Battery Collection Panel for the .25C version of the PowerTitan 2.0?</t>
+  </si>
+  <si>
+    <t>Where is the BSC located withing the PowerTitan 2.0?</t>
+  </si>
+  <si>
+    <t>In the Battery Collection Panel</t>
+  </si>
+  <si>
+    <t>In the LCU</t>
+  </si>
+  <si>
+    <t>In the MVS</t>
+  </si>
+  <si>
+    <t>In the Battery Supply Panel</t>
+  </si>
+  <si>
+    <t>Where is QF1 in the Battery Supply Panel receiving power from? (Select the best answer)</t>
+  </si>
+  <si>
+    <t>The Batteries</t>
+  </si>
+  <si>
+    <t>PV Panels</t>
+  </si>
+  <si>
+    <t>The MVS</t>
+  </si>
+  <si>
+    <t>Site external power source</t>
+  </si>
+  <si>
+    <t>Which port in the Network Interface in the Battery Container is used when connection to the BSC?</t>
+  </si>
+  <si>
+    <t>Port 1</t>
+  </si>
+  <si>
+    <t>Port 2</t>
+  </si>
+  <si>
+    <t>Port 3</t>
+  </si>
+  <si>
+    <t>Port 4</t>
+  </si>
+  <si>
+    <t>The Battery System Controller communicates with the fire alarm control panel.</t>
+  </si>
+  <si>
+    <t>What is the voltage on the LV bushings of the MVT?</t>
+  </si>
+  <si>
+    <t>130V</t>
+  </si>
+  <si>
+    <t>230V</t>
+  </si>
+  <si>
+    <t>480V</t>
+  </si>
+  <si>
+    <t>690V</t>
+  </si>
+  <si>
+    <t>List the following components in order of power flow: Battery pack, MVT, BCP, PCS, MVS</t>
+  </si>
+  <si>
+    <t>List the following components in order of communicates. Start with the smallest level of communication: LC, BMU, BSC, CMU, SCADA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -322,6 +535,20 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -347,12 +574,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,24 +912,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:L29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="247" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="218.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="126" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -730,349 +950,346 @@
         <v>11</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="J2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="J3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="K4" t="s">
+      <c r="J4" t="s">
         <v>8</v>
       </c>
-      <c r="L4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K5" t="s">
-        <v>8</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="K6" t="s">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="J7" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C8" s="3">
+        <v>645</v>
+      </c>
+      <c r="D8" s="3">
+        <v>690</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F8" s="3">
+        <v>480</v>
+      </c>
+      <c r="J8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K7" t="s">
+      <c r="E9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" t="s">
         <v>7</v>
       </c>
-      <c r="L7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="6">
-        <v>645</v>
-      </c>
-      <c r="D8" s="6">
-        <v>690</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="6">
-        <v>480</v>
-      </c>
-      <c r="K8" t="s">
-        <v>6</v>
-      </c>
-      <c r="L8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="K10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K10" t="s">
+      <c r="G11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K12">
         <v>7</v>
       </c>
-      <c r="L10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="K11" t="s">
-        <v>56</v>
-      </c>
-      <c r="L11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="4" t="s">
+    </row>
+    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K12" t="s">
+      <c r="F13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="L12">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
-      <c r="K13" t="s">
-        <v>72</v>
-      </c>
-      <c r="L13">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="J13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="4" t="b">
+      <c r="B14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D14" t="b">
@@ -1080,21 +1297,21 @@
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="K14" t="s">
+      <c r="J14" t="s">
         <v>7</v>
       </c>
-      <c r="L14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="4" t="b">
+      <c r="B15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D15" t="b">
@@ -1102,41 +1319,41 @@
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
-      <c r="K15" t="s">
+      <c r="J15" t="s">
         <v>7</v>
       </c>
-      <c r="L15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="4" t="b">
+      <c r="B16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="D16" s="4" t="b">
+      <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="K16" t="s">
-        <v>6</v>
-      </c>
-      <c r="L16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="J16" t="s">
+        <v>6</v>
+      </c>
+      <c r="K16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>76</v>
+      <c r="B17" s="3" t="s">
+        <v>71</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1146,114 +1363,671 @@
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
-      <c r="K17" t="s">
-        <v>6</v>
-      </c>
-      <c r="L17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="4" t="b">
+      <c r="B18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
       </c>
-      <c r="K18" t="s">
-        <v>6</v>
-      </c>
-      <c r="L18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="J18" t="s">
+        <v>6</v>
+      </c>
+      <c r="K18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L19">
+      <c r="F20" t="s">
+        <v>81</v>
+      </c>
+      <c r="J20" t="s">
+        <v>6</v>
+      </c>
+      <c r="K20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="J21" t="s">
+        <v>6</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" t="s">
+        <v>87</v>
+      </c>
+      <c r="J22" t="s">
+        <v>9</v>
+      </c>
+      <c r="K22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" t="s">
+        <v>91</v>
+      </c>
+      <c r="F23" t="s">
+        <v>92</v>
+      </c>
+      <c r="J23" t="s">
+        <v>6</v>
+      </c>
+      <c r="K23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" t="s">
+        <v>91</v>
+      </c>
+      <c r="F24" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" t="s">
+        <v>7</v>
+      </c>
+      <c r="K24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" t="s">
+        <v>92</v>
+      </c>
+      <c r="J25" t="s">
+        <v>6</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" t="s">
+        <v>91</v>
+      </c>
+      <c r="F26" t="s">
+        <v>92</v>
+      </c>
+      <c r="J26" t="s">
+        <v>9</v>
+      </c>
+      <c r="K26">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" t="s">
+        <v>98</v>
+      </c>
+      <c r="E27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J27" t="s">
+        <v>6</v>
+      </c>
+      <c r="K27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" t="s">
+        <v>102</v>
+      </c>
+      <c r="D28" t="s">
+        <v>103</v>
+      </c>
+      <c r="E28" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" t="s">
+        <v>105</v>
+      </c>
+      <c r="J28" t="s">
+        <v>8</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" t="s">
+        <v>108</v>
+      </c>
+      <c r="J29" t="s">
+        <v>7</v>
+      </c>
+      <c r="K29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>4</v>
+      </c>
+      <c r="J30" t="s">
+        <v>6</v>
+      </c>
+      <c r="K30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31">
+        <v>6</v>
+      </c>
+      <c r="D31">
+        <v>10</v>
+      </c>
+      <c r="E31">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <v>24</v>
+      </c>
+      <c r="J31" t="s">
+        <v>8</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32">
+        <v>3</v>
+      </c>
+      <c r="F32">
+        <v>4</v>
+      </c>
+      <c r="J32" t="s">
+        <v>7</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" t="s">
+        <v>7</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" t="s">
+        <v>115</v>
+      </c>
+      <c r="E34" t="s">
+        <v>116</v>
+      </c>
+      <c r="F34" t="s">
+        <v>117</v>
+      </c>
+      <c r="J34" t="s">
+        <v>6</v>
+      </c>
+      <c r="K34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" t="s">
+        <v>119</v>
+      </c>
+      <c r="D35" t="s">
+        <v>120</v>
+      </c>
+      <c r="E35" t="s">
+        <v>121</v>
+      </c>
+      <c r="F35" t="s">
+        <v>122</v>
+      </c>
+      <c r="J35" t="s">
+        <v>8</v>
+      </c>
+      <c r="K35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C36" t="s">
+        <v>124</v>
+      </c>
+      <c r="D36" t="s">
+        <v>125</v>
+      </c>
+      <c r="E36" t="s">
+        <v>126</v>
+      </c>
+      <c r="F36" t="s">
+        <v>127</v>
+      </c>
+      <c r="J36" t="s">
+        <v>6</v>
+      </c>
+      <c r="K36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37">
+        <v>3</v>
+      </c>
+      <c r="D37">
+        <v>6</v>
+      </c>
+      <c r="E37">
+        <v>9</v>
+      </c>
+      <c r="F37">
+        <v>12</v>
+      </c>
+      <c r="J37" t="s">
+        <v>6</v>
+      </c>
+      <c r="K37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C38">
+        <v>12</v>
+      </c>
+      <c r="D38">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>6</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+      <c r="J38" t="s">
+        <v>9</v>
+      </c>
+      <c r="K38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" t="s">
+        <v>131</v>
+      </c>
+      <c r="D39" t="s">
+        <v>132</v>
+      </c>
+      <c r="E39" t="s">
+        <v>133</v>
+      </c>
+      <c r="F39" t="s">
+        <v>134</v>
+      </c>
+      <c r="J39" t="s">
+        <v>9</v>
+      </c>
+      <c r="K39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C40" t="s">
+        <v>136</v>
+      </c>
+      <c r="D40" t="s">
+        <v>137</v>
+      </c>
+      <c r="E40" t="s">
+        <v>138</v>
+      </c>
+      <c r="F40" t="s">
+        <v>139</v>
+      </c>
+      <c r="J40" t="s">
+        <v>8</v>
+      </c>
+      <c r="K40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C41" t="s">
+        <v>141</v>
+      </c>
+      <c r="D41" t="s">
+        <v>142</v>
+      </c>
+      <c r="E41" t="s">
+        <v>143</v>
+      </c>
+      <c r="F41" t="s">
+        <v>144</v>
+      </c>
+      <c r="J41" t="s">
+        <v>8</v>
+      </c>
+      <c r="K41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C42" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" t="s">
+        <v>7</v>
+      </c>
+      <c r="K42">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" t="s">
+        <v>147</v>
+      </c>
+      <c r="D43" t="s">
+        <v>148</v>
+      </c>
+      <c r="E43" t="s">
+        <v>149</v>
+      </c>
+      <c r="F43" t="s">
+        <v>150</v>
+      </c>
+      <c r="J43" t="s">
+        <v>9</v>
+      </c>
+      <c r="K43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="K44">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
+    <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="K45">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated the PT1.0 CSP Safety Test Pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9ADBBCD-6AD9-A941-8319-18FEE1D18518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C724FF59-E4CE-9C41-B702-23459945B6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="760" windowWidth="30840" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="900" yWindow="600" windowWidth="36000" windowHeight="19880" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="162">
   <si>
     <t>Question Text</t>
   </si>
@@ -381,6 +381,147 @@
   </si>
   <si>
     <t>There is no LOTO</t>
+  </si>
+  <si>
+    <t>Which switch in the Battey Supply pannel takes separate aux site power for the Exhaust Fans</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>Which switch is the main Aux switch in the battery supply pannel</t>
+  </si>
+  <si>
+    <t>Q2/Q3</t>
+  </si>
+  <si>
+    <t>In US version battery container, the Sprinkler is connected with water</t>
+  </si>
+  <si>
+    <t>Switch __ and __ can not be closed at the same time</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2 </t>
+  </si>
+  <si>
+    <t>B, C</t>
+  </si>
+  <si>
+    <t>Where is BSC located?</t>
+  </si>
+  <si>
+    <t>Battery container</t>
+  </si>
+  <si>
+    <t>PCS</t>
+  </si>
+  <si>
+    <t>MVS</t>
+  </si>
+  <si>
+    <t>On site</t>
+  </si>
+  <si>
+    <t>How does LC communicate to BSC</t>
+  </si>
+  <si>
+    <t>Bluetooth</t>
+  </si>
+  <si>
+    <t>Canbus</t>
+  </si>
+  <si>
+    <t>Ethernet</t>
+  </si>
+  <si>
+    <t>RS485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does BSC communicate to CMU </t>
+  </si>
+  <si>
+    <t>The DC power get converted to AC power in DCDC</t>
+  </si>
+  <si>
+    <t>The power come out from PCS to the grid is AC power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery pack A and pack B are mostly the same but different in </t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polarity </t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>The fuse is connected parallel with the batteries</t>
+  </si>
+  <si>
+    <t>How many packs form a rack</t>
+  </si>
+  <si>
+    <t>There is a BSC in each battery pack</t>
+  </si>
+  <si>
+    <t>When the DCDC indicator light is gray, It means the system is de-energized</t>
+  </si>
+  <si>
+    <t>At __ % LEL, FSS will fault off.</t>
+  </si>
+  <si>
+    <t>A lock need to be placed on the pressure relief valve during commissioning to prevent air release</t>
+  </si>
+  <si>
+    <t>Having an alarm on LC won't fault out the system</t>
+  </si>
+  <si>
+    <t>What is the last testing point in LOTO that verify no DC is flowing through the battery container?</t>
+  </si>
+  <si>
+    <t>Fuses in BCP</t>
+  </si>
+  <si>
+    <t>QS1 in BSP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuses in PCS </t>
+  </si>
+  <si>
+    <t>DC load switch in PCS</t>
+  </si>
+  <si>
+    <t>When will the nitrogen gas protection needs to be taken off?</t>
+  </si>
+  <si>
+    <t>During transportation</t>
+  </si>
+  <si>
+    <t>During Maintainance</t>
+  </si>
+  <si>
+    <t>Hot Commissioning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cold commissioning </t>
+  </si>
+  <si>
+    <t>What's the PPE requirement to enter a site?</t>
+  </si>
+  <si>
+    <t>Not needed yet</t>
+  </si>
+  <si>
+    <t>What's the PPE requirement during LOTO?</t>
   </si>
 </sst>
 </file>
@@ -441,12 +582,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,18 +925,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J46"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="146.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" customWidth="1"/>
+    <col min="2" max="2" width="143.1640625" customWidth="1"/>
+    <col min="3" max="3" width="37" customWidth="1"/>
+    <col min="4" max="4" width="41.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1640625" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -846,7 +991,7 @@
         <v>6</v>
       </c>
       <c r="J2" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -872,7 +1017,7 @@
         <v>6</v>
       </c>
       <c r="J3" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -897,8 +1042,8 @@
       <c r="I4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J4">
-        <v>4</v>
+      <c r="J4" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -923,8 +1068,8 @@
       <c r="I5" t="s">
         <v>6</v>
       </c>
-      <c r="J5">
-        <v>4</v>
+      <c r="J5" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -943,8 +1088,8 @@
       <c r="I6" t="s">
         <v>6</v>
       </c>
-      <c r="J6">
-        <v>4</v>
+      <c r="J6" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -966,8 +1111,8 @@
       <c r="I7" t="s">
         <v>8</v>
       </c>
-      <c r="J7">
-        <v>4</v>
+      <c r="J7" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -998,8 +1143,8 @@
       <c r="I8" t="s">
         <v>44</v>
       </c>
-      <c r="J8">
-        <v>5</v>
+      <c r="J8" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1027,8 +1172,8 @@
       <c r="I9" t="s">
         <v>51</v>
       </c>
-      <c r="J9">
-        <v>5</v>
+      <c r="J9" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1053,8 +1198,8 @@
       <c r="I10" t="s">
         <v>55</v>
       </c>
-      <c r="J10">
-        <v>5</v>
+      <c r="J10" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1079,8 +1224,8 @@
       <c r="I11" t="s">
         <v>6</v>
       </c>
-      <c r="J11">
-        <v>4</v>
+      <c r="J11" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1105,8 +1250,8 @@
       <c r="I12" t="s">
         <v>7</v>
       </c>
-      <c r="J12">
-        <v>4</v>
+      <c r="J12" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1132,8 +1277,8 @@
       <c r="I13" t="s">
         <v>6</v>
       </c>
-      <c r="J13">
-        <v>4</v>
+      <c r="J13" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1153,8 +1298,8 @@
       <c r="I14" t="s">
         <v>6</v>
       </c>
-      <c r="J14">
-        <v>4</v>
+      <c r="J14" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1185,8 +1330,8 @@
       <c r="I15" t="s">
         <v>77</v>
       </c>
-      <c r="J15">
-        <v>4</v>
+      <c r="J15" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1206,8 +1351,8 @@
       <c r="I16" t="s">
         <v>6</v>
       </c>
-      <c r="J16">
-        <v>4</v>
+      <c r="J16" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1233,7 +1378,7 @@
       <c r="I17" t="s">
         <v>55</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="2">
         <v>4</v>
       </c>
     </row>
@@ -1262,8 +1407,8 @@
       <c r="I18" t="s">
         <v>51</v>
       </c>
-      <c r="J18">
-        <v>5</v>
+      <c r="J18" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1291,8 +1436,8 @@
       <c r="I19" t="s">
         <v>11</v>
       </c>
-      <c r="J19">
-        <v>4</v>
+      <c r="J19" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1318,7 +1463,7 @@
       <c r="I20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="2">
         <v>4</v>
       </c>
     </row>
@@ -1341,8 +1486,8 @@
       <c r="I21" t="s">
         <v>7</v>
       </c>
-      <c r="J21">
-        <v>4</v>
+      <c r="J21" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1368,8 +1513,8 @@
       <c r="I22" t="s">
         <v>8</v>
       </c>
-      <c r="J22">
-        <v>4</v>
+      <c r="J22" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1395,8 +1540,8 @@
       <c r="I23" t="s">
         <v>6</v>
       </c>
-      <c r="J23">
-        <v>4</v>
+      <c r="J23" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1422,8 +1567,8 @@
       <c r="I24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J24">
-        <v>4</v>
+      <c r="J24" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="17" x14ac:dyDescent="0.25">
@@ -1449,26 +1594,507 @@
       <c r="I25" t="s">
         <v>8</v>
       </c>
-      <c r="J25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
+      <c r="J25" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>115</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" t="s">
+        <v>74</v>
+      </c>
+      <c r="I26" t="s">
+        <v>9</v>
+      </c>
+      <c r="J26" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" t="s">
+        <v>72</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="I27" t="s">
+        <v>8</v>
+      </c>
+      <c r="J27" s="2">
+        <v>5</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
+      <c r="A28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="s">
+        <v>6</v>
+      </c>
+      <c r="J28" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="I29" t="s">
+        <v>123</v>
+      </c>
+      <c r="J29" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C30" t="s">
+        <v>125</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" t="s">
+        <v>127</v>
+      </c>
+      <c r="F30" t="s">
+        <v>128</v>
+      </c>
+      <c r="I30" t="s">
+        <v>7</v>
+      </c>
+      <c r="J30" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E31" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="I31" t="s">
+        <v>8</v>
+      </c>
+      <c r="J31" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E32" t="s">
+        <v>132</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="I32" t="s">
+        <v>6</v>
+      </c>
+      <c r="J32" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="s">
+        <v>6</v>
+      </c>
+      <c r="J33" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="s">
+        <v>7</v>
+      </c>
+      <c r="J34" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" t="s">
+        <v>138</v>
+      </c>
+      <c r="D35" t="s">
+        <v>139</v>
+      </c>
+      <c r="E35" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" t="s">
+        <v>141</v>
+      </c>
+      <c r="I35" t="s">
+        <v>6</v>
+      </c>
+      <c r="J35" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>142</v>
+      </c>
+      <c r="C36" t="b">
+        <v>1</v>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="s">
+        <v>6</v>
+      </c>
+      <c r="J36" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>143</v>
+      </c>
+      <c r="C37">
+        <v>6</v>
+      </c>
+      <c r="D37">
+        <v>8</v>
+      </c>
+      <c r="E37">
+        <v>10</v>
+      </c>
+      <c r="F37">
+        <v>12</v>
+      </c>
+      <c r="I37" t="s">
+        <v>7</v>
+      </c>
+      <c r="J37" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="s">
+        <v>6</v>
+      </c>
+      <c r="J38" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" t="b">
+        <v>1</v>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="s">
+        <v>6</v>
+      </c>
+      <c r="J39" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>146</v>
+      </c>
+      <c r="C40">
+        <v>5</v>
+      </c>
+      <c r="D40">
+        <v>10</v>
+      </c>
+      <c r="E40">
+        <v>15</v>
+      </c>
+      <c r="F40">
+        <v>20</v>
+      </c>
+      <c r="I40" t="s">
+        <v>9</v>
+      </c>
+      <c r="J40" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>147</v>
+      </c>
+      <c r="C41" t="b">
+        <v>1</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="s">
+        <v>6</v>
+      </c>
+      <c r="J41" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>148</v>
+      </c>
+      <c r="C42" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="s">
+        <v>7</v>
+      </c>
+      <c r="J42" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>149</v>
+      </c>
+      <c r="C43" t="s">
+        <v>150</v>
+      </c>
+      <c r="D43" t="s">
+        <v>151</v>
+      </c>
+      <c r="E43" t="s">
+        <v>152</v>
+      </c>
+      <c r="F43" t="s">
+        <v>153</v>
+      </c>
+      <c r="I43" t="s">
+        <v>7</v>
+      </c>
+      <c r="J43" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" t="s">
+        <v>154</v>
+      </c>
+      <c r="C44" t="s">
+        <v>155</v>
+      </c>
+      <c r="D44" t="s">
+        <v>156</v>
+      </c>
+      <c r="E44" t="s">
+        <v>157</v>
+      </c>
+      <c r="F44" t="s">
+        <v>158</v>
+      </c>
+      <c r="I44" t="s">
+        <v>9</v>
+      </c>
+      <c r="J44" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
+        <v>159</v>
+      </c>
+      <c r="C45" t="s">
+        <v>30</v>
+      </c>
+      <c r="D45" t="s">
+        <v>31</v>
+      </c>
+      <c r="E45" t="s">
+        <v>32</v>
+      </c>
+      <c r="F45" t="s">
+        <v>160</v>
+      </c>
+      <c r="I45" t="s">
+        <v>7</v>
+      </c>
+      <c r="J45" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" t="s">
+        <v>161</v>
+      </c>
+      <c r="C46" t="s">
+        <v>30</v>
+      </c>
+      <c r="D46" t="s">
+        <v>31</v>
+      </c>
+      <c r="E46" t="s">
+        <v>32</v>
+      </c>
+      <c r="F46" t="s">
+        <v>160</v>
+      </c>
+      <c r="I46" t="s">
+        <v>8</v>
+      </c>
+      <c r="J46" s="2">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated the SG4400UD-MV Safety Questions Pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C064B60-9F58-F842-B671-E9D3F5038BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D33C32-FBEF-D340-B253-DE4C293BA04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2000" yWindow="600" windowWidth="33500" windowHeight="19880" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="182">
   <si>
     <t>Question Text</t>
   </si>
@@ -590,12 +590,6 @@
     <t>During the power-up cycle, can the MVT load switch be operated only by site personnel?</t>
   </si>
   <si>
-    <t xml:space="preserve"> True</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> False</t>
-  </si>
-  <si>
     <t>Should the Transformer MVT switch and DC combiner boxes be operated only by site personnel?</t>
   </si>
   <si>
@@ -606,6 +600,9 @@
   </si>
   <si>
     <t>A,B,C,D</t>
+  </si>
+  <si>
+    <t>The SG4400UD-MV skid has 28 DC inputs.</t>
   </si>
 </sst>
 </file>
@@ -673,12 +670,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1014,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1022,12 +1022,12 @@
     <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="88.6640625" customWidth="1"/>
     <col min="5" max="5" width="83" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="133.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="152.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -2048,7 +2048,7 @@
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
       <c r="J35" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="K35" s="3">
         <v>4</v>
@@ -2077,7 +2077,7 @@
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="J36" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="K36" s="3">
         <v>4</v>
@@ -2113,7 +2113,7 @@
         <v>4</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="C38" s="3" t="b">
         <v>1</v>
@@ -2127,7 +2127,7 @@
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="J38" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K38" s="3">
         <v>3</v>
@@ -2138,7 +2138,7 @@
         <v>4</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C39" s="3" t="b">
         <v>1</v>
@@ -2152,7 +2152,7 @@
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
       <c r="J39" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K39" s="3">
         <v>3</v>
@@ -2163,7 +2163,7 @@
         <v>4</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C40" s="3" t="b">
         <v>1</v>
@@ -2177,7 +2177,7 @@
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
       <c r="J40" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K40" s="3">
         <v>3</v>
@@ -2188,7 +2188,7 @@
         <v>4</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C41" s="3" t="b">
         <v>1</v>
@@ -2202,7 +2202,7 @@
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
       <c r="J41" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K41" s="3">
         <v>3</v>
@@ -2213,7 +2213,7 @@
         <v>4</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C42" s="3" t="b">
         <v>1</v>
@@ -2227,7 +2227,7 @@
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
       <c r="J42" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K42" s="3">
         <v>3</v>
@@ -2238,7 +2238,7 @@
         <v>4</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C43" s="3" t="b">
         <v>1</v>
@@ -2252,7 +2252,7 @@
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
       <c r="J43" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K43" s="3">
         <v>3</v>
@@ -2263,7 +2263,7 @@
         <v>4</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C44" s="3" t="b">
         <v>1</v>
@@ -2277,7 +2277,7 @@
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
       <c r="J44" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K44" s="3">
         <v>3</v>
@@ -2288,7 +2288,7 @@
         <v>4</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C45" s="3" t="b">
         <v>1</v>
@@ -2302,7 +2302,7 @@
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
       <c r="J45" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K45" s="3">
         <v>3</v>
@@ -2313,7 +2313,7 @@
         <v>4</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C46" s="3" t="b">
         <v>1</v>
@@ -2327,7 +2327,7 @@
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
       <c r="J46" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K46" s="3">
         <v>3</v>
@@ -2338,13 +2338,13 @@
         <v>4</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>178</v>
+        <v>175</v>
+      </c>
+      <c r="C47" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47" s="3" t="b">
+        <v>0</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -2352,7 +2352,7 @@
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
       <c r="J47" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K47" s="3">
         <v>3</v>
@@ -2363,13 +2363,13 @@
         <v>4</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
+      </c>
+      <c r="C48" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D48" s="3" t="b">
+        <v>0</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -2388,13 +2388,13 @@
         <v>4</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="C49" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>178</v>
+      <c r="C49" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D49" s="3" t="b">
+        <v>0</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -2402,7 +2402,7 @@
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
       <c r="J49" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K49" s="3">
         <v>3</v>
@@ -2413,13 +2413,13 @@
         <v>4</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D50" s="3" t="s">
         <v>178</v>
+      </c>
+      <c r="C50" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D50" s="3" t="b">
+        <v>0</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -2433,6 +2433,47 @@
         <v>3</v>
       </c>
     </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C51" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D51" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K51" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated a typo in the script.
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D33C32-FBEF-D340-B253-DE4C293BA04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A091A5-FC12-3D42-9FE1-E9CF6852E9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2000" yWindow="600" windowWidth="33500" windowHeight="19880" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19880" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1019,9 +1019,7 @@
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="168.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="88.6640625" customWidth="1"/>
-    <col min="5" max="5" width="83" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="149.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="152.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="2.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2.1640625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Updated the questions pool points weight
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4314835F-21BC-3C4C-8D88-1281C86ED003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2215081-E622-474A-9735-A718856D6E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="1680" windowWidth="31800" windowHeight="15580" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="2760" yWindow="1680" windowWidth="31800" windowHeight="18120" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="222">
   <si>
     <t>Question Text</t>
   </si>
@@ -483,21 +483,6 @@
   </si>
   <si>
     <t>Accurately record inverter operation during commissioning.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> What are the components of a GFI (Ground Fault Interrupter) detection circuit? </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t>(Select all that apply)</t>
-    </r>
   </si>
   <si>
     <t>KM5 (Contactor)</t>
@@ -857,7 +842,19 @@
     <t>If there is no incident energy sticker found on the power distribution/aux cabinet, I am permitted to access it while the skid is energized, as long as I have on a CAT4 suit.</t>
   </si>
   <si>
-    <t>G</t>
+    <r>
+      <t xml:space="preserve">What are the components of a GFI (Ground Fault Interrupter) detection circuit? </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Select all that apply)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1259,7 +1256,7 @@
     <col min="6" max="6" width="55.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="82.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="65" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -1288,12 +1285,9 @@
         <v>27</v>
       </c>
       <c r="I1" t="s">
-        <v>222</v>
+        <v>1</v>
       </c>
       <c r="J1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1318,13 +1312,13 @@
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="1">
-        <v>4</v>
-      </c>
+      <c r="J2" s="1">
+        <v>4</v>
+      </c>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1347,13 +1341,13 @@
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="1">
-        <v>4</v>
-      </c>
+      <c r="J3" s="1">
+        <v>4</v>
+      </c>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1376,13 +1370,13 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="1">
-        <v>4</v>
-      </c>
+      <c r="J4" s="1">
+        <v>4</v>
+      </c>
+      <c r="K4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -1405,13 +1399,13 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="1">
-        <v>4</v>
-      </c>
+      <c r="J5" s="1">
+        <v>4</v>
+      </c>
+      <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -1434,13 +1428,13 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="1">
-        <v>4</v>
-      </c>
+      <c r="J6" s="1">
+        <v>4</v>
+      </c>
+      <c r="K6" s="1"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
@@ -1463,13 +1457,13 @@
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="1">
-        <v>4</v>
-      </c>
+      <c r="J7" s="1">
+        <v>4</v>
+      </c>
+      <c r="K7" s="1"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -1492,13 +1486,13 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K8" s="1">
-        <v>4</v>
-      </c>
+      <c r="J8" s="1">
+        <v>4</v>
+      </c>
+      <c r="K8" s="1"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
@@ -1521,13 +1515,13 @@
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K9" s="1">
-        <v>4</v>
-      </c>
+      <c r="J9" s="1">
+        <v>4</v>
+      </c>
+      <c r="K9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
@@ -1550,13 +1544,13 @@
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K10" s="1">
-        <v>4</v>
-      </c>
+      <c r="J10" s="1">
+        <v>4</v>
+      </c>
+      <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -1579,13 +1573,13 @@
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K11" s="1">
-        <v>4</v>
-      </c>
+      <c r="J11" s="1">
+        <v>4</v>
+      </c>
+      <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
@@ -1608,13 +1602,13 @@
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="1">
-        <v>4</v>
-      </c>
+      <c r="J12" s="1">
+        <v>4</v>
+      </c>
+      <c r="K12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
@@ -1637,13 +1631,13 @@
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K13" s="1">
-        <v>4</v>
-      </c>
+      <c r="J13" s="1">
+        <v>4</v>
+      </c>
+      <c r="K13" s="1"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -1666,13 +1660,13 @@
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K14" s="1">
-        <v>4</v>
-      </c>
+      <c r="J14" s="1">
+        <v>4</v>
+      </c>
+      <c r="K14" s="1"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -1695,13 +1689,13 @@
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="1">
-        <v>4</v>
-      </c>
+      <c r="J15" s="1">
+        <v>4</v>
+      </c>
+      <c r="K15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -1724,13 +1718,13 @@
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K16" s="1">
-        <v>4</v>
-      </c>
+      <c r="J16" s="1">
+        <v>4</v>
+      </c>
+      <c r="K16" s="1"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
@@ -1753,13 +1747,13 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1" t="s">
+      <c r="I17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K17" s="1">
-        <v>4</v>
-      </c>
+      <c r="J17" s="1">
+        <v>4</v>
+      </c>
+      <c r="K17" s="1"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -1782,13 +1776,13 @@
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K18" s="1">
-        <v>4</v>
-      </c>
+      <c r="J18" s="1">
+        <v>4</v>
+      </c>
+      <c r="K18" s="1"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
@@ -1811,13 +1805,13 @@
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K19" s="1">
-        <v>4</v>
-      </c>
+      <c r="J19" s="1">
+        <v>4</v>
+      </c>
+      <c r="K19" s="1"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -1840,13 +1834,13 @@
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K20" s="1">
-        <v>4</v>
-      </c>
+      <c r="J20" s="1">
+        <v>4</v>
+      </c>
+      <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -1869,13 +1863,13 @@
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K21" s="1">
-        <v>4</v>
-      </c>
+      <c r="J21" s="1">
+        <v>4</v>
+      </c>
+      <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -1898,13 +1892,13 @@
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K22" s="1">
-        <v>4</v>
-      </c>
+      <c r="J22" s="1">
+        <v>4</v>
+      </c>
+      <c r="K22" s="1"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -1927,13 +1921,13 @@
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K23" s="1">
-        <v>4</v>
-      </c>
+      <c r="J23" s="1">
+        <v>4</v>
+      </c>
+      <c r="K23" s="1"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -1956,13 +1950,13 @@
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K24" s="1">
-        <v>4</v>
-      </c>
+      <c r="J24" s="1">
+        <v>4</v>
+      </c>
+      <c r="K24" s="1"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -1987,13 +1981,13 @@
         <v>121</v>
       </c>
       <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="K25" s="1">
-        <v>4</v>
-      </c>
+      <c r="J25" s="1">
+        <v>5</v>
+      </c>
+      <c r="K25" s="1"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -2020,13 +2014,13 @@
       <c r="H26" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="K26" s="1">
-        <v>4</v>
-      </c>
+      <c r="J26" s="1">
+        <v>5</v>
+      </c>
+      <c r="K26" s="1"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
@@ -2053,136 +2047,136 @@
       <c r="H27" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="K27" s="1">
-        <v>4</v>
-      </c>
+      <c r="J27" s="1">
+        <v>5</v>
+      </c>
+      <c r="K27" s="1"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="K28" s="1">
-        <v>4</v>
-      </c>
+      <c r="I28" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="J28" s="1">
+        <v>5</v>
+      </c>
+      <c r="K28" s="1"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K29" s="1">
-        <v>4</v>
-      </c>
+      <c r="J29" s="1">
+        <v>5</v>
+      </c>
+      <c r="K29" s="1"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>60</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K30" s="1">
-        <v>4</v>
-      </c>
+      <c r="J30" s="1">
+        <v>5</v>
+      </c>
+      <c r="K30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K31" s="1">
-        <v>4</v>
-      </c>
+      <c r="J31" s="1">
+        <v>5</v>
+      </c>
+      <c r="K31" s="1"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>33</v>
@@ -2198,20 +2192,20 @@
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="K32" s="1">
-        <v>4</v>
-      </c>
+      <c r="I32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="J32" s="1">
+        <v>5</v>
+      </c>
+      <c r="K32" s="1"/>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>28</v>
@@ -2227,13 +2221,13 @@
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K33" s="1">
-        <v>4</v>
-      </c>
+      <c r="I33" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="J33" s="1">
+        <v>5</v>
+      </c>
+      <c r="K33" s="1"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
@@ -2246,299 +2240,299 @@
         <v>5</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="K34" s="1">
-        <v>4</v>
-      </c>
+      <c r="I34" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="J34" s="1">
+        <v>5</v>
+      </c>
+      <c r="K34" s="1"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="K35" s="1">
-        <v>4</v>
-      </c>
+      <c r="I35" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="J35" s="1">
+        <v>5</v>
+      </c>
+      <c r="K35" s="1"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="K36" s="1">
-        <v>4</v>
-      </c>
+      <c r="I36" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="J36" s="1">
+        <v>5</v>
+      </c>
+      <c r="K36" s="1"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="K37" s="1">
-        <v>4</v>
-      </c>
+      <c r="I37" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="J37" s="1">
+        <v>5</v>
+      </c>
+      <c r="K37" s="1"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="K38" s="1">
-        <v>4</v>
-      </c>
+      <c r="I38" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="J38" s="1">
+        <v>5</v>
+      </c>
+      <c r="K38" s="1"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-      <c r="J39" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="K39" s="1">
-        <v>4</v>
-      </c>
+      <c r="I39" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="J39" s="1">
+        <v>5</v>
+      </c>
+      <c r="K39" s="1"/>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B40" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K40" s="1">
-        <v>4</v>
-      </c>
+      <c r="I40" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="J40" s="1">
+        <v>5</v>
+      </c>
+      <c r="K40" s="1"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B41" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="K41" s="1">
-        <v>4</v>
-      </c>
+      <c r="I41" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="J41" s="1">
+        <v>5</v>
+      </c>
+      <c r="K41" s="1"/>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>208</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="K42" s="1">
-        <v>4</v>
-      </c>
+      <c r="I42" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="J42" s="1">
+        <v>5</v>
+      </c>
+      <c r="K42" s="1"/>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="K43" s="1">
-        <v>4</v>
-      </c>
+      <c r="J43" s="1">
+        <v>5</v>
+      </c>
+      <c r="K43" s="1"/>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C44" s="1" t="b">
         <v>1</v>
@@ -2550,20 +2544,20 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-      <c r="J44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K44" s="1">
-        <v>3</v>
-      </c>
+      <c r="J44" s="1">
+        <v>4</v>
+      </c>
+      <c r="K44" s="1"/>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C45" s="1" t="b">
         <v>1</v>
@@ -2575,20 +2569,20 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K45" s="1">
-        <v>3</v>
-      </c>
+      <c r="J45" s="1">
+        <v>4</v>
+      </c>
+      <c r="K45" s="1"/>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C46" s="1" t="b">
         <v>1</v>
@@ -2600,20 +2594,20 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="J46" s="1" t="s">
+      <c r="I46" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K46" s="1">
-        <v>3</v>
-      </c>
+      <c r="J46" s="1">
+        <v>4</v>
+      </c>
+      <c r="K46" s="1"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C47" s="1" t="b">
         <v>1</v>
@@ -2625,20 +2619,20 @@
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K47" s="1">
-        <v>3</v>
-      </c>
+      <c r="J47" s="1">
+        <v>4</v>
+      </c>
+      <c r="K47" s="1"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C48" s="1" t="b">
         <v>1</v>
@@ -2650,13 +2644,13 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1" t="s">
+      <c r="I48" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K48" s="1">
-        <v>3</v>
-      </c>
+      <c r="J48" s="1">
+        <v>4</v>
+      </c>
+      <c r="K48" s="1"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
@@ -2675,20 +2669,20 @@
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1" t="s">
+      <c r="I49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K49" s="1">
-        <v>3</v>
-      </c>
+      <c r="J49" s="1">
+        <v>4</v>
+      </c>
+      <c r="K49" s="1"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C50" s="1" t="b">
         <v>1</v>
@@ -2700,20 +2694,20 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1" t="s">
+      <c r="I50" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K50" s="1">
-        <v>3</v>
-      </c>
+      <c r="J50" s="1">
+        <v>4</v>
+      </c>
+      <c r="K50" s="1"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C51" s="1" t="b">
         <v>1</v>
@@ -2725,13 +2719,13 @@
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K51" s="1">
-        <v>3</v>
-      </c>
+      <c r="J51" s="1">
+        <v>4</v>
+      </c>
+      <c r="K51" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update question pool for PT1.0-CSP-Safety
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT1_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C724FF59-E4CE-9C41-B702-23459945B6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D611F50-88D7-1249-B512-799D06946B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="600" windowWidth="36000" windowHeight="19880" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{F6BB879B-BAA8-D548-B6AE-4A8E8CC9CCF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,295 +38,295 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="162">
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Question Text</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
     <t>Correct Answer</t>
   </si>
   <si>
     <t>Points</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Single</t>
   </si>
   <si>
+    <t>You can test for zero voltage from the AC capacitors in the PCS immediately after the AC breaker if opened.</t>
+  </si>
+  <si>
+    <t>Which of the following must be changed in the Local controller before beginning to isolate a unit?</t>
+  </si>
+  <si>
+    <t>Minimum number of racks in operation</t>
+  </si>
+  <si>
+    <t>Change from Local/Remote to Local Mode</t>
+  </si>
+  <si>
+    <t>Rated power of the PCS</t>
+  </si>
+  <si>
+    <t>Clear Faults</t>
+  </si>
+  <si>
+    <t>At what voltage is a safety second required?</t>
+  </si>
+  <si>
+    <t>120V</t>
+  </si>
+  <si>
+    <t>230V</t>
+  </si>
+  <si>
+    <t>600V</t>
+  </si>
+  <si>
+    <t>480V</t>
+  </si>
+  <si>
+    <t>What is the minimum category PPE that must be worn to be on onsite.</t>
+  </si>
+  <si>
+    <t>Category 1</t>
+  </si>
+  <si>
+    <t>Category 2</t>
+  </si>
+  <si>
+    <t>Category 3</t>
+  </si>
+  <si>
+    <t>Category 4</t>
+  </si>
+  <si>
+    <t>If you wear prescription glasses those can be worn instead of ANSI Z87.1 eye ware?  </t>
+  </si>
+  <si>
+    <t>How often should you check your PPE for damages.</t>
+  </si>
+  <si>
+    <t>Before going to site</t>
+  </si>
+  <si>
+    <t>After going to site</t>
+  </si>
+  <si>
+    <t>Before and after each use</t>
+  </si>
+  <si>
     <t>Multi</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
+    <t>What are the 4 energy sources present in the Power Titan 1.0 battery container and PCS.</t>
+  </si>
+  <si>
+    <t>DC capacitors</t>
   </si>
   <si>
     <t>Wind Power</t>
   </si>
   <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
+    <t>AC capacitors</t>
+  </si>
+  <si>
+    <t>Batteries</t>
+  </si>
+  <si>
+    <t>Utility Power</t>
+  </si>
+  <si>
+    <t>Fire Power</t>
+  </si>
+  <si>
+    <t>A, C, D, E</t>
+  </si>
+  <si>
+    <t>What are all the points in the PCS and the Power Titan 1.0 battery container where site power is being fed?</t>
+  </si>
+  <si>
+    <t>QF1 in the BSP</t>
+  </si>
+  <si>
+    <t>Q3 in the PCS</t>
+  </si>
+  <si>
+    <t>Q7 in the BSP</t>
+  </si>
+  <si>
+    <t>Q2 in the PCS</t>
+  </si>
+  <si>
+    <t>Q1 in the PCS</t>
+  </si>
+  <si>
+    <t>A, C, D</t>
+  </si>
+  <si>
+    <t>Which of the Following need to be checked to verify that the AC capacitors are de-energized? Select all that apply.</t>
+  </si>
+  <si>
+    <t>AC Voltage</t>
+  </si>
+  <si>
+    <t>DC Voltage</t>
   </si>
   <si>
     <t>Capacitance</t>
   </si>
   <si>
-    <t>DC Voltage</t>
+    <t>Inductance</t>
+  </si>
+  <si>
+    <t>A, B</t>
+  </si>
+  <si>
+    <t>Where is Q7 in the Battery Supply Panel being powered from?</t>
+  </si>
+  <si>
+    <t>The DC/DC converters</t>
+  </si>
+  <si>
+    <t>The micro circuit breakers in the LC1000 cabinet</t>
+  </si>
+  <si>
+    <t>The BCP</t>
+  </si>
+  <si>
+    <t>Who is responsible for maintaining PPE?</t>
+  </si>
+  <si>
+    <t>The employee</t>
+  </si>
+  <si>
+    <t>The employer</t>
+  </si>
+  <si>
+    <t>The supervisor</t>
+  </si>
+  <si>
+    <t>The safety second</t>
+  </si>
+  <si>
+    <t>How do you connect your laptop to the LC200?</t>
+  </si>
+  <si>
+    <t>Using CANanalyst</t>
+  </si>
+  <si>
+    <t>Using ethernet</t>
+  </si>
+  <si>
+    <t>Using bluetooth</t>
+  </si>
+  <si>
+    <t>Using Wifi</t>
+  </si>
+  <si>
+    <t>If you are wearing category 4 PPE but your suit does not meet the calorie rating specified by the incident energy sticker you are still able to safely work on the equipment.</t>
+  </si>
+  <si>
+    <t>What are all the LOTO points on JUST the PCS? (As specified by Sungrow).</t>
+  </si>
+  <si>
+    <t>QF1</t>
+  </si>
+  <si>
+    <t>Q2 or Q3</t>
+  </si>
+  <si>
+    <t>Q7</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q8</t>
   </si>
   <si>
     <t>QS1</t>
   </si>
   <si>
+    <t>A, B, D, F</t>
+  </si>
+  <si>
+    <t>After you have finished isolating the system the batteries can be treated as dead.</t>
+  </si>
+  <si>
+    <t>What are all of the LOTO points in the battery container? (As specified by Sungrow)</t>
+  </si>
+  <si>
+    <t>DC/DC load switches</t>
+  </si>
+  <si>
+    <t>QS11</t>
+  </si>
+  <si>
+    <t>What are the steps that need to be taken to confirm zero voltage from the AC busbar in the PCS? Select all that apply.</t>
+  </si>
+  <si>
+    <t>Check phase to phase voltage</t>
+  </si>
+  <si>
+    <t>Check positive to negative</t>
+  </si>
+  <si>
+    <t>Check each phase to ground</t>
+  </si>
+  <si>
+    <t>Use proving unit before and after each measurement</t>
+  </si>
+  <si>
+    <t>Check ground to neutral</t>
+  </si>
+  <si>
+    <t>Above what voltage is live-dead-live (or hot-cold-hot) required?</t>
+  </si>
+  <si>
+    <t>230V </t>
+  </si>
+  <si>
+    <t>690V</t>
+  </si>
+  <si>
+    <t>All Voltages</t>
+  </si>
+  <si>
+    <t>What pieces of equipment are needed for live-dead-live (or hot-cold-hot) testing?</t>
+  </si>
+  <si>
+    <t>Multimeter</t>
+  </si>
+  <si>
+    <t>Hot stick</t>
+  </si>
+  <si>
+    <t>Proving unit</t>
+  </si>
+  <si>
+    <t>Non-contact voltage detector</t>
+  </si>
+  <si>
     <t>A, C</t>
-  </si>
-  <si>
-    <t>You can test for zero voltage from the AC capacitors in the PCS immediately after the AC breaker if opened.</t>
-  </si>
-  <si>
-    <t>Which of the following must be changed in the Local controller before beginning to isolate a unit?</t>
-  </si>
-  <si>
-    <t>Minimum number of racks in operation</t>
-  </si>
-  <si>
-    <t>Change from Local/Remote to Local Mode</t>
-  </si>
-  <si>
-    <t>Rated power of the PCS</t>
-  </si>
-  <si>
-    <t>Clear Faults</t>
-  </si>
-  <si>
-    <t>At what voltage is a safety second required?</t>
-  </si>
-  <si>
-    <t>120V</t>
-  </si>
-  <si>
-    <t>230V</t>
-  </si>
-  <si>
-    <t>600V</t>
-  </si>
-  <si>
-    <t>480V</t>
-  </si>
-  <si>
-    <t>What is the minimum category PPE that must be worn to be on onsite.</t>
-  </si>
-  <si>
-    <t>Category 1</t>
-  </si>
-  <si>
-    <t>Category 2</t>
-  </si>
-  <si>
-    <t>Category 3</t>
-  </si>
-  <si>
-    <t>Category 4</t>
-  </si>
-  <si>
-    <t>If you wear prescription glasses those can be worn instead of ANSI Z87.1 eye ware?  </t>
-  </si>
-  <si>
-    <t>How often should you check your PPE for damages.</t>
-  </si>
-  <si>
-    <t>Before going to site</t>
-  </si>
-  <si>
-    <t>After going to site</t>
-  </si>
-  <si>
-    <t>Before and after each use</t>
-  </si>
-  <si>
-    <t>What are the 4 energy sources present in the Power Titan 1.0 battery container and PCS.</t>
-  </si>
-  <si>
-    <t>DC capacitors</t>
-  </si>
-  <si>
-    <t>AC capacitors</t>
-  </si>
-  <si>
-    <t>Batteries</t>
-  </si>
-  <si>
-    <t>Utility Power</t>
-  </si>
-  <si>
-    <t>Fire Power</t>
-  </si>
-  <si>
-    <t>A, C, D, E</t>
-  </si>
-  <si>
-    <t>What are all the points in the PCS and the Power Titan 1.0 battery container where site power is being fed?</t>
-  </si>
-  <si>
-    <t>QF1 in the BSP</t>
-  </si>
-  <si>
-    <t>Q3 in the PCS</t>
-  </si>
-  <si>
-    <t>Q7 in the BSP</t>
-  </si>
-  <si>
-    <t>Q2 in the PCS</t>
-  </si>
-  <si>
-    <t>Q1 in the PCS</t>
-  </si>
-  <si>
-    <t>A, C, D</t>
-  </si>
-  <si>
-    <t>Which of the Following need to be checked to verify that the AC capacitors are de-energized? Select all that apply.</t>
-  </si>
-  <si>
-    <t>AC Voltage</t>
-  </si>
-  <si>
-    <t>Inductance</t>
-  </si>
-  <si>
-    <t>A, B</t>
-  </si>
-  <si>
-    <t>Where is Q7 in the Battery Supply Panel being powered from?</t>
-  </si>
-  <si>
-    <t>The DC/DC converters</t>
-  </si>
-  <si>
-    <t>The micro circuit breakers in the LC1000 cabinet</t>
-  </si>
-  <si>
-    <t>The BCP</t>
-  </si>
-  <si>
-    <t>Who is responsible for maintaining PPE?</t>
-  </si>
-  <si>
-    <t>The employee</t>
-  </si>
-  <si>
-    <t>The employer</t>
-  </si>
-  <si>
-    <t>The supervisor</t>
-  </si>
-  <si>
-    <t>The safety second</t>
-  </si>
-  <si>
-    <t>How do you connect your laptop to the LC200?</t>
-  </si>
-  <si>
-    <t>Using CANanalyst</t>
-  </si>
-  <si>
-    <t>Using ethernet</t>
-  </si>
-  <si>
-    <t>Using bluetooth</t>
-  </si>
-  <si>
-    <t>Using Wifi</t>
-  </si>
-  <si>
-    <t>If you are wearing category 4 PPE but your suit does not meet the calorie rating specified by the incident energy sticker you are still able to safely work on the equipment.</t>
-  </si>
-  <si>
-    <t>What are all the LOTO points on JUST the PCS? (As specified by Sungrow).</t>
-  </si>
-  <si>
-    <t>QF1</t>
-  </si>
-  <si>
-    <t>Q2 or Q3</t>
-  </si>
-  <si>
-    <t>Q7</t>
-  </si>
-  <si>
-    <t>Q1</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>A, B, D, F</t>
-  </si>
-  <si>
-    <t>After you have finished isolating the system the batteries can be treated as dead.</t>
-  </si>
-  <si>
-    <t>What are all of the LOTO points in the battery container? (As specified by Sungrow)</t>
-  </si>
-  <si>
-    <t>DC/DC load switches</t>
-  </si>
-  <si>
-    <t>QS11</t>
-  </si>
-  <si>
-    <t>What are the steps that need to be taken to confirm zero voltage from the AC busbar in the PCS? Select all that apply.</t>
-  </si>
-  <si>
-    <t>Check phase to phase voltage</t>
-  </si>
-  <si>
-    <t>Check positive to negative</t>
-  </si>
-  <si>
-    <t>Check each phase to ground</t>
-  </si>
-  <si>
-    <t>Use proving unit before and after each measurement</t>
-  </si>
-  <si>
-    <t>Check ground to neutral</t>
-  </si>
-  <si>
-    <t>Above what voltage is live-dead-live (or hot-cold-hot) required?</t>
-  </si>
-  <si>
-    <t>230V </t>
-  </si>
-  <si>
-    <t>690V</t>
-  </si>
-  <si>
-    <t>All Voltages</t>
-  </si>
-  <si>
-    <t>What pieces of equipment are needed for live-dead-live (or hot-cold-hot) testing?</t>
-  </si>
-  <si>
-    <t>Multimeter</t>
-  </si>
-  <si>
-    <t>Hot stick</t>
-  </si>
-  <si>
-    <t>Proving unit</t>
-  </si>
-  <si>
-    <t>Non-contact voltage detector</t>
   </si>
   <si>
     <t>The site LOTO procedure can include more steps than those included in the Sungrow LOTO procedure.</t>
@@ -532,15 +532,9 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF1B1C1D"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -553,6 +547,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1B1C1D"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
@@ -584,8 +584,8 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -619,39 +619,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -703,7 +703,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -814,6 +814,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -822,13 +829,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -893,453 +893,429 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B7BEAE-809A-6B44-81E1-03BCF0676C22}">
   <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" customWidth="1"/>
-    <col min="2" max="2" width="143.1640625" customWidth="1"/>
-    <col min="3" max="3" width="37" customWidth="1"/>
-    <col min="4" max="4" width="41.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.1640625" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="17.5" customWidth="1"/>
-    <col min="10" max="10" width="8.5" customWidth="1"/>
+    <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="3" t="b">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="b">
+      <c r="D2" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="2">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="2">
+      <c r="J4" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>6</v>
-      </c>
-      <c r="J5" s="2">
+        <v>3</v>
+      </c>
+      <c r="J5" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="3" t="b">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D6" s="3" t="b">
+      <c r="D6" s="2" t="b">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>6</v>
-      </c>
-      <c r="J6" s="2">
+        <v>3</v>
+      </c>
+      <c r="J6" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7" t="s">
-        <v>8</v>
-      </c>
-      <c r="J7" s="2">
+      <c r="J7" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="H8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="I8" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="I8" t="s">
-        <v>44</v>
-      </c>
-      <c r="J8" s="2">
-        <v>8</v>
+      <c r="J8" s="3">
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="I9" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="2">
-        <v>6</v>
+      <c r="J9" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="I10" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="I10" t="s">
-        <v>55</v>
-      </c>
-      <c r="J10" s="2">
-        <v>4</v>
+      <c r="J10" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>46</v>
+      <c r="F11" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="I11" t="s">
-        <v>6</v>
-      </c>
-      <c r="J11" s="2">
+        <v>3</v>
+      </c>
+      <c r="J11" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="I12" t="s">
-        <v>7</v>
-      </c>
-      <c r="J12" s="2">
+        <v>2</v>
+      </c>
+      <c r="J12" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" s="2"/>
+      <c r="H13" s="3"/>
       <c r="I13" t="s">
-        <v>6</v>
-      </c>
-      <c r="J13" s="2">
+        <v>3</v>
+      </c>
+      <c r="J13" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="3" t="b">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D14" s="3" t="b">
+      <c r="D14" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="2"/>
+      <c r="H14" s="3"/>
       <c r="I14" t="s">
-        <v>6</v>
-      </c>
-      <c r="J14" s="2">
+        <v>3</v>
+      </c>
+      <c r="J14" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="G15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="H15" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="I15" t="s">
         <v>76</v>
       </c>
-      <c r="H15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" t="s">
-        <v>77</v>
-      </c>
-      <c r="J15" s="2">
-        <v>8</v>
+      <c r="J15" s="3">
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>78</v>
+        <v>10</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>77</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
@@ -1347,338 +1323,338 @@
       <c r="D16" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="3"/>
       <c r="I16" t="s">
-        <v>6</v>
-      </c>
-      <c r="J16" s="2">
+        <v>3</v>
+      </c>
+      <c r="J16" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="3"/>
       <c r="I17" t="s">
-        <v>55</v>
-      </c>
-      <c r="J17" s="2">
-        <v>4</v>
+        <v>53</v>
+      </c>
+      <c r="J17" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="I18" t="s">
-        <v>51</v>
-      </c>
-      <c r="J18" s="2">
-        <v>6</v>
+        <v>47</v>
+      </c>
+      <c r="J18" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="I19" t="s">
-        <v>11</v>
-      </c>
-      <c r="J19" s="2">
+        <v>6</v>
+      </c>
+      <c r="J19" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3"/>
+      <c r="I20" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G20" s="2"/>
-      <c r="I20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="2">
-        <v>4</v>
+      <c r="J20" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C21" s="2" t="b">
+      <c r="C21" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="D21" s="2" t="b">
+      <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
       <c r="I21" t="s">
-        <v>7</v>
-      </c>
-      <c r="J21" s="2">
+        <v>2</v>
+      </c>
+      <c r="J21" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="3"/>
+      <c r="I22" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="G22" s="2"/>
-      <c r="I22" t="s">
-        <v>8</v>
-      </c>
-      <c r="J22" s="2">
+      <c r="J22" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G23" s="2"/>
+      <c r="F23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G23" s="3"/>
       <c r="I23" t="s">
-        <v>6</v>
-      </c>
-      <c r="J23" s="2">
+        <v>3</v>
+      </c>
+      <c r="J23" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="I24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J24" s="2">
+      <c r="G24" s="3"/>
+      <c r="I24" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J24" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G25" s="3"/>
+      <c r="I25" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G25" s="2"/>
-      <c r="I25" t="s">
-        <v>8</v>
-      </c>
-      <c r="J25" s="2">
+      <c r="J25" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="C26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F26" t="s">
-        <v>74</v>
-      </c>
       <c r="I26" t="s">
-        <v>9</v>
-      </c>
-      <c r="J26" s="2">
+        <v>5</v>
+      </c>
+      <c r="J26" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>75</v>
       </c>
+      <c r="D27" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="E27" t="s">
-        <v>72</v>
-      </c>
-      <c r="F27" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>118</v>
       </c>
       <c r="I27" t="s">
-        <v>8</v>
-      </c>
-      <c r="J27" s="2">
+        <v>4</v>
+      </c>
+      <c r="J27" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
         <v>119</v>
       </c>
-      <c r="C28" s="2" t="b">
+      <c r="C28" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D28" t="b">
         <v>0</v>
       </c>
       <c r="I28" t="s">
-        <v>6</v>
-      </c>
-      <c r="J28" s="2">
+        <v>3</v>
+      </c>
+      <c r="J28" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="B29" t="s">
         <v>120</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>75</v>
+      <c r="C29" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="D29" t="s">
         <v>121</v>
@@ -1686,19 +1662,19 @@
       <c r="E29" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="2" t="s">
         <v>122</v>
       </c>
       <c r="I29" t="s">
         <v>123</v>
       </c>
-      <c r="J29" s="2">
-        <v>4</v>
+      <c r="J29" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>124</v>
@@ -1706,7 +1682,7 @@
       <c r="C30" t="s">
         <v>125</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>126</v>
       </c>
       <c r="E30" t="s">
@@ -1716,67 +1692,67 @@
         <v>128</v>
       </c>
       <c r="I30" t="s">
-        <v>7</v>
-      </c>
-      <c r="J30" s="2">
+        <v>2</v>
+      </c>
+      <c r="J30" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
         <v>129</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>131</v>
       </c>
       <c r="E31" t="s">
         <v>132</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="2" t="s">
         <v>133</v>
       </c>
       <c r="I31" t="s">
-        <v>8</v>
-      </c>
-      <c r="J31" s="2">
+        <v>4</v>
+      </c>
+      <c r="J31" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
         <v>134</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="2" t="s">
         <v>131</v>
       </c>
       <c r="E32" t="s">
         <v>132</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="2" t="s">
         <v>133</v>
       </c>
       <c r="I32" t="s">
-        <v>6</v>
-      </c>
-      <c r="J32" s="2">
+        <v>3</v>
+      </c>
+      <c r="J32" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>135</v>
@@ -1788,15 +1764,15 @@
         <v>0</v>
       </c>
       <c r="I33" t="s">
-        <v>6</v>
-      </c>
-      <c r="J33" s="2">
+        <v>3</v>
+      </c>
+      <c r="J33" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
         <v>136</v>
@@ -1808,15 +1784,15 @@
         <v>0</v>
       </c>
       <c r="I34" t="s">
-        <v>7</v>
-      </c>
-      <c r="J34" s="2">
+        <v>2</v>
+      </c>
+      <c r="J34" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
         <v>137</v>
@@ -1834,15 +1810,15 @@
         <v>141</v>
       </c>
       <c r="I35" t="s">
-        <v>6</v>
-      </c>
-      <c r="J35" s="2">
+        <v>3</v>
+      </c>
+      <c r="J35" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
         <v>142</v>
@@ -1854,15 +1830,15 @@
         <v>0</v>
       </c>
       <c r="I36" t="s">
-        <v>6</v>
-      </c>
-      <c r="J36" s="2">
+        <v>3</v>
+      </c>
+      <c r="J36" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
         <v>143</v>
@@ -1880,15 +1856,15 @@
         <v>12</v>
       </c>
       <c r="I37" t="s">
-        <v>7</v>
-      </c>
-      <c r="J37" s="2">
+        <v>2</v>
+      </c>
+      <c r="J37" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
         <v>144</v>
@@ -1900,15 +1876,15 @@
         <v>0</v>
       </c>
       <c r="I38" t="s">
-        <v>6</v>
-      </c>
-      <c r="J38" s="2">
+        <v>3</v>
+      </c>
+      <c r="J38" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
         <v>145</v>
@@ -1920,15 +1896,15 @@
         <v>0</v>
       </c>
       <c r="I39" t="s">
-        <v>6</v>
-      </c>
-      <c r="J39" s="2">
+        <v>3</v>
+      </c>
+      <c r="J39" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B40" t="s">
         <v>146</v>
@@ -1946,15 +1922,15 @@
         <v>20</v>
       </c>
       <c r="I40" t="s">
-        <v>9</v>
-      </c>
-      <c r="J40" s="2">
+        <v>5</v>
+      </c>
+      <c r="J40" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B41" t="s">
         <v>147</v>
@@ -1966,15 +1942,15 @@
         <v>0</v>
       </c>
       <c r="I41" t="s">
-        <v>6</v>
-      </c>
-      <c r="J41" s="2">
+        <v>3</v>
+      </c>
+      <c r="J41" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B42" t="s">
         <v>148</v>
@@ -1986,15 +1962,15 @@
         <v>0</v>
       </c>
       <c r="I42" t="s">
-        <v>7</v>
-      </c>
-      <c r="J42" s="2">
+        <v>2</v>
+      </c>
+      <c r="J42" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
         <v>149</v>
@@ -2012,15 +1988,15 @@
         <v>153</v>
       </c>
       <c r="I43" t="s">
-        <v>7</v>
-      </c>
-      <c r="J43" s="2">
+        <v>2</v>
+      </c>
+      <c r="J43" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B44" t="s">
         <v>154</v>
@@ -2038,61 +2014,61 @@
         <v>158</v>
       </c>
       <c r="I44" t="s">
-        <v>9</v>
-      </c>
-      <c r="J44" s="2">
+        <v>5</v>
+      </c>
+      <c r="J44" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
         <v>159</v>
       </c>
       <c r="C45" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E45" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F45" t="s">
         <v>160</v>
       </c>
       <c r="I45" t="s">
-        <v>7</v>
-      </c>
-      <c r="J45" s="2">
+        <v>2</v>
+      </c>
+      <c r="J45" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B46" t="s">
         <v>161</v>
       </c>
       <c r="C46" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D46" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E46" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s">
         <v>160</v>
       </c>
       <c r="I46" t="s">
-        <v>8</v>
-      </c>
-      <c r="J46" s="2">
+        <v>4</v>
+      </c>
+      <c r="J46" s="3">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update question pool for PT2.0-CSP
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98330A9B-BA95-CE49-B3D6-3B7DC49CA484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F911A6-B4F6-8642-B53B-50CABDCC397A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,40 +38,64 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="153">
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Question Text</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
     <t>Correct Answer</t>
   </si>
   <si>
     <t>Points</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Single</t>
   </si>
   <si>
+    <t>You can upgrade the firmware of every BSC connected to an LC through the LC web portal.</t>
+  </si>
+  <si>
+    <t>230V</t>
+  </si>
+  <si>
+    <t>480V</t>
+  </si>
+  <si>
+    <t>690V</t>
+  </si>
+  <si>
     <t>Multi</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
+    <t>As long as I have properly isolated/de-energized the skid, I may replace a BMU board without insulating gloves.</t>
+  </si>
+  <si>
+    <t>Every six months</t>
+  </si>
+  <si>
+    <t>All of the above</t>
   </si>
   <si>
     <t>What is the voltage that feeds QF1 of the BESS containers for auxiliary power?</t>
@@ -119,6 +143,9 @@
     <t>192.168.0.50</t>
   </si>
   <si>
+    <t>0.5C (2 hour) variants of the battery containers have __ load switches.</t>
+  </si>
+  <si>
     <t>The Main AC Circuit Breakers (QF1 and QF2 of the SCC) automatically open upon pressing 'OFF' in the Local Controller Web Page.</t>
   </si>
   <si>
@@ -245,30 +272,18 @@
     <t>If the coolant pH falls below 7.3, it is required to replace the coolant</t>
   </si>
   <si>
-    <t>You can upgrade the firmware of every BSC connected to an LC through the LC web portal.</t>
-  </si>
-  <si>
     <t>The power-on switch on the injection/drainage tooling must be turned on to drain the coolant</t>
   </si>
   <si>
     <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, battery container doors can still be opened.</t>
   </si>
   <si>
-    <t>As long as I have properly isolated/de-energized the skid, I may replace a BMU board without insulating gloves.</t>
+    <t>Text</t>
   </si>
   <si>
     <t>According to the General Isolation Procedure (not to be used on site), name in order the testing points for de-energization, and what voltage mode (AC or DC) they need to be tested for. Also list, what are the 3 measurement-related equipment (not PPE) needed to safely test for de-energization.</t>
   </si>
   <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
-    <t>0.5C (2 hour) variants of the battery containers have __ load switches.</t>
-  </si>
-  <si>
     <t>What kind of password is needed to log into the LC300?</t>
   </si>
   <si>
@@ -335,9 +350,6 @@
     <t>Once a month</t>
   </si>
   <si>
-    <t>Every six months</t>
-  </si>
-  <si>
     <t>Once a year</t>
   </si>
   <si>
@@ -401,9 +413,6 @@
     <t>DC to AC</t>
   </si>
   <si>
-    <t>All of the above</t>
-  </si>
-  <si>
     <t>None of the above</t>
   </si>
   <si>
@@ -480,15 +489,6 @@
   </si>
   <si>
     <t>130V</t>
-  </si>
-  <si>
-    <t>230V</t>
-  </si>
-  <si>
-    <t>480V</t>
-  </si>
-  <si>
-    <t>690V</t>
   </si>
   <si>
     <t>List the following components in order of power flow: Battery pack, MVT, BCP, PCS, MVS</t>
@@ -911,7 +911,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42415D1-61AD-4746-A067-51E213EE90DC}">
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -926,60 +926,60 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K2" s="2">
         <v>5</v>
@@ -987,25 +987,25 @@
     </row>
     <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K3" s="2">
         <v>5</v>
@@ -1013,25 +1013,25 @@
     </row>
     <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
         <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" t="s">
-        <v>8</v>
       </c>
       <c r="K4">
         <v>5</v>
@@ -1039,10 +1039,10 @@
     </row>
     <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3">
         <v>2</v>
@@ -1057,7 +1057,7 @@
         <v>6</v>
       </c>
       <c r="J5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>5</v>
@@ -1065,10 +1065,10 @@
     </row>
     <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="b">
         <v>1</v>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -1085,25 +1085,25 @@
     </row>
     <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="J7" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <v>5</v>
@@ -1111,10 +1111,10 @@
     </row>
     <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C8" s="3">
         <v>645</v>
@@ -1123,13 +1123,13 @@
         <v>690</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="F8" s="3">
         <v>480</v>
       </c>
       <c r="J8" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -1137,25 +1137,25 @@
     </row>
     <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="J9" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -1163,25 +1163,25 @@
     </row>
     <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="J10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K10">
         <v>5</v>
@@ -1189,28 +1189,28 @@
     </row>
     <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="J11" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="K11">
         <v>5</v>
@@ -1218,65 +1218,65 @@
     </row>
     <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="J12" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="K12">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="K13">
         <v>5</v>
@@ -1284,10 +1284,10 @@
     </row>
     <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -1298,7 +1298,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K14">
         <v>5</v>
@@ -1306,10 +1306,10 @@
     </row>
     <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="C15" s="3" t="b">
         <v>1</v>
@@ -1320,7 +1320,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K15">
         <v>5</v>
@@ -1328,10 +1328,10 @@
     </row>
     <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C16" s="3" t="b">
         <v>1</v>
@@ -1342,7 +1342,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K16">
         <v>5</v>
@@ -1350,10 +1350,10 @@
     </row>
     <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1364,7 +1364,7 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K17">
         <v>5</v>
@@ -1372,10 +1372,10 @@
     </row>
     <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="C18" s="3" t="b">
         <v>1</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K18">
         <v>5</v>
@@ -1392,10 +1392,10 @@
     </row>
     <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="K19">
         <v>20</v>
@@ -1403,25 +1403,25 @@
     </row>
     <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="J20" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K20">
         <v>5</v>
@@ -1429,10 +1429,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1447,7 +1447,7 @@
         <v>4</v>
       </c>
       <c r="J21" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K21">
         <v>5</v>
@@ -1455,25 +1455,25 @@
     </row>
     <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J22" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K22">
         <v>5</v>
@@ -1481,25 +1481,25 @@
     </row>
     <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D23" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E23" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F23" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J23" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K23">
         <v>5</v>
@@ -1507,25 +1507,25 @@
     </row>
     <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E24" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J24" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K24">
         <v>5</v>
@@ -1533,25 +1533,25 @@
     </row>
     <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" t="s">
         <v>94</v>
       </c>
-      <c r="C25" t="s">
-        <v>89</v>
-      </c>
       <c r="D25" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E25" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F25" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J25" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K25">
         <v>5</v>
@@ -1559,25 +1559,25 @@
     </row>
     <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" t="s">
         <v>95</v>
       </c>
-      <c r="C26" t="s">
-        <v>89</v>
-      </c>
-      <c r="D26" t="s">
-        <v>90</v>
-      </c>
       <c r="E26" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F26" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J26" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K26">
         <v>5</v>
@@ -1585,25 +1585,25 @@
     </row>
     <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J27" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K27">
         <v>5</v>
@@ -1611,25 +1611,25 @@
     </row>
     <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" t="s">
+        <v>107</v>
+      </c>
+      <c r="E28" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" t="s">
+        <v>109</v>
+      </c>
+      <c r="J28" t="s">
         <v>4</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C28" t="s">
-        <v>102</v>
-      </c>
-      <c r="D28" t="s">
-        <v>103</v>
-      </c>
-      <c r="E28" t="s">
-        <v>104</v>
-      </c>
-      <c r="F28" t="s">
-        <v>105</v>
-      </c>
-      <c r="J28" t="s">
-        <v>8</v>
       </c>
       <c r="K28">
         <v>5</v>
@@ -1637,19 +1637,19 @@
     </row>
     <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C29" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="J29" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K29">
         <v>5</v>
@@ -1657,10 +1657,10 @@
     </row>
     <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1675,7 +1675,7 @@
         <v>4</v>
       </c>
       <c r="J30" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -1683,10 +1683,10 @@
     </row>
     <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C31">
         <v>6</v>
@@ -1701,7 +1701,7 @@
         <v>24</v>
       </c>
       <c r="J31" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K31">
         <v>5</v>
@@ -1709,10 +1709,10 @@
     </row>
     <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1727,7 +1727,7 @@
         <v>4</v>
       </c>
       <c r="J32" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K32">
         <v>5</v>
@@ -1735,10 +1735,10 @@
     </row>
     <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1747,7 +1747,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K33">
         <v>5</v>
@@ -1755,25 +1755,25 @@
     </row>
     <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D34" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E34" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F34" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="J34" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K34">
         <v>5</v>
@@ -1781,25 +1781,25 @@
     </row>
     <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" t="s">
+        <v>124</v>
+      </c>
+      <c r="E35" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" t="s">
+        <v>125</v>
+      </c>
+      <c r="J35" t="s">
         <v>4</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C35" t="s">
-        <v>119</v>
-      </c>
-      <c r="D35" t="s">
-        <v>120</v>
-      </c>
-      <c r="E35" t="s">
-        <v>121</v>
-      </c>
-      <c r="F35" t="s">
-        <v>122</v>
-      </c>
-      <c r="J35" t="s">
-        <v>8</v>
       </c>
       <c r="K35">
         <v>5</v>
@@ -1807,25 +1807,25 @@
     </row>
     <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D36" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E36" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F36" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="J36" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K36">
         <v>5</v>
@@ -1833,10 +1833,10 @@
     </row>
     <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C37">
         <v>3</v>
@@ -1851,7 +1851,7 @@
         <v>12</v>
       </c>
       <c r="J37" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K37">
         <v>5</v>
@@ -1859,10 +1859,10 @@
     </row>
     <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C38">
         <v>12</v>
@@ -1877,7 +1877,7 @@
         <v>3</v>
       </c>
       <c r="J38" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K38">
         <v>5</v>
@@ -1885,25 +1885,25 @@
     </row>
     <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E39" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F39" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J39" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K39">
         <v>5</v>
@@ -1911,25 +1911,25 @@
     </row>
     <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C40" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" t="s">
+        <v>140</v>
+      </c>
+      <c r="E40" t="s">
+        <v>141</v>
+      </c>
+      <c r="F40" t="s">
+        <v>142</v>
+      </c>
+      <c r="J40" t="s">
         <v>4</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C40" t="s">
-        <v>136</v>
-      </c>
-      <c r="D40" t="s">
-        <v>137</v>
-      </c>
-      <c r="E40" t="s">
-        <v>138</v>
-      </c>
-      <c r="F40" t="s">
-        <v>139</v>
-      </c>
-      <c r="J40" t="s">
-        <v>8</v>
       </c>
       <c r="K40">
         <v>5</v>
@@ -1937,25 +1937,25 @@
     </row>
     <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C41" t="s">
+        <v>144</v>
+      </c>
+      <c r="D41" t="s">
+        <v>145</v>
+      </c>
+      <c r="E41" t="s">
+        <v>146</v>
+      </c>
+      <c r="F41" t="s">
+        <v>147</v>
+      </c>
+      <c r="J41" t="s">
         <v>4</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C41" t="s">
-        <v>141</v>
-      </c>
-      <c r="D41" t="s">
-        <v>142</v>
-      </c>
-      <c r="E41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F41" t="s">
-        <v>144</v>
-      </c>
-      <c r="J41" t="s">
-        <v>8</v>
       </c>
       <c r="K41">
         <v>5</v>
@@ -1963,10 +1963,10 @@
     </row>
     <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C42" t="b">
         <v>1</v>
@@ -1975,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K42">
         <v>5</v>
@@ -1983,25 +1983,25 @@
     </row>
     <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D43" t="s">
-        <v>148</v>
+        <v>13</v>
       </c>
       <c r="E43" t="s">
-        <v>149</v>
+        <v>14</v>
       </c>
       <c r="F43" t="s">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="J43" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K43">
         <v>5</v>
@@ -2009,7 +2009,7 @@
     </row>
     <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>151</v>
@@ -2020,7 +2020,7 @@
     </row>
     <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>152</v>
@@ -2031,5 +2031,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" copies="8" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update question pool for PT2.0-CSP-Safety
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT2_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2704692-7E97-3645-9AFF-A87B8E4129CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7808970-0D2E-0B41-B60A-C80F83897062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20000" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{E8EEE946-DEB3-4041-95C0-A3908F45A14E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,229 +38,241 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="164">
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Question Text</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
     <t>Correct Answer</t>
   </si>
   <si>
     <t>Points</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Single</t>
   </si>
   <si>
+    <t>You can upgrade the firmware of every BSC connected to an LC through the LC web portal.</t>
+  </si>
+  <si>
+    <t>The site's LOTO procedure document</t>
+  </si>
+  <si>
+    <t>Sungrow's LOTO guidance document</t>
+  </si>
+  <si>
+    <t>Best judgement</t>
+  </si>
+  <si>
+    <t>PowerTitan 2.0 Power Cycle MOP</t>
+  </si>
+  <si>
+    <t>When turning off the system block from the LC, AC breakers QF1 and QF2 in the SCC open automatically.</t>
+  </si>
+  <si>
+    <t>What color LED indicator proves that the battery container is de-energized?</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>When the LED is off</t>
+  </si>
+  <si>
+    <t>The LED indicator doesn't prove de-energization</t>
+  </si>
+  <si>
+    <t>What is the voltage on the AC busbar between the main AC breakers in the SCC and the low voltage bushings of the Medium Voltage Transformer?</t>
+  </si>
+  <si>
+    <t>115V</t>
+  </si>
+  <si>
+    <t>230V</t>
+  </si>
+  <si>
+    <t>480V</t>
+  </si>
+  <si>
+    <t>690V</t>
+  </si>
+  <si>
+    <t>What is the AC voltage of the auxiliary power being fed into QF1 in the Battery Supply Panel?</t>
+  </si>
+  <si>
+    <t>What is the first step to appropriately de-energize / isolate the PowerTitan 2.0 system?</t>
+  </si>
+  <si>
+    <t>Open the MVT load switch</t>
+  </si>
+  <si>
+    <t>Use the LC to switch from Local/Remote mode to Local Mode</t>
+  </si>
+  <si>
+    <t>Open QF1 and QF2 in the SCC</t>
+  </si>
+  <si>
+    <t>Open QS1 and QS2 in the SCC</t>
+  </si>
+  <si>
+    <t>When testing for zero voltage on QF3/QF4 in the SCC, what is being confirmed?</t>
+  </si>
+  <si>
+    <t>There is no energy going into or out of the batteries</t>
+  </si>
+  <si>
+    <t>There is no power coming from the auxiliary power source</t>
+  </si>
+  <si>
+    <t>The AC capacitors are de-energized</t>
+  </si>
+  <si>
+    <t>There is no power coming from the MVT</t>
+  </si>
+  <si>
+    <t>QF3 and QF4 can be closed at the same time.</t>
+  </si>
+  <si>
+    <t>Which of the following can never be considered de-energized? </t>
+  </si>
+  <si>
+    <t>Batteries</t>
+  </si>
+  <si>
+    <t>Auxiliary transformer</t>
+  </si>
+  <si>
+    <t>DC capacitors</t>
+  </si>
+  <si>
+    <t>The Local controller</t>
+  </si>
+  <si>
     <t>Multi</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
+    <t>Which of the following are de-energization testing points in the integrated compartment of the battery container? Select all that apply.</t>
+  </si>
+  <si>
+    <t>QS1-QS6</t>
+  </si>
+  <si>
+    <t>QS11</t>
+  </si>
+  <si>
+    <t>Q1-Q8</t>
+  </si>
+  <si>
+    <t>QF1</t>
+  </si>
+  <si>
+    <t>A, D</t>
+  </si>
+  <si>
+    <t>The main AC breakers in the SCC can be remotely opened from the LC.</t>
+  </si>
+  <si>
+    <t>Before uninstalling the MSDs in a rack, which of the following connections should be removed?</t>
+  </si>
+  <si>
+    <t>Top DC+</t>
+  </si>
+  <si>
+    <t>Top DC-</t>
+  </si>
+  <si>
+    <t>Bottom DC+</t>
+  </si>
+  <si>
+    <t>Bottom DC-</t>
+  </si>
+  <si>
+    <t>Which of the following are LOTO points in the SCC? Select all that apply.</t>
+  </si>
+  <si>
+    <t>QF2</t>
+  </si>
+  <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>QF3/QF4</t>
+  </si>
+  <si>
+    <t>QF5</t>
+  </si>
+  <si>
+    <t>QS1 and/or QS2</t>
+  </si>
+  <si>
+    <t>A, B, C, D, E, F</t>
+  </si>
+  <si>
+    <t>How many total measurements with a multi-meter need to be taken to confirm zero AC voltage on the AC busbars coming out of QF1 and QF2 in the SCC?</t>
+  </si>
+  <si>
+    <t>The incident energy sticker dictates the calorie rating of the suit that must be worn in order to open that cabinet door.</t>
+  </si>
+  <si>
+    <t>Who should be notified when beginning LOTO on the ESS? Choose the best answer.</t>
+  </si>
+  <si>
+    <t>Sungrow Headquarters</t>
+  </si>
+  <si>
+    <t>The local fire department</t>
+  </si>
+  <si>
+    <t>All affected employees</t>
+  </si>
+  <si>
+    <t>Just your safety second</t>
+  </si>
+  <si>
+    <t>As long as I have properly isolated/de-energized the skid, I may replace a BMU board without insulating gloves.</t>
+  </si>
+  <si>
+    <t>What are the energy sources that need to be isolated during the de-energization process of the PowerTitan 2.0? Select all that apply.</t>
+  </si>
+  <si>
+    <t>Solar Power</t>
+  </si>
+  <si>
+    <t>Grid Power</t>
+  </si>
+  <si>
+    <t>External Auxiliary Power (if used)</t>
   </si>
   <si>
     <t>Wind Power</t>
   </si>
   <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>The site's LOTO procedure document</t>
-  </si>
-  <si>
-    <t>Best judgement</t>
-  </si>
-  <si>
-    <t>You can upgrade the firmware of every BSC connected to an LC through the LC web portal.</t>
-  </si>
-  <si>
-    <t>Sungrow's LOTO guidance document</t>
-  </si>
-  <si>
-    <t>PowerTitan 2.0 Power Cycle MOP</t>
-  </si>
-  <si>
-    <t>When turning off the system block from the LC, AC breakers QF1 and QF2 in the SCC open automatically.</t>
-  </si>
-  <si>
-    <t>What color LED indicator proves that the battery container is de-energized?</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>When the LED is off</t>
-  </si>
-  <si>
-    <t>The LED indicator doesn't prove de-energization</t>
-  </si>
-  <si>
-    <t>What is the voltage on the AC busbar between the main AC breakers in the SCC and the low voltage bushings of the Medium Voltage Transformer?</t>
-  </si>
-  <si>
-    <t>115V</t>
-  </si>
-  <si>
-    <t>230V</t>
-  </si>
-  <si>
-    <t>480V</t>
-  </si>
-  <si>
-    <t>690V</t>
-  </si>
-  <si>
-    <t>What is the AC voltage of the auxiliary power being fed into QF1 in the Battery Supply Panel?</t>
-  </si>
-  <si>
-    <t>What is the first step to appropriately de-energize / isolate the PowerTitan 2.0 system?</t>
-  </si>
-  <si>
-    <t>Open the MVT load switch</t>
-  </si>
-  <si>
-    <t>Use the LC to switch from Local/Remote mode to Local Mode</t>
-  </si>
-  <si>
-    <t>Open QF1 and QF2 in the SCC</t>
-  </si>
-  <si>
-    <t>Open QS1 and QS2 in the SCC</t>
-  </si>
-  <si>
-    <t>When testing for zero voltage on QF3/QF4 in the SCC, what is being confirmed?</t>
-  </si>
-  <si>
-    <t>There is no energy going into or out of the batteries</t>
-  </si>
-  <si>
-    <t>There is no power coming from the auxiliary power source</t>
-  </si>
-  <si>
-    <t>The AC capacitors are de-energized</t>
-  </si>
-  <si>
-    <t>There is no power coming from the MVT</t>
-  </si>
-  <si>
-    <t>QF3 and QF4 can be closed at the same time.</t>
-  </si>
-  <si>
-    <t>Which of the following can never be considered de-energized? </t>
-  </si>
-  <si>
-    <t>Batteries</t>
-  </si>
-  <si>
-    <t>Auxiliary transformer</t>
-  </si>
-  <si>
-    <t>DC capacitors</t>
-  </si>
-  <si>
-    <t>The Local controller</t>
-  </si>
-  <si>
-    <t>Which of the following are de-energization testing points in the integrated compartment of the battery container? Select all that apply.</t>
-  </si>
-  <si>
-    <t>QS1-QS6</t>
-  </si>
-  <si>
-    <t>QS11</t>
-  </si>
-  <si>
-    <t>Q1-Q8</t>
-  </si>
-  <si>
-    <t>QF1</t>
-  </si>
-  <si>
-    <t>The main AC breakers in the SCC can be remotely opened from the LC.</t>
-  </si>
-  <si>
-    <t>Before uninstalling the MSDs in a rack, which of the following connections should be removed?</t>
-  </si>
-  <si>
-    <t>Top DC+</t>
-  </si>
-  <si>
-    <t>Top DC-</t>
-  </si>
-  <si>
-    <t>Bottom DC+</t>
-  </si>
-  <si>
-    <t>Bottom DC-</t>
-  </si>
-  <si>
-    <t>Which of the following are LOTO points in the SCC? Select all that apply.</t>
-  </si>
-  <si>
-    <t>QF2</t>
-  </si>
-  <si>
-    <t>UPS</t>
-  </si>
-  <si>
-    <t>QF3/QF4</t>
-  </si>
-  <si>
-    <t>QF5</t>
-  </si>
-  <si>
-    <t>QS1 and/or QS2</t>
-  </si>
-  <si>
-    <t>How many total measurements with a multi-meter need to be taken to confirm zero AC voltage on the AC busbars coming out of QF1 and QF2 in the SCC?</t>
-  </si>
-  <si>
-    <t>The incident energy sticker dictates the calorie rating of the suit that must be worn in order to open that cabinet door.</t>
-  </si>
-  <si>
-    <t>Who should be notified when beginning LOTO on the ESS? Choose the best answer.</t>
-  </si>
-  <si>
-    <t>Sungrow Headquarters</t>
-  </si>
-  <si>
-    <t>The local fire department</t>
-  </si>
-  <si>
-    <t>All affected employees</t>
-  </si>
-  <si>
-    <t>Just your safety second</t>
-  </si>
-  <si>
-    <t>As long as I have properly isolated/de-energized the skid, I may replace a BMU board without insulating gloves.</t>
-  </si>
-  <si>
-    <t>What are the energy sources that need to be isolated during the de-energization process of the PowerTitan 2.0? Select all that apply.</t>
-  </si>
-  <si>
-    <t>Solar Power</t>
-  </si>
-  <si>
-    <t>Grid Power</t>
-  </si>
-  <si>
-    <t>External Auxiliary Power (if used)</t>
+    <t>B, C, D</t>
   </si>
   <si>
     <t>If the PowerTitan 2.0 system has been properly de-energized / isolated, I still need gloves to replace a BMU.</t>
@@ -296,6 +308,9 @@
     <t>Proving unit</t>
   </si>
   <si>
+    <t>A, B, D</t>
+  </si>
+  <si>
     <t>What MSDs need to be removed if I am replacing pack #2 of rack #1?</t>
   </si>
   <si>
@@ -327,21 +342,6 @@
   </si>
   <si>
     <t>FRC</t>
-  </si>
-  <si>
-    <t>A, D</t>
-  </si>
-  <si>
-    <t>A, B, C, D, E, F</t>
-  </si>
-  <si>
-    <t>B, C, D</t>
-  </si>
-  <si>
-    <t>A, B, D</t>
-  </si>
-  <si>
-    <t>G</t>
   </si>
   <si>
     <t>What Multimeter testing mode is needed when testing the busbars above QF1 and QF2 in the MVS?</t>
@@ -538,15 +538,17 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
-      <color rgb="FF1B1C1D"/>
-      <name val="Arial"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -562,18 +564,16 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF1B1C1D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -599,10 +599,10 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,39 +631,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -715,7 +715,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -826,6 +826,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -834,13 +841,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -905,154 +905,125 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8BC162-2202-0049-81DD-82F1455E7C57}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FDD113C-2248-8C4A-9AEA-78392E6FAF4A}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="129.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="42" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2">
+      <c r="J2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D3" s="3" t="b">
+      <c r="D3" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="J3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" s="2">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="J3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="J4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K4">
         <v>5</v>
@@ -1060,25 +1031,25 @@
     </row>
     <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="J5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>5</v>
@@ -1086,25 +1057,25 @@
     </row>
     <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" t="s">
         <v>4</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J6" t="s">
-        <v>8</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -1112,25 +1083,25 @@
     </row>
     <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="J7" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K7">
         <v>5</v>
@@ -1138,25 +1109,25 @@
     </row>
     <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>39</v>
-      </c>
       <c r="J8" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -1164,21 +1135,21 @@
     </row>
     <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D9" s="3" t="b">
+      <c r="D9" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
       <c r="J9" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -1186,25 +1157,25 @@
     </row>
     <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="J10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K10">
         <v>5</v>
@@ -1212,26 +1183,26 @@
     </row>
     <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" s="2"/>
       <c r="J11" t="s">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="K11">
         <v>5</v>
@@ -1239,24 +1210,24 @@
     </row>
     <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D12" s="3" t="b">
+      <c r="D12" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
       <c r="J12" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K12">
         <v>5</v>
@@ -1264,28 +1235,28 @@
     </row>
     <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K13">
         <v>5</v>
@@ -1293,32 +1264,32 @@
     </row>
     <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="3"/>
       <c r="J14" t="s">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="K14">
         <v>5</v>
@@ -1326,12 +1297,12 @@
     </row>
     <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="3">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="2">
         <v>3</v>
       </c>
       <c r="D15">
@@ -1343,10 +1314,10 @@
       <c r="F15">
         <v>12</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
       <c r="J15" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K15">
         <v>5</v>
@@ -1354,21 +1325,21 @@
     </row>
     <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D16" s="3" t="b">
+      <c r="D16" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
       <c r="J16" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K16">
         <v>5</v>
@@ -1376,27 +1347,27 @@
     </row>
     <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" t="s">
         <v>4</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" t="s">
-        <v>8</v>
       </c>
       <c r="K17">
         <v>5</v>
@@ -1404,19 +1375,19 @@
     </row>
     <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="b">
         <v>1</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
       </c>
       <c r="J18" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K18">
         <v>5</v>
@@ -1424,28 +1395,28 @@
     </row>
     <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>71</v>
+        <v>45</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>99</v>
+      <c r="D19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="K19">
         <v>5</v>
@@ -1453,19 +1424,19 @@
     </row>
     <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="3" t="b">
+        <v>11</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="2" t="b">
         <v>1</v>
       </c>
       <c r="D20" t="b">
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K20">
         <v>5</v>
@@ -1473,25 +1444,25 @@
     </row>
     <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>80</v>
       </c>
+      <c r="C21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="J21" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K21">
         <v>5</v>
@@ -1499,25 +1470,25 @@
     </row>
     <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F22" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>85</v>
       </c>
+      <c r="C22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J22" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="K22">
         <v>5</v>
@@ -1525,25 +1496,25 @@
     </row>
     <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J23" t="s">
         <v>4</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J23" t="s">
-        <v>8</v>
       </c>
       <c r="K23">
         <v>5</v>
@@ -1551,28 +1522,28 @@
     </row>
     <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="G24" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="J24" s="3" t="s">
-        <v>6</v>
+      <c r="C24" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="K24">
         <v>5</v>
@@ -1580,25 +1551,25 @@
     </row>
     <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>80</v>
+      <c r="C25" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="J25" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K25">
         <v>5</v>
@@ -1606,25 +1577,25 @@
     </row>
     <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>80</v>
+      <c r="C26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="J26" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K26">
         <v>5</v>
@@ -1632,25 +1603,25 @@
     </row>
     <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J27" t="s">
         <v>4</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="J27" t="s">
-        <v>8</v>
       </c>
       <c r="K27">
         <v>5</v>
@@ -1658,9 +1629,9 @@
     </row>
     <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C28" t="b">
@@ -1670,7 +1641,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K28">
         <v>5</v>
@@ -1678,25 +1649,25 @@
     </row>
     <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="3" t="s">
+      <c r="E29" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>113</v>
       </c>
       <c r="J29" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K29">
         <v>5</v>
@@ -1704,9 +1675,9 @@
     </row>
     <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B30" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>114</v>
       </c>
       <c r="C30">
@@ -1722,7 +1693,7 @@
         <v>60</v>
       </c>
       <c r="J30" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -1730,19 +1701,19 @@
     </row>
     <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B31" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C31" s="3" t="b">
+      <c r="C31" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D31" s="3" t="b">
+      <c r="D31" s="2" t="b">
         <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K31">
         <v>5</v>
@@ -1750,9 +1721,9 @@
     </row>
     <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>116</v>
       </c>
       <c r="C32" t="s">
@@ -1768,7 +1739,7 @@
         <v>120</v>
       </c>
       <c r="J32" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K32">
         <v>5</v>
@@ -1776,9 +1747,9 @@
     </row>
     <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B33" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C33" t="b">
@@ -1788,7 +1759,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K33">
         <v>5</v>
@@ -1796,9 +1767,9 @@
     </row>
     <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>122</v>
       </c>
       <c r="C34" t="s">
@@ -1814,7 +1785,7 @@
         <v>126</v>
       </c>
       <c r="J34" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K34">
         <v>5</v>
@@ -1822,9 +1793,9 @@
     </row>
     <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>127</v>
       </c>
       <c r="C35" t="s">
@@ -1840,7 +1811,7 @@
         <v>131</v>
       </c>
       <c r="J35" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K35">
         <v>5</v>
@@ -1848,9 +1819,9 @@
     </row>
     <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>132</v>
       </c>
       <c r="C36" t="s">
@@ -1866,7 +1837,7 @@
         <v>136</v>
       </c>
       <c r="J36" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K36">
         <v>5</v>
@@ -1874,9 +1845,9 @@
     </row>
     <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C37" t="b">
@@ -1886,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K37">
         <v>5</v>
@@ -1894,9 +1865,9 @@
     </row>
     <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>138</v>
       </c>
       <c r="C38" t="s">
@@ -1912,7 +1883,7 @@
         <v>113</v>
       </c>
       <c r="J38" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K38">
         <v>5</v>
@@ -1920,9 +1891,9 @@
     </row>
     <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>142</v>
       </c>
       <c r="C39" t="s">
@@ -1938,7 +1909,7 @@
         <v>120</v>
       </c>
       <c r="J39" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K39">
         <v>5</v>
@@ -1946,9 +1917,9 @@
     </row>
     <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B40" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>143</v>
       </c>
       <c r="C40" t="s">
@@ -1964,7 +1935,7 @@
         <v>120</v>
       </c>
       <c r="J40" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K40">
         <v>5</v>
@@ -1972,9 +1943,9 @@
     </row>
     <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>144</v>
       </c>
       <c r="C41" t="b">
@@ -1984,7 +1955,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K41">
         <v>5</v>
@@ -1992,9 +1963,9 @@
     </row>
     <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B42" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>145</v>
       </c>
       <c r="C42" t="b">
@@ -2004,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K42">
         <v>5</v>
@@ -2012,9 +1983,9 @@
     </row>
     <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B43" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>146</v>
       </c>
       <c r="C43" t="b">
@@ -2024,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K43">
         <v>5</v>
@@ -2032,9 +2003,9 @@
     </row>
     <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B44" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>147</v>
       </c>
       <c r="C44" t="b">
@@ -2044,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K44">
         <v>5</v>
@@ -2052,9 +2023,9 @@
     </row>
     <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B45" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>148</v>
       </c>
       <c r="C45" t="s">
@@ -2070,7 +2041,7 @@
         <v>113</v>
       </c>
       <c r="J45" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K45">
         <v>5</v>
@@ -2078,9 +2049,9 @@
     </row>
     <row r="46" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>152</v>
       </c>
       <c r="C46" t="b">
@@ -2090,7 +2061,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K46">
         <v>5</v>
@@ -2098,9 +2069,9 @@
     </row>
     <row r="47" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B47" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>153</v>
       </c>
       <c r="C47" t="b">
@@ -2110,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K47">
         <v>5</v>
@@ -2118,9 +2089,9 @@
     </row>
     <row r="48" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B48" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>154</v>
       </c>
       <c r="C48" t="s">
@@ -2144,9 +2115,9 @@
     </row>
     <row r="49" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B49" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>160</v>
       </c>
       <c r="C49" t="s">
@@ -2156,7 +2127,7 @@
         <v>162</v>
       </c>
       <c r="J49" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K49">
         <v>5</v>
@@ -2164,9 +2135,9 @@
     </row>
     <row r="50" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B50" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>163</v>
       </c>
       <c r="C50" t="b">
@@ -2176,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K50">
         <v>5</v>

</xml_diff>

<commit_message>
Update question pool for SG3150U-MV
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG3150/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29CDC5C-BA5C-8F44-8EDA-50BA64DD0CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B27BC715-EFCC-6D47-A20B-CCF662CFA7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{C1094EB1-E11C-4826-97C7-12D07005C403}"/>
   </bookViews>
@@ -1513,7 +1513,7 @@
         <v>2</v>
       </c>
       <c r="J2" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1539,7 +1539,7 @@
         <v>5</v>
       </c>
       <c r="J3" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1565,7 +1565,7 @@
         <v>4</v>
       </c>
       <c r="J4" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1591,7 +1591,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1617,7 +1617,7 @@
         <v>5</v>
       </c>
       <c r="J6" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.25">
@@ -1643,7 +1643,7 @@
         <v>4</v>
       </c>
       <c r="J7" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.25">
@@ -1669,7 +1669,7 @@
         <v>3</v>
       </c>
       <c r="J8" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1695,7 +1695,7 @@
         <v>5</v>
       </c>
       <c r="J9" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1721,7 +1721,7 @@
         <v>4</v>
       </c>
       <c r="J10" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1747,7 +1747,7 @@
         <v>5</v>
       </c>
       <c r="J11" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1773,7 +1773,7 @@
         <v>3</v>
       </c>
       <c r="J12" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1799,7 +1799,7 @@
         <v>2</v>
       </c>
       <c r="J13" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1825,7 +1825,7 @@
         <v>4</v>
       </c>
       <c r="J14" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1851,7 +1851,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1877,7 +1877,7 @@
         <v>4</v>
       </c>
       <c r="J16" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1903,7 +1903,7 @@
         <v>3</v>
       </c>
       <c r="J17" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1929,7 +1929,7 @@
         <v>3</v>
       </c>
       <c r="J18" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1955,7 +1955,7 @@
         <v>5</v>
       </c>
       <c r="J19" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -1981,7 +1981,7 @@
         <v>4</v>
       </c>
       <c r="J20" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2003,7 +2003,7 @@
         <v>3</v>
       </c>
       <c r="J21" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2023,7 +2023,7 @@
         <v>2</v>
       </c>
       <c r="J22" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2043,7 +2043,7 @@
         <v>3</v>
       </c>
       <c r="J23" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2063,7 +2063,7 @@
         <v>3</v>
       </c>
       <c r="J24" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2083,7 +2083,7 @@
         <v>3</v>
       </c>
       <c r="J25" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2103,7 +2103,7 @@
         <v>3</v>
       </c>
       <c r="J26" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2123,7 +2123,7 @@
         <v>3</v>
       </c>
       <c r="J27" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2145,7 +2145,7 @@
         <v>2</v>
       </c>
       <c r="J28" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2165,7 +2165,7 @@
         <v>2</v>
       </c>
       <c r="J29" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2185,7 +2185,7 @@
         <v>3</v>
       </c>
       <c r="J30" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2205,7 +2205,7 @@
         <v>3</v>
       </c>
       <c r="J31" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2225,7 +2225,7 @@
         <v>2</v>
       </c>
       <c r="J32" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.25">
@@ -2251,7 +2251,7 @@
         <v>2</v>
       </c>
       <c r="J33" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2332,7 +2332,7 @@
         <v>134</v>
       </c>
       <c r="J36" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
@@ -2384,7 +2384,7 @@
         <v>146</v>
       </c>
       <c r="J38" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
change the multiple question answer bank structure and added a success pageat the end
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG3600_safety/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CA70879-DCA9-D44C-A72A-8CFA0B970C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6C2595-EA5C-B94C-8D23-DB186A33ED42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19880" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="205">
   <si>
     <t>Type</t>
   </si>
@@ -522,9 +522,6 @@
     <t>AC SPD circuit, before the fuses. Either in Aux cabinet or in Unit 1</t>
   </si>
   <si>
-    <t>ABC</t>
-  </si>
-  <si>
     <t>Which protections are available in the SG3600 unit?</t>
   </si>
   <si>
@@ -561,9 +558,6 @@
     <t xml:space="preserve"> QS4</t>
   </si>
   <si>
-    <t>A,C</t>
-  </si>
-  <si>
     <t>Which of the following are considered LOTO points when performing maintenance on a PV system with an inverter?</t>
   </si>
   <si>
@@ -601,9 +595,6 @@
   </si>
   <si>
     <t>QS4</t>
-  </si>
-  <si>
-    <t>AC</t>
   </si>
   <si>
     <r>
@@ -629,12 +620,6 @@
     <t>Multimeter</t>
   </si>
   <si>
-    <t xml:space="preserve">A,B,C </t>
-  </si>
-  <si>
-    <t>What is the replationship between resistance of NTC sensor and temperature?</t>
-  </si>
-  <si>
     <t>Proportional</t>
   </si>
   <si>
@@ -659,9 +644,6 @@
     <t>Battery Power</t>
   </si>
   <si>
-    <t>ABCD</t>
-  </si>
-  <si>
     <t xml:space="preserve">As temperature increases, the capacity rating of an inverter usually decreases. </t>
   </si>
   <si>
@@ -726,6 +708,21 @@
   </si>
   <si>
     <t>Open circuit voltage of the PV module is directly proportional to temperature</t>
+  </si>
+  <si>
+    <t>A, B, C</t>
+  </si>
+  <si>
+    <t>A, C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A, B, C </t>
+  </si>
+  <si>
+    <t>A, B, C, D</t>
+  </si>
+  <si>
+    <t>What is the relationship between resistance of NTC sensor and temperature?</t>
   </si>
 </sst>
 </file>
@@ -816,9 +813,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -856,7 +853,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -962,7 +959,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1104,7 +1101,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2023,7 +2020,7 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1" t="s">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="K31" s="1">
         <v>5</v>
@@ -2034,27 +2031,27 @@
         <v>135</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K32" s="1">
         <v>10</v>
@@ -2065,25 +2062,25 @@
         <v>135</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>154</v>
+        <v>201</v>
       </c>
       <c r="K33" s="1">
         <v>5</v>
@@ -2094,29 +2091,29 @@
         <v>135</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="I34" s="1"/>
       <c r="J34" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="K34" s="1">
         <v>10</v>
@@ -2127,25 +2124,25 @@
         <v>135</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>168</v>
+        <v>201</v>
       </c>
       <c r="K35" s="1">
         <v>5</v>
@@ -2156,23 +2153,23 @@
         <v>135</v>
       </c>
       <c r="B36" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="K36" s="1">
         <v>5</v>
@@ -2180,25 +2177,27 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
+      <c r="J37" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="K37" s="1">
         <v>5</v>
       </c>
@@ -2208,25 +2207,25 @@
         <v>135</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="K38" s="1">
         <v>5</v>
@@ -2237,7 +2236,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C39" s="1" t="b">
         <v>1</v>
@@ -2262,7 +2261,7 @@
         <v>10</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C40" s="1" t="b">
         <v>1</v>
@@ -2287,7 +2286,7 @@
         <v>10</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C41" s="1" t="b">
         <v>1</v>
@@ -2312,7 +2311,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C42" s="1" t="b">
         <v>1</v>
@@ -2337,7 +2336,7 @@
         <v>10</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C43" s="1" t="b">
         <v>1</v>
@@ -2362,7 +2361,7 @@
         <v>10</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C44" s="1" t="b">
         <v>1</v>
@@ -2387,7 +2386,7 @@
         <v>10</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C45" s="1" t="b">
         <v>1</v>
@@ -2412,7 +2411,7 @@
         <v>10</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C46" s="1" t="b">
         <v>1</v>
@@ -2437,7 +2436,7 @@
         <v>10</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C47" s="1" t="b">
         <v>1</v>
@@ -2462,7 +2461,7 @@
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C48" s="1" t="b">
         <v>1</v>
@@ -2487,7 +2486,7 @@
         <v>10</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C49" s="1" t="b">
         <v>1</v>
@@ -2512,7 +2511,7 @@
         <v>10</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C50" s="1" t="b">
         <v>1</v>
@@ -2537,7 +2536,7 @@
         <v>10</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C51" s="1" t="b">
         <v>1</v>
@@ -2562,7 +2561,7 @@
         <v>10</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C52" s="1" t="b">
         <v>1</v>
@@ -2587,7 +2586,7 @@
         <v>10</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C53" s="1" t="b">
         <v>1</v>
@@ -2612,7 +2611,7 @@
         <v>10</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C54" s="1" t="b">
         <v>1</v>
@@ -2637,7 +2636,7 @@
         <v>10</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C55" s="1" t="b">
         <v>1</v>
@@ -2662,7 +2661,7 @@
         <v>10</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C56" s="1" t="b">
         <v>1</v>
@@ -2687,7 +2686,7 @@
         <v>10</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C57" s="1" t="b">
         <v>1</v>
@@ -2707,7 +2706,7 @@
         <v>10</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C58" s="1" t="b">
         <v>1</v>
@@ -2727,7 +2726,7 @@
         <v>10</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C59" s="1" t="b">
         <v>1</v>
@@ -2747,7 +2746,7 @@
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C60" s="1" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
fix the indentation error for the last finishing page
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6C2595-EA5C-B94C-8D23-DB186A33ED42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C98718F-B527-6B40-B63C-1DAD76B17D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19880" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
   </bookViews>
@@ -1119,8 +1119,8 @@
     <col min="5" max="5" width="29.83203125" customWidth="1"/>
     <col min="6" max="6" width="19.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
-    <col min="8" max="8" width="2.5" customWidth="1"/>
-    <col min="9" max="9" width="14.5" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" customWidth="1"/>
     <col min="10" max="10" width="14.5" customWidth="1"/>
     <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
update the question pool data structure
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C98718F-B527-6B40-B63C-1DAD76B17D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0818F493-BFA2-D544-86AE-DE6B5EC33820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19880" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
   </bookViews>
@@ -1120,7 +1120,7 @@
     <col min="6" max="6" width="19.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="20.6640625" customWidth="1"/>
-    <col min="9" max="9" width="21.33203125" customWidth="1"/>
+    <col min="9" max="9" width="62.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.5" customWidth="1"/>
     <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Update the script to revise the mapping back answer data structure and the submission finish page
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG3600_safety/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CA70879-DCA9-D44C-A72A-8CFA0B970C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B8CEAF-59D5-F044-BE0A-586FB990249E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="205">
   <si>
     <t>Type</t>
   </si>
@@ -522,9 +522,6 @@
     <t>AC SPD circuit, before the fuses. Either in Aux cabinet or in Unit 1</t>
   </si>
   <si>
-    <t>ABC</t>
-  </si>
-  <si>
     <t>Which protections are available in the SG3600 unit?</t>
   </si>
   <si>
@@ -561,9 +558,6 @@
     <t xml:space="preserve"> QS4</t>
   </si>
   <si>
-    <t>A,C</t>
-  </si>
-  <si>
     <t>Which of the following are considered LOTO points when performing maintenance on a PV system with an inverter?</t>
   </si>
   <si>
@@ -601,9 +595,6 @@
   </si>
   <si>
     <t>QS4</t>
-  </si>
-  <si>
-    <t>AC</t>
   </si>
   <si>
     <r>
@@ -629,9 +620,6 @@
     <t>Multimeter</t>
   </si>
   <si>
-    <t xml:space="preserve">A,B,C </t>
-  </si>
-  <si>
     <t>What is the replationship between resistance of NTC sensor and temperature?</t>
   </si>
   <si>
@@ -659,9 +647,6 @@
     <t>Battery Power</t>
   </si>
   <si>
-    <t>ABCD</t>
-  </si>
-  <si>
     <t xml:space="preserve">As temperature increases, the capacity rating of an inverter usually decreases. </t>
   </si>
   <si>
@@ -726,6 +711,18 @@
   </si>
   <si>
     <t>Open circuit voltage of the PV module is directly proportional to temperature</t>
+  </si>
+  <si>
+    <t>A, B, C</t>
+  </si>
+  <si>
+    <t>A, C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A, B, C </t>
+  </si>
+  <si>
+    <t>A, B, C, D</t>
   </si>
 </sst>
 </file>
@@ -816,9 +813,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -856,7 +853,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -962,7 +959,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1104,7 +1101,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2023,7 +2020,7 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1" t="s">
-        <v>141</v>
+        <v>201</v>
       </c>
       <c r="K31" s="1">
         <v>5</v>
@@ -2034,27 +2031,27 @@
         <v>135</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K32" s="1">
         <v>10</v>
@@ -2065,25 +2062,25 @@
         <v>135</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="K33" s="1">
         <v>5</v>
@@ -2094,29 +2091,29 @@
         <v>135</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="I34" s="1"/>
       <c r="J34" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="K34" s="1">
         <v>10</v>
@@ -2127,25 +2124,25 @@
         <v>135</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>168</v>
+        <v>202</v>
       </c>
       <c r="K35" s="1">
         <v>5</v>
@@ -2156,23 +2153,23 @@
         <v>135</v>
       </c>
       <c r="B36" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="K36" s="1">
         <v>5</v>
@@ -2180,25 +2177,27 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
+      <c r="J37" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="K37" s="1">
         <v>5</v>
       </c>
@@ -2208,25 +2207,25 @@
         <v>135</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>182</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="K38" s="1">
         <v>5</v>
@@ -2237,7 +2236,7 @@
         <v>10</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C39" s="1" t="b">
         <v>1</v>
@@ -2262,7 +2261,7 @@
         <v>10</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C40" s="1" t="b">
         <v>1</v>
@@ -2287,7 +2286,7 @@
         <v>10</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C41" s="1" t="b">
         <v>1</v>
@@ -2312,7 +2311,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C42" s="1" t="b">
         <v>1</v>
@@ -2337,7 +2336,7 @@
         <v>10</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C43" s="1" t="b">
         <v>1</v>
@@ -2362,7 +2361,7 @@
         <v>10</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C44" s="1" t="b">
         <v>1</v>
@@ -2387,7 +2386,7 @@
         <v>10</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C45" s="1" t="b">
         <v>1</v>
@@ -2412,7 +2411,7 @@
         <v>10</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C46" s="1" t="b">
         <v>1</v>
@@ -2437,7 +2436,7 @@
         <v>10</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C47" s="1" t="b">
         <v>1</v>
@@ -2462,7 +2461,7 @@
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C48" s="1" t="b">
         <v>1</v>
@@ -2487,7 +2486,7 @@
         <v>10</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C49" s="1" t="b">
         <v>1</v>
@@ -2512,7 +2511,7 @@
         <v>10</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C50" s="1" t="b">
         <v>1</v>
@@ -2537,7 +2536,7 @@
         <v>10</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C51" s="1" t="b">
         <v>1</v>
@@ -2562,7 +2561,7 @@
         <v>10</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C52" s="1" t="b">
         <v>1</v>
@@ -2587,7 +2586,7 @@
         <v>10</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C53" s="1" t="b">
         <v>1</v>
@@ -2612,7 +2611,7 @@
         <v>10</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C54" s="1" t="b">
         <v>1</v>
@@ -2637,7 +2636,7 @@
         <v>10</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C55" s="1" t="b">
         <v>1</v>
@@ -2662,7 +2661,7 @@
         <v>10</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C56" s="1" t="b">
         <v>1</v>
@@ -2687,7 +2686,7 @@
         <v>10</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C57" s="1" t="b">
         <v>1</v>
@@ -2707,7 +2706,7 @@
         <v>10</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C58" s="1" t="b">
         <v>1</v>
@@ -2727,7 +2726,7 @@
         <v>10</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C59" s="1" t="b">
         <v>1</v>
@@ -2747,7 +2746,7 @@
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C60" s="1" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
change the multiple question answer bank structure and added a success page at the end of submission
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F911A6-B4F6-8642-B53B-50CABDCC397A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6520E602-7817-3E42-832D-30A473F46B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -245,9 +245,6 @@
     <t>Door Switch</t>
   </si>
   <si>
-    <t>A,B,D,E,F</t>
-  </si>
-  <si>
     <t>Which of the following are functions of the LC300?</t>
   </si>
   <si>
@@ -266,9 +263,6 @@
     <t>SOC Protection Parameter modification</t>
   </si>
   <si>
-    <t>A,B,E</t>
-  </si>
-  <si>
     <t>If the coolant pH falls below 7.3, it is required to replace the coolant</t>
   </si>
   <si>
@@ -495,6 +489,12 @@
   </si>
   <si>
     <t>List the following components in order of communicates. Start with the smallest level of communication: LC, BMU, BSC, CMU, SCADA</t>
+  </si>
+  <si>
+    <t>A, B, D, E, F</t>
+  </si>
+  <si>
+    <t>A, B, E</t>
   </si>
 </sst>
 </file>
@@ -922,6 +922,7 @@
     <col min="5" max="5" width="67.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="126" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="34.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -1245,7 +1246,7 @@
         <v>68</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>151</v>
       </c>
       <c r="K12">
         <v>5</v>
@@ -1256,27 +1257,27 @@
         <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>75</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" t="s">
-        <v>76</v>
+        <v>152</v>
       </c>
       <c r="K13">
         <v>5</v>
@@ -1287,7 +1288,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -1331,7 +1332,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C16" s="3" t="b">
         <v>1</v>
@@ -1353,7 +1354,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1392,10 +1393,10 @@
     </row>
     <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K19">
         <v>20</v>
@@ -1406,19 +1407,19 @@
         <v>11</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" t="s">
         <v>82</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
         <v>83</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
         <v>84</v>
-      </c>
-      <c r="E20" t="s">
-        <v>85</v>
-      </c>
-      <c r="F20" t="s">
-        <v>86</v>
       </c>
       <c r="J20" t="s">
         <v>3</v>
@@ -1432,7 +1433,7 @@
         <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1455,22 +1456,22 @@
     </row>
     <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" t="s">
         <v>88</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" t="s">
-        <v>90</v>
       </c>
       <c r="D22" t="s">
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J22" t="s">
         <v>5</v>
@@ -1484,19 +1485,19 @@
         <v>11</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" t="s">
         <v>93</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>94</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>95</v>
-      </c>
-      <c r="E23" t="s">
-        <v>96</v>
-      </c>
-      <c r="F23" t="s">
-        <v>97</v>
       </c>
       <c r="J23" t="s">
         <v>3</v>
@@ -1510,19 +1511,19 @@
         <v>11</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" t="s">
         <v>94</v>
       </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
         <v>95</v>
-      </c>
-      <c r="E24" t="s">
-        <v>96</v>
-      </c>
-      <c r="F24" t="s">
-        <v>97</v>
       </c>
       <c r="J24" t="s">
         <v>2</v>
@@ -1536,19 +1537,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C25" t="s">
+        <v>92</v>
+      </c>
+      <c r="D25" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25" t="s">
         <v>94</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
         <v>95</v>
-      </c>
-      <c r="E25" t="s">
-        <v>96</v>
-      </c>
-      <c r="F25" t="s">
-        <v>97</v>
       </c>
       <c r="J25" t="s">
         <v>3</v>
@@ -1562,19 +1563,19 @@
         <v>11</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26" t="s">
         <v>94</v>
       </c>
-      <c r="D26" t="s">
+      <c r="F26" t="s">
         <v>95</v>
-      </c>
-      <c r="E26" t="s">
-        <v>96</v>
-      </c>
-      <c r="F26" t="s">
-        <v>97</v>
       </c>
       <c r="J26" t="s">
         <v>5</v>
@@ -1588,19 +1589,19 @@
         <v>11</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" t="s">
         <v>101</v>
-      </c>
-      <c r="C27" t="s">
-        <v>102</v>
-      </c>
-      <c r="D27" t="s">
-        <v>103</v>
       </c>
       <c r="E27" t="s">
         <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J27" t="s">
         <v>3</v>
@@ -1614,19 +1615,19 @@
         <v>11</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" t="s">
         <v>105</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E28" t="s">
         <v>106</v>
       </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
         <v>107</v>
-      </c>
-      <c r="E28" t="s">
-        <v>108</v>
-      </c>
-      <c r="F28" t="s">
-        <v>109</v>
       </c>
       <c r="J28" t="s">
         <v>4</v>
@@ -1640,13 +1641,13 @@
         <v>11</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
+        <v>109</v>
+      </c>
+      <c r="D29" t="s">
         <v>110</v>
-      </c>
-      <c r="C29" t="s">
-        <v>111</v>
-      </c>
-      <c r="D29" t="s">
-        <v>112</v>
       </c>
       <c r="J29" t="s">
         <v>2</v>
@@ -1660,7 +1661,7 @@
         <v>11</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1686,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C31">
         <v>6</v>
@@ -1712,7 +1713,7 @@
         <v>11</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1738,7 +1739,7 @@
         <v>11</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1758,19 +1759,19 @@
         <v>11</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C34" t="s">
+        <v>116</v>
+      </c>
+      <c r="D34" t="s">
         <v>117</v>
       </c>
-      <c r="C34" t="s">
+      <c r="E34" t="s">
         <v>118</v>
       </c>
-      <c r="D34" t="s">
+      <c r="F34" t="s">
         <v>119</v>
-      </c>
-      <c r="E34" t="s">
-        <v>120</v>
-      </c>
-      <c r="F34" t="s">
-        <v>121</v>
       </c>
       <c r="J34" t="s">
         <v>3</v>
@@ -1784,19 +1785,19 @@
         <v>11</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C35" t="s">
+        <v>121</v>
+      </c>
+      <c r="D35" t="s">
         <v>122</v>
-      </c>
-      <c r="C35" t="s">
-        <v>123</v>
-      </c>
-      <c r="D35" t="s">
-        <v>124</v>
       </c>
       <c r="E35" t="s">
         <v>19</v>
       </c>
       <c r="F35" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J35" t="s">
         <v>4</v>
@@ -1810,19 +1811,19 @@
         <v>11</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C36" t="s">
+        <v>125</v>
+      </c>
+      <c r="D36" t="s">
         <v>126</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" t="s">
         <v>127</v>
       </c>
-      <c r="D36" t="s">
+      <c r="F36" t="s">
         <v>128</v>
-      </c>
-      <c r="E36" t="s">
-        <v>129</v>
-      </c>
-      <c r="F36" t="s">
-        <v>130</v>
       </c>
       <c r="J36" t="s">
         <v>3</v>
@@ -1836,7 +1837,7 @@
         <v>11</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C37">
         <v>3</v>
@@ -1862,7 +1863,7 @@
         <v>11</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C38">
         <v>12</v>
@@ -1888,19 +1889,19 @@
         <v>11</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" t="s">
+        <v>132</v>
+      </c>
+      <c r="D39" t="s">
         <v>133</v>
       </c>
-      <c r="C39" t="s">
+      <c r="E39" t="s">
         <v>134</v>
       </c>
-      <c r="D39" t="s">
+      <c r="F39" t="s">
         <v>135</v>
-      </c>
-      <c r="E39" t="s">
-        <v>136</v>
-      </c>
-      <c r="F39" t="s">
-        <v>137</v>
       </c>
       <c r="J39" t="s">
         <v>5</v>
@@ -1914,19 +1915,19 @@
         <v>11</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C40" t="s">
+        <v>137</v>
+      </c>
+      <c r="D40" t="s">
         <v>138</v>
       </c>
-      <c r="C40" t="s">
+      <c r="E40" t="s">
         <v>139</v>
       </c>
-      <c r="D40" t="s">
+      <c r="F40" t="s">
         <v>140</v>
-      </c>
-      <c r="E40" t="s">
-        <v>141</v>
-      </c>
-      <c r="F40" t="s">
-        <v>142</v>
       </c>
       <c r="J40" t="s">
         <v>4</v>
@@ -1940,19 +1941,19 @@
         <v>11</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D41" t="s">
         <v>143</v>
       </c>
-      <c r="C41" t="s">
+      <c r="E41" t="s">
         <v>144</v>
       </c>
-      <c r="D41" t="s">
+      <c r="F41" t="s">
         <v>145</v>
-      </c>
-      <c r="E41" t="s">
-        <v>146</v>
-      </c>
-      <c r="F41" t="s">
-        <v>147</v>
       </c>
       <c r="J41" t="s">
         <v>4</v>
@@ -1966,7 +1967,7 @@
         <v>11</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C42" t="b">
         <v>1</v>
@@ -1986,10 +1987,10 @@
         <v>11</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C43" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D43" t="s">
         <v>13</v>
@@ -2009,10 +2010,10 @@
     </row>
     <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="K44">
         <v>20</v>
@@ -2020,10 +2021,10 @@
     </row>
     <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K45">
         <v>20</v>

</xml_diff>

<commit_message>
Update SG350HX-US question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG350/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D11477-640C-A14A-AC9C-52E83736DBE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14AC34C-8EA8-FE48-A029-E3785A12681F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{12464BFD-7489-403B-87AC-4F10CC74C954}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{12464BFD-7489-403B-87AC-4F10CC74C954}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,6 +77,21 @@
     <t>Multi</t>
   </si>
   <si>
+    <t>A,D</t>
+  </si>
+  <si>
+    <t>A,C,D</t>
+  </si>
+  <si>
+    <t>B,C</t>
+  </si>
+  <si>
+    <t>A,B</t>
+  </si>
+  <si>
+    <t>A,C</t>
+  </si>
+  <si>
     <t>Text</t>
   </si>
   <si>
@@ -443,6 +458,9 @@
     <t>Aux Power Distribution Cabinet</t>
   </si>
   <si>
+    <t>A,B,C,D</t>
+  </si>
+  <si>
     <t>Which of the following are components on the MVS4480-US transformer?</t>
   </si>
   <si>
@@ -467,6 +485,9 @@
     <t>Door Switch</t>
   </si>
   <si>
+    <t>A,B,D,E,F</t>
+  </si>
+  <si>
     <t>Explain the LOTO Procedure for the SG350HX-US and MVS4480-US. Be sure to include all steps and the testing point(s) to confirm de-energization. </t>
   </si>
   <si>
@@ -492,27 +513,6 @@
   </si>
   <si>
     <t>Explain how to configure grid protection and grid support parameters</t>
-  </si>
-  <si>
-    <t>B, C</t>
-  </si>
-  <si>
-    <t>A, B</t>
-  </si>
-  <si>
-    <t>A, C</t>
-  </si>
-  <si>
-    <t>A, C, D</t>
-  </si>
-  <si>
-    <t>A, D</t>
-  </si>
-  <si>
-    <t>A, B, C, D</t>
-  </si>
-  <si>
-    <t>A, B, D, E, F</t>
   </si>
 </sst>
 </file>
@@ -926,13 +926,13 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J1" t="s">
         <v>6</v>
@@ -946,7 +946,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C2">
         <v>12</v>
@@ -972,19 +972,19 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J3" t="s">
         <v>5</v>
@@ -998,19 +998,19 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>2</v>
@@ -1024,19 +1024,19 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="J5" t="s">
         <v>4</v>
@@ -1050,19 +1050,19 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="J6" t="s">
         <v>5</v>
@@ -1076,19 +1076,19 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="J7" t="s">
         <v>3</v>
@@ -1102,19 +1102,19 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J8" t="s">
         <v>5</v>
@@ -1128,19 +1128,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="J9" t="s">
         <v>3</v>
@@ -1154,10 +1154,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -1180,19 +1180,19 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="J11" t="s">
         <v>3</v>
@@ -1206,19 +1206,19 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="J12" t="s">
         <v>5</v>
@@ -1232,7 +1232,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1258,19 +1258,19 @@
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J14" t="s">
         <v>4</v>
@@ -1284,19 +1284,19 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J15" t="s">
         <v>5</v>
@@ -1310,19 +1310,19 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J16" t="s">
         <v>3</v>
@@ -1336,7 +1336,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1362,19 +1362,19 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F18" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J18" t="s">
         <v>5</v>
@@ -1388,19 +1388,19 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D19" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F19" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J19" t="s">
         <v>5</v>
@@ -1414,19 +1414,19 @@
         <v>8</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D20" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J20" t="s">
         <v>3</v>
@@ -1440,7 +1440,7 @@
         <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C21" t="b">
         <v>1</v>
@@ -1465,7 +1465,7 @@
         <v>8</v>
       </c>
       <c r="B22" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C22" t="b">
         <v>1</v>
@@ -1485,7 +1485,7 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
@@ -1505,7 +1505,7 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C24" t="b">
         <v>1</v>
@@ -1525,7 +1525,7 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
@@ -1545,7 +1545,7 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C26" t="b">
         <v>1</v>
@@ -1565,7 +1565,7 @@
         <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C27" t="b">
         <v>1</v>
@@ -1585,7 +1585,7 @@
         <v>8</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C28" t="b">
         <v>1</v>
@@ -1605,7 +1605,7 @@
         <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C29" t="b">
         <v>1</v>
@@ -1630,7 +1630,7 @@
         <v>8</v>
       </c>
       <c r="B30" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C30" t="b">
         <v>1</v>
@@ -1655,7 +1655,7 @@
         <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C31" t="b">
         <v>1</v>
@@ -1680,7 +1680,7 @@
         <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C32" t="b">
         <v>1</v>
@@ -1705,7 +1705,7 @@
         <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1730,7 +1730,7 @@
         <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C34" t="b">
         <v>1</v>
@@ -1755,25 +1755,25 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>153</v>
+        <v>16</v>
       </c>
       <c r="K35">
         <v>5</v>
@@ -1784,22 +1784,22 @@
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D36" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E36" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F36" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="J36" t="s">
-        <v>154</v>
+        <v>17</v>
       </c>
       <c r="K36">
         <v>5</v>
@@ -1810,22 +1810,22 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D37" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E37" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F37" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="J37" t="s">
-        <v>155</v>
+        <v>14</v>
       </c>
       <c r="K37">
         <v>5</v>
@@ -1836,22 +1836,22 @@
         <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C38" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D38" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E38" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F38" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="J38" t="s">
-        <v>156</v>
+        <v>13</v>
       </c>
       <c r="K38">
         <v>5</v>
@@ -1862,22 +1862,22 @@
         <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C39" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E39" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F39" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J39" t="s">
-        <v>152</v>
+        <v>15</v>
       </c>
       <c r="K39">
         <v>5</v>
@@ -1888,22 +1888,22 @@
         <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C40" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D40" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E40" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="F40" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="J40" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="K40">
         <v>5</v>
@@ -1914,31 +1914,31 @@
         <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C41" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D41" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E41" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F41" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="G41" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="H41" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="I41" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="J41" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="K41">
         <v>10</v>
@@ -1946,10 +1946,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B42" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="K42">
         <v>10</v>
@@ -1957,10 +1957,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -1974,10 +1974,10 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -1991,10 +1991,10 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B45" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -2008,10 +2008,10 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -2025,10 +2025,10 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -2042,10 +2042,10 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B48" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -2059,10 +2059,10 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B49" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -2076,10 +2076,10 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B50" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="K50">
         <v>10</v>

</xml_diff>

<commit_message>
Update SG350HX-US-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG350_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5421E68F-C743-FC45-9434-C12E8E48D3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A2774B-2192-C640-A3A1-10EE90D70423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{D88B995F-255D-AC4D-BBF8-CDAE9D204577}"/>
   </bookViews>
@@ -407,6 +407,9 @@
     <t>soft brush</t>
   </si>
   <si>
+    <t>A,D</t>
+  </si>
+  <si>
     <t>You can not open the inverter cover in which conditions?</t>
   </si>
   <si>
@@ -422,6 +425,9 @@
     <t>Sand storm</t>
   </si>
   <si>
+    <t>A,C,D</t>
+  </si>
+  <si>
     <t>During cold commission you must ensure that all HV cables are_____</t>
   </si>
   <si>
@@ -437,6 +443,9 @@
     <t>opened with no debris on cable</t>
   </si>
   <si>
+    <t>B,C</t>
+  </si>
+  <si>
     <t>Why is the correct system time important?</t>
   </si>
   <si>
@@ -452,6 +461,9 @@
     <t>Ensure MPPT tracking</t>
   </si>
   <si>
+    <t>A,B</t>
+  </si>
+  <si>
     <t>Why do you reserve specific clearance between the inverters</t>
   </si>
   <si>
@@ -467,6 +479,9 @@
     <t>To allow smooth bluetooth connection</t>
   </si>
   <si>
+    <t>A,C</t>
+  </si>
+  <si>
     <t>Text</t>
   </si>
   <si>
@@ -486,21 +501,6 @@
   </si>
   <si>
     <t>Why you should not stretch a DC wire on the SG350?</t>
-  </si>
-  <si>
-    <t>A, C, D</t>
-  </si>
-  <si>
-    <t>B, C</t>
-  </si>
-  <si>
-    <t>A, B</t>
-  </si>
-  <si>
-    <t>A, C</t>
-  </si>
-  <si>
-    <t>A, D</t>
   </si>
 </sst>
 </file>
@@ -566,9 +566,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -606,7 +606,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -712,7 +712,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -854,7 +854,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -862,7 +862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDE9EF6-57F4-9041-8353-DDD0DBD53FBC}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -870,11 +870,11 @@
     <col min="3" max="3" width="19.1640625" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="5" width="43.5" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -893,16 +893,14 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -921,16 +919,14 @@
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -949,16 +945,14 @@
       <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H3" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -977,16 +971,14 @@
       <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1005,16 +997,14 @@
       <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J5" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H5" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1033,16 +1023,14 @@
       <c r="F6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1061,16 +1049,14 @@
       <c r="F7" s="1">
         <v>120</v>
       </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H7" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1089,16 +1075,14 @@
       <c r="F8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J8" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H8" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1117,16 +1101,14 @@
       <c r="F9" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J9" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H9" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1145,16 +1127,14 @@
       <c r="F10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J10" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1173,16 +1153,14 @@
       <c r="F11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1201,16 +1179,14 @@
       <c r="F12" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J12" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H12" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1229,16 +1205,14 @@
       <c r="F13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J13" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H13" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -1257,16 +1231,14 @@
       <c r="F14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J14" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H14" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -1285,16 +1257,14 @@
       <c r="F15" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J15" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H15" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
@@ -1313,16 +1283,14 @@
       <c r="F16" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1341,16 +1309,14 @@
       <c r="F17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J17" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H17" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1369,16 +1335,14 @@
       <c r="F18" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J18" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H18" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
@@ -1397,16 +1361,14 @@
       <c r="F19" s="3">
         <v>0.1</v>
       </c>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J19" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H19" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -1425,16 +1387,14 @@
       <c r="F20" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J20" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H20" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
@@ -1453,16 +1413,14 @@
       <c r="F21" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J21" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H21" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -1481,16 +1439,14 @@
       <c r="F22" s="1">
         <v>16</v>
       </c>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J22" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H22" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1509,16 +1465,14 @@
       <c r="F23" s="1">
         <v>42</v>
       </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J23" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G23" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -1537,16 +1491,14 @@
       <c r="F24" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J24" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H24" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -1561,16 +1513,14 @@
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J25" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H25" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1585,16 +1535,14 @@
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J26" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H26" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1609,16 +1557,14 @@
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J27" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H27" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1633,16 +1579,14 @@
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J28" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H28" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1657,16 +1601,14 @@
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J29" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H29" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1681,16 +1623,14 @@
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J30" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H30" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1705,16 +1645,14 @@
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J31" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H31" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1729,16 +1667,14 @@
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J32" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H32" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1753,16 +1689,14 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1" t="s">
+      <c r="G33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J33" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H33" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1777,16 +1711,14 @@
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J34" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H34" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1801,16 +1733,14 @@
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J35" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H35" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1825,16 +1755,14 @@
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J36" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H36" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1849,16 +1777,14 @@
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J37" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H37" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1873,16 +1799,14 @@
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J38" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H38" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -1897,16 +1821,14 @@
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J39" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H39" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>117</v>
       </c>
@@ -1925,188 +1847,180 @@
       <c r="F40" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="J40" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G40" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H40" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>117</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C41" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D41" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="J41" s="1">
+        <v>128</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H41" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>117</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C42" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D42" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="J42" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H42" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>117</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C43" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="J43" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H43" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>117</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D44" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I44" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H44" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>148</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H45" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B46" t="s">
+        <v>150</v>
+      </c>
+      <c r="H46" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" t="s">
+        <v>151</v>
+      </c>
+      <c r="H47" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H48" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>148</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="J44" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>143</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J45" s="1">
+      <c r="H49" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>143</v>
-      </c>
-      <c r="B46" t="s">
-        <v>145</v>
-      </c>
-      <c r="J46" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>143</v>
-      </c>
-      <c r="B47" t="s">
-        <v>146</v>
-      </c>
-      <c r="J47" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>143</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="J48" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>143</v>
-      </c>
-      <c r="B49" s="1" t="s">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>148</v>
       </c>
-      <c r="J49" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>143</v>
-      </c>
       <c r="B50" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="J50" s="1">
+        <v>154</v>
+      </c>
+      <c r="H50" s="1">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update SG4400UD-MV-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG4400_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A20E774-64D0-6B45-9DE0-06F8365FDAC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D839C5-57CD-B64D-AB8F-2E40A6913899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{DEE7CDAF-3686-8344-A83E-8AE1519D283D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="263">
   <si>
     <t>Type</t>
   </si>
@@ -832,12 +832,27 @@
   <si>
     <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, inverter cabinet doors can still be opened.</t>
   </si>
+  <si>
+    <t>Correct Answer</t>
+  </si>
+  <si>
+    <t>Points</t>
+  </si>
+  <si>
+    <t>A,B,C,D</t>
+  </si>
+  <si>
+    <t>B, D, E</t>
+  </si>
+  <si>
+    <t>A, E</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -876,6 +891,12 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -897,7 +918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -906,6 +927,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1221,10 +1245,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B9D14F3-5CCD-E146-AD37-6ECFB6A100CC}">
-  <dimension ref="A1:H78"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O78"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="127.1640625" customWidth="1"/>
+    <col min="3" max="3" width="65.5" style="4" customWidth="1"/>
+    <col min="4" max="4" width="85" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="58.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5" style="4" customWidth="1"/>
+    <col min="9" max="9" width="5.83203125" customWidth="1"/>
+    <col min="10" max="10" width="19.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1249,8 +1283,15 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="1"/>
+      <c r="J1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1271,8 +1312,19 @@
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="1"/>
+      <c r="J2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="1">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1293,8 +1345,19 @@
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="1">
+        <v>5</v>
+      </c>
+      <c r="L3" s="1"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1315,8 +1378,19 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I4" s="1"/>
+      <c r="J4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5</v>
+      </c>
+      <c r="L4" s="1"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1337,8 +1411,19 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K5" s="1">
+        <v>5</v>
+      </c>
+      <c r="L5" s="1"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1359,8 +1444,19 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" s="1"/>
+      <c r="J6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K6" s="1">
+        <v>5</v>
+      </c>
+      <c r="L6" s="1"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1381,8 +1477,19 @@
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7" s="1">
+        <v>5</v>
+      </c>
+      <c r="L7" s="1"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1403,8 +1510,19 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="1">
+        <v>5</v>
+      </c>
+      <c r="L8" s="1"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1425,8 +1543,15 @@
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" s="1"/>
+      <c r="J9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1447,8 +1572,15 @@
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I10" s="1"/>
+      <c r="J10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1469,8 +1601,15 @@
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I11" s="1"/>
+      <c r="J11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K11" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1491,8 +1630,15 @@
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I12" s="1"/>
+      <c r="J12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K12" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1513,8 +1659,15 @@
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I13" s="1"/>
+      <c r="J13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K13" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -1535,8 +1688,15 @@
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I14" s="1"/>
+      <c r="J14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -1557,8 +1717,15 @@
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I15" s="1"/>
+      <c r="J15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K15" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
@@ -1579,8 +1746,15 @@
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I16" s="1"/>
+      <c r="J16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1601,8 +1775,15 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="1"/>
+      <c r="J17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K17" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1623,8 +1804,15 @@
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="1"/>
+      <c r="J18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
@@ -1645,8 +1833,15 @@
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="1"/>
+      <c r="J19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -1667,8 +1862,15 @@
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="1"/>
+      <c r="J20" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K20" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
@@ -1689,8 +1891,15 @@
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="1"/>
+      <c r="J21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K21" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -1711,8 +1920,15 @@
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="1"/>
+      <c r="J22" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K22" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1733,8 +1949,19 @@
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" s="1"/>
+      <c r="J23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K23" s="1">
+        <v>5</v>
+      </c>
+      <c r="L23" s="1"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
@@ -1755,8 +1982,19 @@
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" s="1"/>
+      <c r="J24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K24" s="1">
+        <v>5</v>
+      </c>
+      <c r="L24" s="1"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>8</v>
       </c>
@@ -1777,8 +2015,19 @@
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I25" s="1"/>
+      <c r="J25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" s="1">
+        <v>5</v>
+      </c>
+      <c r="L25" s="1"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
@@ -1799,8 +2048,19 @@
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I26" s="1"/>
+      <c r="J26" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K26" s="1">
+        <v>5</v>
+      </c>
+      <c r="L26" s="1"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="5"/>
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
@@ -1821,8 +2081,19 @@
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I27" s="1"/>
+      <c r="J27" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K27" s="1">
+        <v>5</v>
+      </c>
+      <c r="L27" s="1"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>8</v>
       </c>
@@ -1843,8 +2114,19 @@
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
-    </row>
-    <row r="29" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="I28" s="1"/>
+      <c r="J28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K28" s="1">
+        <v>5</v>
+      </c>
+      <c r="L28" s="1"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+    </row>
+    <row r="29" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>8</v>
       </c>
@@ -1865,8 +2147,19 @@
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I29" s="1"/>
+      <c r="J29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K29" s="1">
+        <v>5</v>
+      </c>
+      <c r="L29" s="1"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
@@ -1887,8 +2180,19 @@
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I30" s="1"/>
+      <c r="J30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K30" s="1">
+        <v>5</v>
+      </c>
+      <c r="L30" s="1"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>8</v>
       </c>
@@ -1909,8 +2213,19 @@
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I31" s="1"/>
+      <c r="J31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K31" s="1">
+        <v>5</v>
+      </c>
+      <c r="L31" s="1"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>8</v>
       </c>
@@ -1931,8 +2246,19 @@
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I32" s="1"/>
+      <c r="J32" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K32" s="1">
+        <v>5</v>
+      </c>
+      <c r="L32" s="1"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>8</v>
       </c>
@@ -1953,8 +2279,19 @@
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I33" s="1"/>
+      <c r="J33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K33" s="1">
+        <v>5</v>
+      </c>
+      <c r="L33" s="1"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>8</v>
       </c>
@@ -1975,8 +2312,19 @@
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I34" s="1"/>
+      <c r="J34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K34" s="1">
+        <v>5</v>
+      </c>
+      <c r="L34" s="1"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>149</v>
       </c>
@@ -1997,8 +2345,19 @@
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I35" s="1"/>
+      <c r="J35" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K35" s="1">
+        <v>5</v>
+      </c>
+      <c r="L35" s="1"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>149</v>
       </c>
@@ -2019,8 +2378,19 @@
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I36" s="1"/>
+      <c r="J36" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K36" s="1">
+        <v>5</v>
+      </c>
+      <c r="L36" s="1"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>8</v>
       </c>
@@ -2037,8 +2407,19 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I37" s="1"/>
+      <c r="J37" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K37" s="1">
+        <v>5</v>
+      </c>
+      <c r="L37" s="1"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>8</v>
       </c>
@@ -2055,8 +2436,19 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I38" s="1"/>
+      <c r="J38" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K38" s="1">
+        <v>5</v>
+      </c>
+      <c r="L38" s="1"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>8</v>
       </c>
@@ -2073,8 +2465,19 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I39" s="1"/>
+      <c r="J39" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K39" s="1">
+        <v>5</v>
+      </c>
+      <c r="L39" s="1"/>
+      <c r="M39" s="5"/>
+      <c r="N39" s="5"/>
+      <c r="O39" s="5"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>8</v>
       </c>
@@ -2091,8 +2494,19 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I40" s="1"/>
+      <c r="J40" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K40" s="1">
+        <v>5</v>
+      </c>
+      <c r="L40" s="1"/>
+      <c r="M40" s="5"/>
+      <c r="N40" s="5"/>
+      <c r="O40" s="5"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>8</v>
       </c>
@@ -2109,8 +2523,19 @@
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I41" s="1"/>
+      <c r="J41" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K41" s="1">
+        <v>5</v>
+      </c>
+      <c r="L41" s="1"/>
+      <c r="M41" s="5"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>8</v>
       </c>
@@ -2127,8 +2552,19 @@
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I42" s="1"/>
+      <c r="J42" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K42" s="1">
+        <v>5</v>
+      </c>
+      <c r="L42" s="1"/>
+      <c r="M42" s="5"/>
+      <c r="N42" s="5"/>
+      <c r="O42" s="5"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>8</v>
       </c>
@@ -2145,8 +2581,19 @@
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I43" s="1"/>
+      <c r="J43" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K43" s="1">
+        <v>5</v>
+      </c>
+      <c r="L43" s="1"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="5"/>
+      <c r="O43" s="5"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>8</v>
       </c>
@@ -2163,8 +2610,19 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I44" s="1"/>
+      <c r="J44" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K44" s="1">
+        <v>5</v>
+      </c>
+      <c r="L44" s="1"/>
+      <c r="M44" s="5"/>
+      <c r="N44" s="5"/>
+      <c r="O44" s="5"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>8</v>
       </c>
@@ -2181,8 +2639,19 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I45" s="1"/>
+      <c r="J45" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K45" s="1">
+        <v>5</v>
+      </c>
+      <c r="L45" s="1"/>
+      <c r="M45" s="5"/>
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>8</v>
       </c>
@@ -2199,8 +2668,19 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I46" s="1"/>
+      <c r="J46" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K46" s="1">
+        <v>5</v>
+      </c>
+      <c r="L46" s="1"/>
+      <c r="M46" s="5"/>
+      <c r="N46" s="5"/>
+      <c r="O46" s="5"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>8</v>
       </c>
@@ -2217,8 +2697,19 @@
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I47" s="1"/>
+      <c r="J47" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K47" s="1">
+        <v>5</v>
+      </c>
+      <c r="L47" s="1"/>
+      <c r="M47" s="5"/>
+      <c r="N47" s="5"/>
+      <c r="O47" s="5"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -2235,8 +2726,15 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I48" s="1"/>
+      <c r="J48" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K48" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -2253,8 +2751,15 @@
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I49" s="1"/>
+      <c r="J49" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K49" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>8</v>
       </c>
@@ -2271,8 +2776,15 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I50" s="1"/>
+      <c r="J50" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K50" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>8</v>
       </c>
@@ -2289,8 +2801,15 @@
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
-    </row>
-    <row r="52" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="I51" s="1"/>
+      <c r="J51" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K51" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>8</v>
       </c>
@@ -2309,10 +2828,14 @@
       <c r="F52" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-    </row>
-    <row r="53" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J52" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K52" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>8</v>
       </c>
@@ -2331,10 +2854,14 @@
       <c r="F53" s="4">
         <v>4</v>
       </c>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-    </row>
-    <row r="54" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J53" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K53" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>8</v>
       </c>
@@ -2347,12 +2874,14 @@
       <c r="D54" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-    </row>
-    <row r="55" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J54" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K54" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>8</v>
       </c>
@@ -2371,10 +2900,14 @@
       <c r="F55" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-    </row>
-    <row r="56" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J55" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K55" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>8</v>
       </c>
@@ -2387,12 +2920,14 @@
       <c r="D56" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-    </row>
-    <row r="57" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J56" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K56" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>8</v>
       </c>
@@ -2411,10 +2946,14 @@
       <c r="F57" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-    </row>
-    <row r="58" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J57" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K57" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>8</v>
       </c>
@@ -2433,10 +2972,14 @@
       <c r="F58" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-    </row>
-    <row r="59" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J58" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K58" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>8</v>
       </c>
@@ -2455,10 +2998,14 @@
       <c r="F59" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-    </row>
-    <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J59" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K59" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>8</v>
       </c>
@@ -2471,12 +3018,14 @@
       <c r="D60" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-    </row>
-    <row r="61" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J60" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K60" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>8</v>
       </c>
@@ -2492,11 +3041,14 @@
       <c r="E61" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-    </row>
-    <row r="62" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J61" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K61" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>8</v>
       </c>
@@ -2515,10 +3067,14 @@
       <c r="F62" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-    </row>
-    <row r="63" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J62" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K62" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>8</v>
       </c>
@@ -2531,12 +3087,14 @@
       <c r="D63" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-    </row>
-    <row r="64" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J63" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K63" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>8</v>
       </c>
@@ -2555,10 +3113,14 @@
       <c r="F64" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-    </row>
-    <row r="65" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J64" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K64" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>8</v>
       </c>
@@ -2577,10 +3139,14 @@
       <c r="F65" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-    </row>
-    <row r="66" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J65" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K65" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>8</v>
       </c>
@@ -2593,12 +3159,14 @@
       <c r="D66" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-    </row>
-    <row r="67" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J66" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K66" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>8</v>
       </c>
@@ -2617,10 +3185,14 @@
       <c r="F67" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-    </row>
-    <row r="68" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J67" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K67" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>8</v>
       </c>
@@ -2639,10 +3211,14 @@
       <c r="F68" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-    </row>
-    <row r="69" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J68" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K68" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>8</v>
       </c>
@@ -2655,12 +3231,14 @@
       <c r="D69" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-    </row>
-    <row r="70" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J69" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K69" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>8</v>
       </c>
@@ -2679,10 +3257,14 @@
       <c r="F70" s="3">
         <v>4</v>
       </c>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-    </row>
-    <row r="71" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J70" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K70" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>8</v>
       </c>
@@ -2701,10 +3283,14 @@
       <c r="F71" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-    </row>
-    <row r="72" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J71" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K71" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>8</v>
       </c>
@@ -2723,10 +3309,14 @@
       <c r="F72" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="G72" s="4"/>
-      <c r="H72" s="4"/>
-    </row>
-    <row r="73" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J72" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K72" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>8</v>
       </c>
@@ -2739,12 +3329,14 @@
       <c r="D73" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-    </row>
-    <row r="74" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J73" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K73" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>8</v>
       </c>
@@ -2757,12 +3349,14 @@
       <c r="D74" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E74" s="4"/>
-      <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4"/>
-    </row>
-    <row r="75" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J74" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K74" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>8</v>
       </c>
@@ -2781,10 +3375,14 @@
       <c r="F75" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="G75" s="4"/>
-      <c r="H75" s="4"/>
-    </row>
-    <row r="76" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J75" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K75" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>149</v>
       </c>
@@ -2806,9 +3404,14 @@
       <c r="G76" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="H76" s="4"/>
-    </row>
-    <row r="77" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J76" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K76" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
@@ -2830,9 +3433,14 @@
       <c r="G77" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="H77" s="4"/>
-    </row>
-    <row r="78" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+      <c r="J77" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="K77" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>8</v>
       </c>
@@ -2845,10 +3453,12 @@
       <c r="D78" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="E78" s="4"/>
-      <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
-      <c r="H78" s="4"/>
+      <c r="J78" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K78" s="1">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update SG3150U-MV-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG3150_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898E1920-8827-FB43-AA1D-66AD02DC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6660FD24-A09E-C749-95CE-14B32CFFF9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{0EF93C32-E07B-4E4A-AC36-FEF3B1CAF2A7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19100" xr2:uid="{0EF93C32-E07B-4E4A-AC36-FEF3B1CAF2A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="142">
   <si>
     <t>Type</t>
   </si>
@@ -368,9 +368,6 @@
     <t>MV Transformer/Grid</t>
   </si>
   <si>
-    <t>B, D, F</t>
-  </si>
-  <si>
     <t>What protective equipment (PPE) should be correctly worn during inverter maintenance?</t>
   </si>
   <si>
@@ -384,9 +381,6 @@
   </si>
   <si>
     <t>EH rated boots</t>
-  </si>
-  <si>
-    <t>A, B, C, D, E</t>
   </si>
   <si>
     <t>What tests do you need to perform when the unit has been in storage for 1 year?</t>
@@ -447,9 +441,6 @@
   </si>
   <si>
     <t>FU35, FU36, and FU37</t>
-  </si>
-  <si>
-    <t>B, C, E</t>
   </si>
   <si>
     <t>Text</t>
@@ -506,6 +497,12 @@
   </si>
   <si>
     <t>A, B, C, D</t>
+  </si>
+  <si>
+    <t>B, D</t>
+  </si>
+  <si>
+    <t>B, C</t>
   </si>
 </sst>
 </file>
@@ -600,9 +597,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -640,7 +637,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -746,7 +743,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -888,7 +885,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -899,9 +896,10 @@
   <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="199" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="122.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.25">
@@ -1705,7 +1703,7 @@
         <v>109</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="H34">
         <v>10</v>
@@ -1716,22 +1714,22 @@
         <v>98</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" t="s">
         <v>111</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>112</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>113</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="G35" s="2" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="H35" s="2">
         <v>10</v>
@@ -1742,22 +1740,22 @@
         <v>98</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" t="s">
+        <v>116</v>
+      </c>
+      <c r="D36" t="s">
         <v>117</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" t="s">
         <v>118</v>
       </c>
-      <c r="D36" t="s">
+      <c r="F36" t="s">
         <v>119</v>
       </c>
-      <c r="E36" t="s">
-        <v>120</v>
-      </c>
-      <c r="F36" t="s">
-        <v>121</v>
-      </c>
       <c r="G36" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H36" s="2">
         <v>10</v>
@@ -1768,22 +1766,22 @@
         <v>98</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="E37" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>126</v>
-      </c>
       <c r="G37" s="1" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="H37">
         <v>5</v>
@@ -1791,10 +1789,10 @@
     </row>
     <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H38">
         <v>5</v>
@@ -1802,10 +1800,10 @@
     </row>
     <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H39">
         <v>5</v>
@@ -1813,10 +1811,10 @@
     </row>
     <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="H40">
         <v>10</v>
@@ -1824,10 +1822,10 @@
     </row>
     <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="H41">
         <v>10</v>
@@ -1835,10 +1833,10 @@
     </row>
     <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H42">
         <v>10</v>
@@ -1846,10 +1844,10 @@
     </row>
     <row r="43" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H43">
         <v>10</v>
@@ -1857,10 +1855,10 @@
     </row>
     <row r="44" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H44">
         <v>5</v>
@@ -1868,10 +1866,10 @@
     </row>
     <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H45">
         <v>10</v>
@@ -1879,10 +1877,10 @@
     </row>
     <row r="46" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H46">
         <v>10</v>
@@ -1890,10 +1888,10 @@
     </row>
     <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H47">
         <v>10</v>
@@ -1901,10 +1899,10 @@
     </row>
     <row r="48" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H48">
         <v>10</v>
@@ -1912,10 +1910,10 @@
     </row>
     <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H49">
         <v>10</v>
@@ -1923,10 +1921,10 @@
     </row>
     <row r="50" spans="1:8" ht="17" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initialization of the transformer branch
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/jannessa_zeng_sungrow-na_com/Documents/Desktop/testing Pool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{7168CEDD-A3A6-4410-B91A-237DEDACDC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0506225F-996E-44CB-BA18-093D01E256D1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9754BA-18EB-4B46-93C8-25A3FE39D259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28020" yWindow="1980" windowWidth="25500" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -64,12 +63,6 @@
     <t>Points</t>
   </si>
   <si>
-    <t>A,C,D</t>
-  </si>
-  <si>
-    <t>A,B,C,D</t>
-  </si>
-  <si>
     <t>When isolating the low voltage equipment from the transformer, what needs to be done first?</t>
   </si>
   <si>
@@ -223,9 +216,6 @@
     <t>The float ball of the oil level gauge falls or the connecting rod malfunctions</t>
   </si>
   <si>
-    <t>A,B,C</t>
-  </si>
-  <si>
     <t>When the pressure relief valve leakage problem occurs, what are the possible causes? (Select all that apply)</t>
   </si>
   <si>
@@ -497,6 +487,15 @@
   </si>
   <si>
     <t>The HV resistance imbalance between each phase should be less than 2%</t>
+  </si>
+  <si>
+    <t>A, C, D</t>
+  </si>
+  <si>
+    <t>A, B, C, D</t>
+  </si>
+  <si>
+    <t>A, B, C</t>
   </si>
 </sst>
 </file>
@@ -571,10 +570,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -841,22 +836,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O46"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="124.7265625" customWidth="1"/>
-    <col min="3" max="3" width="63.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="124.6640625" customWidth="1"/>
+    <col min="3" max="3" width="63.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.1640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.26953125" customWidth="1"/>
+    <col min="7" max="7" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.33203125" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -888,38 +883,38 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="J2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="C3" s="2">
         <v>14253</v>
@@ -943,24 +938,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -972,24 +967,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -1001,24 +996,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -1030,24 +1025,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -1059,24 +1054,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -1088,157 +1083,157 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2" t="s">
-        <v>12</v>
+        <v>154</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>13</v>
+        <v>155</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2" t="s">
-        <v>13</v>
+        <v>155</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>65</v>
+        <v>156</v>
       </c>
       <c r="K12">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>13</v>
+        <v>155</v>
       </c>
       <c r="K13">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C14" s="2" t="b">
         <v>1</v>
@@ -1258,12 +1253,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="b">
         <v>1</v>
@@ -1283,12 +1278,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C16" s="2" t="b">
         <v>1</v>
@@ -1308,12 +1303,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C17" s="2" t="b">
         <v>1</v>
@@ -1333,12 +1328,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C18" s="2" t="b">
         <v>1</v>
@@ -1358,12 +1353,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C19" s="2" t="b">
         <v>1</v>
@@ -1383,12 +1378,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C20" s="2" t="b">
         <v>1</v>
@@ -1408,12 +1403,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>8</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C21" s="2" t="b">
         <v>1</v>
@@ -1433,12 +1428,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>8</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C22" s="2" t="b">
         <v>1</v>
@@ -1458,12 +1453,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C23" s="2" t="b">
         <v>1</v>
@@ -1483,12 +1478,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1502,12 +1497,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1521,12 +1516,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C26" s="2"/>
       <c r="J26" s="2"/>
@@ -1534,24 +1529,24 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -1567,24 +1562,24 @@
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
     </row>
-    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -1600,24 +1595,24 @@
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
     </row>
-    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="F29" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>99</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -1633,24 +1628,24 @@
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
     </row>
-    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>104</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -1666,24 +1661,24 @@
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
     </row>
-    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="F31" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -1699,24 +1694,24 @@
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
     </row>
-    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="F32" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -1732,24 +1727,24 @@
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
     </row>
-    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B33" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="F33" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -1765,24 +1760,24 @@
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
     </row>
-    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>124</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -1798,24 +1793,24 @@
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
     </row>
-    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B35" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -1831,24 +1826,24 @@
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
     </row>
-    <row r="36" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B36" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>134</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -1864,24 +1859,24 @@
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
     </row>
-    <row r="37" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>136</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -1897,24 +1892,24 @@
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
     </row>
-    <row r="38" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>144</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -1930,12 +1925,12 @@
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
     </row>
-    <row r="39" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C39" s="4">
         <v>0.5</v>
@@ -1963,24 +1958,24 @@
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
     </row>
-    <row r="40" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B40" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="F40" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>150</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -1996,12 +1991,12 @@
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
     </row>
-    <row r="41" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C41" s="4" t="b">
         <v>1</v>
@@ -2025,12 +2020,12 @@
       <c r="N41" s="4"/>
       <c r="O41" s="4"/>
     </row>
-    <row r="42" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C42" s="4" t="b">
         <v>1</v>
@@ -2054,12 +2049,12 @@
       <c r="N42" s="4"/>
       <c r="O42" s="4"/>
     </row>
-    <row r="43" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C43" s="4" t="b">
         <v>1</v>
@@ -2083,12 +2078,12 @@
       <c r="N43" s="4"/>
       <c r="O43" s="4"/>
     </row>
-    <row r="44" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C44" s="4" t="b">
         <v>1</v>
@@ -2112,12 +2107,12 @@
       <c r="N44" s="4"/>
       <c r="O44" s="4"/>
     </row>
-    <row r="45" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C45" s="4" t="b">
         <v>1</v>
@@ -2141,12 +2136,12 @@
       <c r="N45" s="4"/>
       <c r="O45" s="4"/>
     </row>
-    <row r="46" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C46" s="4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
initialization of the transformer CSP Safety  branch
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/jannessa_zeng_sungrow-na_com/Documents/Desktop/testing Pool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{196BE576-945B-438E-9011-CA3EC6259116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F58955B7-94CB-475E-AE48-CA0C89A7F4FF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83867A-897A-274A-A53E-0C0454A78D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="100" windowWidth="19380" windowHeight="11180" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
+    <workbookView xWindow="-33560" yWindow="600" windowWidth="26060" windowHeight="18220" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -215,9 +215,6 @@
     <t>Does flipping the oil switch (MVT load switch) isolate the entire HV room?</t>
   </si>
   <si>
-    <t>A,C,D,F</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -392,9 +389,6 @@
     <t>Moisture</t>
   </si>
   <si>
-    <t>A,B,C</t>
-  </si>
-  <si>
     <t>What is the primary function of a four position oil switch?</t>
   </si>
   <si>
@@ -410,7 +404,13 @@
     <t>Isolate H1A from H2A</t>
   </si>
   <si>
-    <t>A,B,D</t>
+    <t>A, C, D, F</t>
+  </si>
+  <si>
+    <t>A, B, C</t>
+  </si>
+  <si>
+    <t>A, B, D</t>
   </si>
 </sst>
 </file>
@@ -825,22 +825,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E0A9B9-0213-449D-9599-DFD4E1E1084D}">
   <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="124.7265625" customWidth="1"/>
-    <col min="3" max="3" width="63.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.1796875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="124.6640625" customWidth="1"/>
+    <col min="3" max="3" width="63.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.1640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.26953125" customWidth="1"/>
+    <col min="7" max="7" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.33203125" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -872,7 +872,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -901,7 +901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -928,7 +928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -957,7 +957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -986,7 +986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1013,13 +1013,13 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="K6">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1243,10 +1243,10 @@
         <v>58</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -1260,24 +1260,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
@@ -1293,12 +1293,12 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
     </row>
-    <row r="17" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17" s="4">
         <v>90</v>
@@ -1326,24 +1326,24 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -1359,24 +1359,24 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
     </row>
-    <row r="19" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>77</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
@@ -1392,24 +1392,24 @@
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
     </row>
-    <row r="20" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="F20" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
@@ -1425,24 +1425,24 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
     </row>
-    <row r="21" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
@@ -1458,24 +1458,24 @@
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
     </row>
-    <row r="22" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
@@ -1491,24 +1491,24 @@
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
@@ -1524,24 +1524,24 @@
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
     </row>
-    <row r="24" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
@@ -1557,12 +1557,12 @@
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
     </row>
-    <row r="25" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C25" s="4" t="b">
         <v>1</v>
@@ -1586,12 +1586,12 @@
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
     </row>
-    <row r="26" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C26" s="4" t="b">
         <v>1</v>
@@ -1615,12 +1615,12 @@
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
     </row>
-    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C27" s="4" t="b">
         <v>1</v>
@@ -1644,12 +1644,12 @@
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
     </row>
-    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="4" t="b">
         <v>1</v>
@@ -1673,12 +1673,12 @@
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
     </row>
-    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C29" s="4" t="b">
         <v>1</v>
@@ -1702,12 +1702,12 @@
       <c r="N29" s="6"/>
       <c r="O29" s="6"/>
     </row>
-    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C30" s="4" t="b">
         <v>1</v>
@@ -1731,12 +1731,12 @@
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
     </row>
-    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C31" s="4" t="b">
         <v>1</v>
@@ -1760,12 +1760,12 @@
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
     </row>
-    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C32" s="4" t="b">
         <v>1</v>
@@ -1789,12 +1789,12 @@
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
     </row>
-    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C33" s="4" t="b">
         <v>1</v>
@@ -1818,30 +1818,30 @@
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
     </row>
-    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="E34" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="K34" s="4">
         <v>5</v>
@@ -1851,24 +1851,24 @@
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
     </row>
-    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B35" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="E35" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
@@ -1876,7 +1876,9 @@
       <c r="J35" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="K35" s="4"/>
+      <c r="K35" s="4">
+        <v>5</v>
+      </c>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
       <c r="N35" s="6"/>
@@ -1884,6 +1886,18 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
     <mergeCell ref="G34:I34"/>
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="G28:I28"/>
@@ -1892,18 +1906,6 @@
     <mergeCell ref="G31:I31"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="G33:I33"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="G21:I21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update SG3600UD-MV question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG3600/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{620DB007-EFC3-6149-A11A-4E3D16A64B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E17B52D1-FD2E-F542-A2FE-4B4324ECE955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87A712DC-3966-4382-9131-53439D8335E7}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="18560" xr2:uid="{C1094EB1-E11C-4826-97C7-12D07005C403}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C1094EB1-E11C-4826-97C7-12D07005C403}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="254">
   <si>
     <t>Type</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>Multi</t>
+  </si>
+  <si>
+    <t>A,C</t>
   </si>
   <si>
     <t>SCU is another name for which board?</t>
@@ -452,6 +455,9 @@
     <t>After completing initial inspections and mechanical checks, begin the transformer soaking process</t>
   </si>
   <si>
+    <t>A,B,C,D,E</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Which of the following checks should be performed during cold commissioning? </t>
     </r>
@@ -543,6 +549,9 @@
   </si>
   <si>
     <t>Cooling fan</t>
+  </si>
+  <si>
+    <t>A,B,C</t>
   </si>
   <si>
     <t>What factors does the output of a PV array depend on?</t>
@@ -623,6 +632,9 @@
     <t>PT</t>
   </si>
   <si>
+    <t>B,D</t>
+  </si>
+  <si>
     <t>Which of the following components/locations need to be checked for oil leakage during MVT commissioning and routine maintenance? </t>
   </si>
   <si>
@@ -630,6 +642,9 @@
   </si>
   <si>
     <t>Oil Thermostat</t>
+  </si>
+  <si>
+    <t>A,B,C,D</t>
   </si>
   <si>
     <r>
@@ -659,6 +674,9 @@
     <t>Steps down voltage, steps up current</t>
   </si>
   <si>
+    <t>C,D</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Which of the following are losses associated with a transformer? </t>
     </r>
@@ -686,6 +704,9 @@
     <t>Friction losses</t>
   </si>
   <si>
+    <t>A,B</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">What are the requirements of transformer bushings? </t>
     </r>
@@ -812,6 +833,9 @@
     <t xml:space="preserve"> All sources of energy involved should be considered during isolation</t>
   </si>
   <si>
+    <t>B,C,D</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">What information should be clearly marked and identified on a red tag for items being returned? </t>
     </r>
@@ -868,6 +892,9 @@
     <t>Combiner Box Switch</t>
   </si>
   <si>
+    <t>A,B,C,DE</t>
+  </si>
+  <si>
     <t>What are the names of the registers that relate to the active power output?</t>
   </si>
   <si>
@@ -935,27 +962,6 @@
   </si>
   <si>
     <t>If there is no incident energy sticker found on the power distribution/aux cabinet, I am permitted to access it while the skid is energized, as long as I have on a CAT4 suit.</t>
-  </si>
-  <si>
-    <t>A, B, C, D, E</t>
-  </si>
-  <si>
-    <t>A, B, C</t>
-  </si>
-  <si>
-    <t>B, D</t>
-  </si>
-  <si>
-    <t>C, D</t>
-  </si>
-  <si>
-    <t>A, B</t>
-  </si>
-  <si>
-    <t>A, C</t>
-  </si>
-  <si>
-    <t>B, C, D</t>
   </si>
 </sst>
 </file>
@@ -1849,21 +1855,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E92F6612-5B7E-41F0-8CF2-706367AFE299}">
   <dimension ref="A1:K60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="126" customWidth="1"/>
-    <col min="3" max="4" width="18.5" customWidth="1"/>
-    <col min="5" max="5" width="23.5" customWidth="1"/>
-    <col min="6" max="6" width="21.5" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.7265625" customWidth="1"/>
+    <col min="3" max="4" width="18.453125" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="6" max="6" width="21.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" customWidth="1"/>
-    <col min="11" max="11" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" customWidth="1"/>
+    <col min="10" max="10" width="15.36328125" customWidth="1"/>
+    <col min="11" max="11" width="8.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1895,24 +1901,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -1924,24 +1930,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -1953,12 +1959,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2">
         <v>18</v>
@@ -1982,24 +1988,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -2011,24 +2017,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -2040,24 +2046,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -2069,24 +2075,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -2098,24 +2104,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -2127,24 +2133,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -2156,24 +2162,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -2185,24 +2191,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="2">
         <v>1111</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -2214,24 +2220,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -2243,24 +2249,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -2272,24 +2278,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E15" s="1">
         <v>2222</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -2301,12 +2307,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="1">
         <v>15</v>
@@ -2318,7 +2324,7 @@
         <v>60</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -2330,24 +2336,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -2359,24 +2365,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -2388,24 +2394,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -2417,24 +2423,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
@@ -2446,12 +2452,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" s="1">
         <v>1</v>
@@ -2475,24 +2481,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -2504,24 +2510,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -2533,24 +2539,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -2562,24 +2568,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -2591,24 +2597,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -2620,24 +2626,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -2649,24 +2655,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -2678,24 +2684,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -2707,24 +2713,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -2736,24 +2742,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -2765,635 +2771,634 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2" t="s">
-        <v>245</v>
+        <v>135</v>
       </c>
       <c r="K32" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>245</v>
+        <v>135</v>
       </c>
       <c r="K33" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2" t="s">
-        <v>245</v>
+        <v>135</v>
       </c>
       <c r="K34" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2" t="s">
-        <v>246</v>
+        <v>155</v>
       </c>
       <c r="K35" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K36" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K37" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K38" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2" t="s">
-        <v>247</v>
+        <v>175</v>
       </c>
       <c r="K39" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:11" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="K40" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2" t="s">
-        <v>248</v>
+        <v>185</v>
       </c>
       <c r="K41" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2" t="s">
-        <v>249</v>
+        <v>191</v>
       </c>
       <c r="K42" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2" t="s">
-        <v>246</v>
+        <v>155</v>
       </c>
       <c r="K43" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2" t="s">
-        <v>250</v>
+        <v>12</v>
       </c>
       <c r="K44" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2" t="s">
-        <v>246</v>
+        <v>155</v>
       </c>
       <c r="K45" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2" t="s">
-        <v>246</v>
+        <v>155</v>
       </c>
       <c r="K46" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="K47" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2" t="s">
-        <v>251</v>
+        <v>222</v>
       </c>
       <c r="K48" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="K49" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="K50" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2" t="s">
-        <v>246</v>
+        <v>155</v>
       </c>
       <c r="K51" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2" t="s">
-        <v>245</v>
+        <v>135</v>
       </c>
       <c r="K52" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C53" s="2" t="b">
         <v>1</v>
@@ -3413,12 +3418,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="C54" s="2" t="b">
         <v>1</v>
@@ -3438,12 +3443,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C55" s="2" t="b">
         <v>1</v>
@@ -3463,12 +3468,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C56" s="2" t="b">
         <v>1</v>
@@ -3488,12 +3493,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C57" s="2" t="b">
         <v>1</v>
@@ -3513,12 +3518,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="C58" s="2" t="b">
         <v>1</v>
@@ -3538,12 +3543,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C59" s="2" t="b">
         <v>1</v>
@@ -3563,12 +3568,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C60" s="2" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update SG3600UD-MV-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG3600_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9702B346-4A74-364F-856B-906E18FD0E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{473BE247-2E39-1742-8E06-AA6236BB4002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05D91AD2-AC15-410D-96B8-E19C8E59AACF}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{13630C2C-D0AF-5B4B-89B4-4D2464ED7687}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -558,6 +558,9 @@
     <t xml:space="preserve"> QS4</t>
   </si>
   <si>
+    <t>A,C</t>
+  </si>
+  <si>
     <t>Which of the following are considered LOTO points when performing maintenance on a PV system with an inverter?</t>
   </si>
   <si>
@@ -620,6 +623,9 @@
     <t>Multimeter</t>
   </si>
   <si>
+    <t xml:space="preserve">A,B,C </t>
+  </si>
+  <si>
     <t>What is the replationship between resistance of NTC sensor and temperature?</t>
   </si>
   <si>
@@ -692,9 +698,6 @@
     <t>In case of extreme weather conditions like sandstorms, thunderstorms, high winds, hail, the inverter cabinet doors can still be opened.</t>
   </si>
   <si>
-    <t>During the start up of the SG3150U, the AC breakers are to be closed in immediately after they are charged. </t>
-  </si>
-  <si>
     <t>The best method to do a functional test of the E-stop button will be during a real-life operating circumstance, such as when the inverter is pushing 100% output power to the grid.</t>
   </si>
   <si>
@@ -713,16 +716,13 @@
     <t>Open circuit voltage of the PV module is directly proportional to temperature</t>
   </si>
   <si>
-    <t>A, B, C</t>
-  </si>
-  <si>
-    <t>A, C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A, B, C </t>
-  </si>
-  <si>
-    <t>A, B, C, D</t>
+    <t>A,B,C,D</t>
+  </si>
+  <si>
+    <t>A,B,C</t>
+  </si>
+  <si>
+    <t>During the start up of the SG3600U, the AC breakers are to be closed in immediately after they are charged. </t>
   </si>
 </sst>
 </file>
@@ -1110,22 +1110,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92A408F5-A3CE-3545-B152-75A361E9D8C0}">
   <dimension ref="A1:K60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
-    <col min="2" max="2" width="162.6640625" customWidth="1"/>
+    <col min="2" max="2" width="59" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="29.83203125" customWidth="1"/>
     <col min="6" max="6" width="19.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
-    <col min="8" max="8" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.25" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" customWidth="1"/>
     <col min="10" max="10" width="14.5" customWidth="1"/>
     <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1187,7 +1187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1533,7 +1533,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1549,10 +1549,10 @@
       <c r="E15" s="1">
         <v>3</v>
       </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1">
+      <c r="F15" s="1">
         <v>4</v>
       </c>
+      <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
@@ -1562,7 +1562,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>10</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>10</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>135</v>
       </c>
@@ -2020,13 +2020,13 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="K31" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>135</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>135</v>
       </c>
@@ -2080,116 +2080,116 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1" t="s">
-        <v>202</v>
+        <v>153</v>
       </c>
       <c r="K33" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I34" s="1"/>
       <c r="J34" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K34" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>202</v>
+        <v>153</v>
       </c>
       <c r="K35" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="18" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="K36" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -2202,41 +2202,41 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K38" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C39" s="1" t="b">
         <v>1</v>
@@ -2256,12 +2256,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C40" s="1" t="b">
         <v>1</v>
@@ -2281,12 +2281,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C41" s="1" t="b">
         <v>1</v>
@@ -2306,12 +2306,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C42" s="1" t="b">
         <v>1</v>
@@ -2331,12 +2331,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C43" s="1" t="b">
         <v>1</v>
@@ -2356,12 +2356,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C44" s="1" t="b">
         <v>1</v>
@@ -2381,12 +2381,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C45" s="1" t="b">
         <v>1</v>
@@ -2406,12 +2406,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C46" s="1" t="b">
         <v>1</v>
@@ -2431,12 +2431,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C47" s="1" t="b">
         <v>1</v>
@@ -2456,12 +2456,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C48" s="1" t="b">
         <v>1</v>
@@ -2481,12 +2481,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C49" s="1" t="b">
         <v>1</v>
@@ -2506,12 +2506,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C50" s="1" t="b">
         <v>1</v>
@@ -2531,12 +2531,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C51" s="1" t="b">
         <v>1</v>
@@ -2556,12 +2556,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C52" s="1" t="b">
         <v>1</v>
@@ -2581,12 +2581,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C53" s="1" t="b">
         <v>1</v>
@@ -2606,12 +2606,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C54" s="1" t="b">
         <v>1</v>
@@ -2631,12 +2631,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C55" s="1" t="b">
         <v>1</v>
@@ -2656,12 +2656,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C56" s="1" t="b">
         <v>1</v>
@@ -2681,12 +2681,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C57" s="1" t="b">
         <v>1</v>
@@ -2701,12 +2701,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C58" s="1" t="b">
         <v>1</v>
@@ -2721,12 +2721,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A59" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C59" s="1" t="b">
         <v>1</v>
@@ -2741,12 +2741,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C60" s="1" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update SG4400UD-MV question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG4400/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93179DFC-13C4-DE47-A818-F40928B52D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{26CF9F63-E7AA-9345-8D1D-DB8A760CC3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B177CD27-427C-4EC8-8ACD-E865AD4E2E3A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{B61A63DB-09B4-4E58-859D-54436AFAE0DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B61A63DB-09B4-4E58-859D-54436AFAE0DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="278">
   <si>
     <t>Type</t>
   </si>
@@ -239,6 +239,9 @@
     <t xml:space="preserve"> Ensure all safety markings and covers are in their proper location</t>
   </si>
   <si>
+    <t xml:space="preserve"> A, B, D</t>
+  </si>
+  <si>
     <t>Which of the following actions are required for safety and sealing during pre-commissioning?</t>
   </si>
   <si>
@@ -254,6 +257,9 @@
     <t xml:space="preserve"> Inspect for corrosion or oxidation inside the container</t>
   </si>
   <si>
+    <t xml:space="preserve"> A, B, C</t>
+  </si>
+  <si>
     <t>Which of the following boards should be checked during inverter component inspection?</t>
   </si>
   <si>
@@ -272,6 +278,9 @@
     <t>As part of pre-commissioning checks, which fuses need to be inspected in the auxiliary cabinet?</t>
   </si>
   <si>
+    <t xml:space="preserve"> A, B</t>
+  </si>
+  <si>
     <t>As part of pre-commissioning checks, which fuses need to be inspected in the AC cabinet?</t>
   </si>
   <si>
@@ -861,9 +870,6 @@
   </si>
   <si>
     <t>List 2 out of the 3 power sources the PE board pulls from.</t>
-  </si>
-  <si>
-    <t>A, B, D</t>
   </si>
 </sst>
 </file>
@@ -1301,18 +1307,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77B48FB6-C0BB-4CBF-AB21-AD8CBDEEA85A}">
   <dimension ref="A1:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="166.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="72.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="108.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="79.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="62.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.453125" customWidth="1"/>
+    <col min="2" max="2" width="67.81640625" customWidth="1"/>
+    <col min="3" max="3" width="32.7265625" customWidth="1"/>
+    <col min="4" max="4" width="27.90625" customWidth="1"/>
+    <col min="5" max="5" width="25.6328125" customWidth="1"/>
+    <col min="6" max="6" width="25.08984375" customWidth="1"/>
+    <col min="10" max="10" width="11.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1344,7 +1350,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
@@ -1373,7 +1379,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
@@ -1402,7 +1408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
@@ -1431,7 +1437,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
         <v>10</v>
       </c>
@@ -1460,7 +1466,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
@@ -1489,7 +1495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
@@ -1511,14 +1517,14 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="K7" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
@@ -1540,14 +1546,14 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K8" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
@@ -1569,14 +1575,14 @@
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="K9" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
@@ -1598,14 +1604,14 @@
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="K10" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="7" t="s">
         <v>10</v>
       </c>
@@ -1627,14 +1633,14 @@
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="2" t="s">
         <v>2</v>
       </c>
       <c r="K11" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A12" s="7" t="s">
         <v>10</v>
       </c>
@@ -1663,7 +1669,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="7" t="s">
         <v>23</v>
       </c>
@@ -1685,77 +1691,77 @@
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
-      <c r="J13" s="3" t="s">
-        <v>275</v>
+      <c r="J13" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="K13" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A14" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K14" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A15" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K15" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A16" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>20</v>
@@ -1773,27 +1779,27 @@
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="3" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="K16" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A17" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>20</v>
@@ -1802,96 +1808,96 @@
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K17" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A18" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K18" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A19" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
       <c r="J19" s="3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="K19" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H20" s="6"/>
       <c r="I20" s="5"/>
-      <c r="J20" s="3" t="s">
-        <v>97</v>
+      <c r="J20" s="5" t="s">
+        <v>100</v>
       </c>
       <c r="K20" s="7">
         <v>5</v>
@@ -1901,47 +1907,47 @@
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A21" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
       <c r="J21" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="K21" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A22" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
@@ -1955,18 +1961,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A23" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
@@ -1980,18 +1986,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A24" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
@@ -2005,18 +2011,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A25" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
@@ -2030,18 +2036,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
@@ -2055,18 +2061,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A27" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
@@ -2080,18 +2086,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A28" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
@@ -2105,18 +2111,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A29" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
@@ -2130,18 +2136,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
@@ -2155,12 +2161,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C31" s="6" t="b">
         <v>1</v>
@@ -2173,7 +2179,7 @@
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
       <c r="I31" s="5"/>
-      <c r="J31" s="3" t="s">
+      <c r="J31" s="5" t="s">
         <v>2</v>
       </c>
       <c r="K31" s="7">
@@ -2184,12 +2190,12 @@
       <c r="N31" s="1"/>
       <c r="O31" s="1"/>
     </row>
-    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C32" s="6" t="b">
         <v>1</v>
@@ -2202,7 +2208,7 @@
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
       <c r="I32" s="5"/>
-      <c r="J32" s="3" t="s">
+      <c r="J32" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K32" s="7">
@@ -2213,29 +2219,29 @@
       <c r="N32" s="1"/>
       <c r="O32" s="1"/>
     </row>
-    <row r="33" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
       <c r="I33" s="5"/>
-      <c r="J33" s="3" t="s">
+      <c r="J33" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K33" s="7">
@@ -2246,29 +2252,29 @@
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
     </row>
-    <row r="34" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
       <c r="I34" s="5"/>
-      <c r="J34" s="3" t="s">
+      <c r="J34" s="5" t="s">
         <v>5</v>
       </c>
       <c r="K34" s="7">
@@ -2279,29 +2285,29 @@
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
     </row>
-    <row r="35" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
       <c r="I35" s="5"/>
-      <c r="J35" s="3" t="s">
+      <c r="J35" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K35" s="7">
@@ -2312,7 +2318,7 @@
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
     </row>
-    <row r="36" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
         <v>10</v>
       </c>
@@ -2334,7 +2340,7 @@
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
       <c r="I36" s="5"/>
-      <c r="J36" s="3" t="s">
+      <c r="J36" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K36" s="7">
@@ -2345,29 +2351,29 @@
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
     </row>
-    <row r="37" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
       <c r="I37" s="5"/>
-      <c r="J37" s="3" t="s">
+      <c r="J37" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K37" s="7">
@@ -2378,29 +2384,29 @@
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
     </row>
-    <row r="38" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
       <c r="I38" s="5"/>
-      <c r="J38" s="3" t="s">
+      <c r="J38" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K38" s="7">
@@ -2411,29 +2417,29 @@
       <c r="N38" s="1"/>
       <c r="O38" s="1"/>
     </row>
-    <row r="39" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="D39" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>140</v>
-      </c>
       <c r="F39" s="6" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
       <c r="I39" s="5"/>
-      <c r="J39" s="3" t="s">
+      <c r="J39" s="5" t="s">
         <v>2</v>
       </c>
       <c r="K39" s="7">
@@ -2444,29 +2450,29 @@
       <c r="N39" s="1"/>
       <c r="O39" s="1"/>
     </row>
-    <row r="40" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
       <c r="I40" s="5"/>
-      <c r="J40" s="3" t="s">
+      <c r="J40" s="5" t="s">
         <v>2</v>
       </c>
       <c r="K40" s="7">
@@ -2477,12 +2483,12 @@
       <c r="N40" s="1"/>
       <c r="O40" s="1"/>
     </row>
-    <row r="41" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C41" s="6">
         <v>2</v>
@@ -2499,7 +2505,7 @@
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
       <c r="I41" s="5"/>
-      <c r="J41" s="3" t="s">
+      <c r="J41" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K41" s="7">
@@ -2510,29 +2516,29 @@
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
-    <row r="42" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="5"/>
-      <c r="J42" s="3" t="s">
+      <c r="J42" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K42" s="7">
@@ -2543,29 +2549,29 @@
       <c r="N42" s="1"/>
       <c r="O42" s="1"/>
     </row>
-    <row r="43" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
       <c r="I43" s="5"/>
-      <c r="J43" s="3" t="s">
+      <c r="J43" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K43" s="7">
@@ -2576,29 +2582,29 @@
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
     </row>
-    <row r="44" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
       <c r="I44" s="5"/>
-      <c r="J44" s="3" t="s">
+      <c r="J44" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K44" s="7">
@@ -2609,29 +2615,29 @@
       <c r="N44" s="1"/>
       <c r="O44" s="1"/>
     </row>
-    <row r="45" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
       <c r="I45" s="5"/>
-      <c r="J45" s="3" t="s">
+      <c r="J45" s="5" t="s">
         <v>2</v>
       </c>
       <c r="K45" s="7">
@@ -2642,29 +2648,29 @@
       <c r="N45" s="1"/>
       <c r="O45" s="1"/>
     </row>
-    <row r="46" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A46" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
       <c r="I46" s="5"/>
-      <c r="J46" s="3" t="s">
+      <c r="J46" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K46" s="7">
@@ -2675,29 +2681,29 @@
       <c r="N46" s="1"/>
       <c r="O46" s="1"/>
     </row>
-    <row r="47" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A47" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
       <c r="I47" s="5"/>
-      <c r="J47" s="3" t="s">
+      <c r="J47" s="5" t="s">
         <v>4</v>
       </c>
       <c r="K47" s="7">
@@ -2708,29 +2714,29 @@
       <c r="N47" s="1"/>
       <c r="O47" s="1"/>
     </row>
-    <row r="48" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A48" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
       <c r="I48" s="5"/>
-      <c r="J48" s="3" t="s">
+      <c r="J48" s="5" t="s">
         <v>4</v>
       </c>
       <c r="K48" s="7">
@@ -2741,12 +2747,12 @@
       <c r="N48" s="1"/>
       <c r="O48" s="1"/>
     </row>
-    <row r="49" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A49" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C49" s="6">
         <v>3</v>
@@ -2763,7 +2769,7 @@
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
       <c r="I49" s="5"/>
-      <c r="J49" s="3" t="s">
+      <c r="J49" s="5" t="s">
         <v>4</v>
       </c>
       <c r="K49" s="7">
@@ -2774,29 +2780,29 @@
       <c r="N49" s="1"/>
       <c r="O49" s="1"/>
     </row>
-    <row r="50" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A50" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
       <c r="I50" s="5"/>
-      <c r="J50" s="3" t="s">
+      <c r="J50" s="5" t="s">
         <v>3</v>
       </c>
       <c r="K50" s="7">
@@ -2807,12 +2813,12 @@
       <c r="N50" s="1"/>
       <c r="O50" s="1"/>
     </row>
-    <row r="51" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A51" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>11</v>
@@ -2824,12 +2830,12 @@
         <v>22</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
       <c r="I51" s="5"/>
-      <c r="J51" s="3" t="s">
+      <c r="J51" s="5" t="s">
         <v>5</v>
       </c>
       <c r="K51" s="7">
@@ -2840,24 +2846,24 @@
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
     </row>
-    <row r="52" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>51</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -2868,24 +2874,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -2896,24 +2902,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -2924,24 +2930,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -2952,24 +2958,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -2980,24 +2986,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -3008,24 +3014,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -3036,12 +3042,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C59" s="9">
         <v>600</v>
@@ -3064,24 +3070,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -3092,136 +3098,136 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H61" s="4"/>
       <c r="J61" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="K61" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="K62" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="H63" s="4"/>
       <c r="J63" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="K63" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="K64" s="7">
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C65" s="9" t="b">
         <v>1</v>
@@ -3240,18 +3246,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E66" s="4"/>
       <c r="F66" s="4"/>
@@ -3264,12 +3270,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C67" s="9" t="b">
         <v>1</v>
@@ -3288,12 +3294,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A68" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C68" s="9" t="b">
         <v>1</v>
@@ -3312,12 +3318,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
@@ -3329,12 +3335,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
@@ -3346,12 +3352,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
@@ -3363,12 +3369,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
@@ -3380,12 +3386,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>

</xml_diff>

<commit_message>
Update SG4400UD-MV-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG4400_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373D96C3-1DEB-8648-8E34-E92B10C7B8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{04D839C5-57CD-B64D-AB8F-2E40A6913899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0E8B13B-6D31-4B84-BA38-C6AF321B7A1E}"/>
   <bookViews>
-    <workbookView xWindow="-36220" yWindow="720" windowWidth="32300" windowHeight="21340" xr2:uid="{DEE7CDAF-3686-8344-A83E-8AE1519D283D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DEE7CDAF-3686-8344-A83E-8AE1519D283D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -839,13 +839,13 @@
     <t>Points</t>
   </si>
   <si>
+    <t>A,B,C,D</t>
+  </si>
+  <si>
     <t>B, D, E</t>
   </si>
   <si>
     <t>A, E</t>
-  </si>
-  <si>
-    <t>A, B, C, D</t>
   </si>
 </sst>
 </file>
@@ -1246,19 +1246,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B9D14F3-5CCD-E146-AD37-6ECFB6A100CC}">
   <dimension ref="A1:O78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="127.1640625" customWidth="1"/>
-    <col min="3" max="3" width="65.5" style="4" customWidth="1"/>
-    <col min="4" max="4" width="85" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="58.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.9140625" customWidth="1"/>
+    <col min="3" max="3" width="37.58203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="33" style="4" customWidth="1"/>
+    <col min="5" max="5" width="25.4140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="27.9140625" style="4" customWidth="1"/>
     <col min="7" max="7" width="22" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.5" style="4" customWidth="1"/>
     <col min="9" max="9" width="5.83203125" customWidth="1"/>
     <col min="10" max="10" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1291,7 +1292,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1324,7 +1325,7 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1357,7 +1358,7 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1390,7 +1391,7 @@
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1423,7 +1424,7 @@
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1456,7 +1457,7 @@
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1489,7 +1490,7 @@
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1522,7 +1523,7 @@
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1551,7 +1552,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1580,7 +1581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1609,7 +1610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1638,7 +1639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -1696,7 +1697,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -1725,7 +1726,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
@@ -1754,7 +1755,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1783,7 +1784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1812,7 +1813,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
@@ -1841,7 +1842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -1870,7 +1871,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
@@ -1899,7 +1900,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -1928,7 +1929,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1961,7 +1962,7 @@
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
@@ -1994,7 +1995,7 @@
       <c r="N24" s="5"/>
       <c r="O24" s="5"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>8</v>
       </c>
@@ -2027,7 +2028,7 @@
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
@@ -2060,7 +2061,7 @@
       <c r="N26" s="5"/>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
@@ -2093,7 +2094,7 @@
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>8</v>
       </c>
@@ -2126,7 +2127,7 @@
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
     </row>
-    <row r="29" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>8</v>
       </c>
@@ -2159,7 +2160,7 @@
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
@@ -2192,7 +2193,7 @@
       <c r="N30" s="5"/>
       <c r="O30" s="5"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>8</v>
       </c>
@@ -2225,7 +2226,7 @@
       <c r="N31" s="5"/>
       <c r="O31" s="5"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>8</v>
       </c>
@@ -2258,7 +2259,7 @@
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>8</v>
       </c>
@@ -2291,7 +2292,7 @@
       <c r="N33" s="5"/>
       <c r="O33" s="5"/>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>8</v>
       </c>
@@ -2324,7 +2325,7 @@
       <c r="N34" s="5"/>
       <c r="O34" s="5"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>149</v>
       </c>
@@ -2347,7 +2348,7 @@
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="K35" s="1">
         <v>5</v>
@@ -2357,7 +2358,7 @@
       <c r="N35" s="5"/>
       <c r="O35" s="5"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>149</v>
       </c>
@@ -2380,7 +2381,7 @@
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="K36" s="1">
         <v>5</v>
@@ -2390,7 +2391,7 @@
       <c r="N36" s="5"/>
       <c r="O36" s="5"/>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>8</v>
       </c>
@@ -2419,7 +2420,7 @@
       <c r="N37" s="5"/>
       <c r="O37" s="5"/>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>8</v>
       </c>
@@ -2448,7 +2449,7 @@
       <c r="N38" s="5"/>
       <c r="O38" s="5"/>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>8</v>
       </c>
@@ -2477,7 +2478,7 @@
       <c r="N39" s="5"/>
       <c r="O39" s="5"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>8</v>
       </c>
@@ -2506,7 +2507,7 @@
       <c r="N40" s="5"/>
       <c r="O40" s="5"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>8</v>
       </c>
@@ -2535,7 +2536,7 @@
       <c r="N41" s="5"/>
       <c r="O41" s="5"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>8</v>
       </c>
@@ -2564,7 +2565,7 @@
       <c r="N42" s="5"/>
       <c r="O42" s="5"/>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>8</v>
       </c>
@@ -2593,7 +2594,7 @@
       <c r="N43" s="5"/>
       <c r="O43" s="5"/>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>8</v>
       </c>
@@ -2622,7 +2623,7 @@
       <c r="N44" s="5"/>
       <c r="O44" s="5"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>8</v>
       </c>
@@ -2651,7 +2652,7 @@
       <c r="N45" s="5"/>
       <c r="O45" s="5"/>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>8</v>
       </c>
@@ -2680,7 +2681,7 @@
       <c r="N46" s="5"/>
       <c r="O46" s="5"/>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>8</v>
       </c>
@@ -2709,7 +2710,7 @@
       <c r="N47" s="5"/>
       <c r="O47" s="5"/>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -2734,7 +2735,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -2759,7 +2760,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>8</v>
       </c>
@@ -2784,7 +2785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>8</v>
       </c>
@@ -2809,7 +2810,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A52" s="1" t="s">
         <v>8</v>
       </c>
@@ -2835,7 +2836,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A53" s="1" t="s">
         <v>8</v>
       </c>
@@ -2861,7 +2862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A54" s="1" t="s">
         <v>8</v>
       </c>
@@ -2881,7 +2882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
         <v>8</v>
       </c>
@@ -2907,7 +2908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
         <v>8</v>
       </c>
@@ -2927,7 +2928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A57" s="1" t="s">
         <v>8</v>
       </c>
@@ -2953,7 +2954,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A58" s="1" t="s">
         <v>8</v>
       </c>
@@ -2979,7 +2980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A59" s="1" t="s">
         <v>8</v>
       </c>
@@ -3005,7 +3006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
         <v>8</v>
       </c>
@@ -3025,7 +3026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A61" s="1" t="s">
         <v>8</v>
       </c>
@@ -3048,7 +3049,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A62" s="1" t="s">
         <v>8</v>
       </c>
@@ -3074,7 +3075,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A63" s="1" t="s">
         <v>8</v>
       </c>
@@ -3094,7 +3095,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A64" s="1" t="s">
         <v>8</v>
       </c>
@@ -3120,7 +3121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A65" s="1" t="s">
         <v>8</v>
       </c>
@@ -3146,7 +3147,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A66" s="1" t="s">
         <v>8</v>
       </c>
@@ -3166,7 +3167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A67" s="1" t="s">
         <v>8</v>
       </c>
@@ -3192,7 +3193,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A68" s="1" t="s">
         <v>8</v>
       </c>
@@ -3218,7 +3219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A69" s="1" t="s">
         <v>8</v>
       </c>
@@ -3238,7 +3239,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A70" s="1" t="s">
         <v>8</v>
       </c>
@@ -3264,7 +3265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A71" s="1" t="s">
         <v>8</v>
       </c>
@@ -3290,7 +3291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A72" s="1" t="s">
         <v>8</v>
       </c>
@@ -3316,7 +3317,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A73" s="1" t="s">
         <v>8</v>
       </c>
@@ -3336,7 +3337,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A74" s="1" t="s">
         <v>8</v>
       </c>
@@ -3356,7 +3357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A75" s="1" t="s">
         <v>8</v>
       </c>
@@ -3382,7 +3383,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A76" s="1" t="s">
         <v>149</v>
       </c>
@@ -3405,13 +3406,13 @@
         <v>251</v>
       </c>
       <c r="J76" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K76" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
@@ -3434,13 +3435,13 @@
         <v>256</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K77" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A78" s="1" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Update SG3150U-MV question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG3150/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF952C7-5FA1-BD47-8777-23D761AEC577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{B27BC715-EFCC-6D47-A20B-CCF662CFA7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5849A3AB-35AB-4DE7-9CF5-0CC1856FB740}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{C1094EB1-E11C-4826-97C7-12D07005C403}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C1094EB1-E11C-4826-97C7-12D07005C403}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -498,6 +498,9 @@
     <t>GFDI pro</t>
   </si>
   <si>
+    <t>C,D</t>
+  </si>
+  <si>
     <t>Which of the following components that need to be checked for oil leakage during MVT commissioning stage?</t>
   </si>
   <si>
@@ -550,9 +553,6 @@
   </si>
   <si>
     <t>Explain what do you do when the DC voltage of the module exceeds the protective threshold.</t>
-  </si>
-  <si>
-    <t>C, D</t>
   </si>
 </sst>
 </file>
@@ -1444,21 +1444,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E92F6612-5B7E-41F0-8CF2-706367AFE299}">
   <dimension ref="A1:J59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="174.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="63.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="111.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.26953125" customWidth="1"/>
+    <col min="3" max="3" width="34.90625" customWidth="1"/>
+    <col min="4" max="4" width="43.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.90625" customWidth="1"/>
     <col min="6" max="6" width="51" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" customWidth="1"/>
+    <col min="8" max="8" width="7.81640625" customWidth="1"/>
     <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>8</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>8</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>8</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>8</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>8</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>8</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>8</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>8</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
         <v>8</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
         <v>8</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
         <v>8</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
         <v>8</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
         <v>9</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
         <v>9</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
         <v>9</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
         <v>9</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
         <v>9</v>
       </c>
@@ -2381,44 +2381,44 @@
         <v>145</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="J38" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J39" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -2429,12 +2429,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
@@ -2442,12 +2442,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -2458,100 +2458,100 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J43" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J44" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J45" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J46" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J47" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J48" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J49" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:10" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25"/>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="52" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="53" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="54" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="55" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="56" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="57" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="58" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
+    <row r="59" spans="1:10" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update SG3150U-MV-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG3150_safety/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG3150_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6660FD24-A09E-C749-95CE-14B32CFFF9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{6660FD24-A09E-C749-95CE-14B32CFFF9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36BEE4CF-66BF-45CB-970D-1AA2CA4F6303}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19100" xr2:uid="{0EF93C32-E07B-4E4A-AC36-FEF3B1CAF2A7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0EF93C32-E07B-4E4A-AC36-FEF3B1CAF2A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -597,9 +597,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -637,7 +637,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -743,7 +743,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -885,7 +885,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -894,15 +894,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1771CFDF-6457-A043-A19D-AE6C94909DD7}">
   <dimension ref="A1:H50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="199" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="122.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="2" max="2" width="50.75" customWidth="1"/>
+    <col min="3" max="3" width="43.75" customWidth="1"/>
+    <col min="4" max="4" width="37.9140625" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" customWidth="1"/>
+    <col min="6" max="6" width="59.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +930,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -954,7 +956,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -980,7 +982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1000,7 +1002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1022,7 +1024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1048,7 +1050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1074,7 +1076,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1100,7 +1102,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1120,7 +1122,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1140,7 +1142,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1166,7 +1168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1189,7 +1191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1215,7 +1217,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -1235,7 +1237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -1255,7 +1257,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
@@ -1275,7 +1277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1301,7 +1303,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1327,7 +1329,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
@@ -1353,7 +1355,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -1379,7 +1381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
@@ -1401,7 +1403,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -1421,7 +1423,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1447,7 +1449,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
@@ -1473,7 +1475,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>8</v>
       </c>
@@ -1499,7 +1501,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
@@ -1519,7 +1521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
@@ -1539,7 +1541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>8</v>
       </c>
@@ -1559,7 +1561,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>8</v>
       </c>
@@ -1585,7 +1587,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
@@ -1611,7 +1613,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>8</v>
       </c>
@@ -1637,7 +1639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>8</v>
       </c>
@@ -1657,7 +1659,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>98</v>
       </c>
@@ -1683,7 +1685,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>98</v>
       </c>
@@ -1709,7 +1711,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>98</v>
       </c>
@@ -1735,7 +1737,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
         <v>98</v>
       </c>
@@ -1761,7 +1763,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>98</v>
       </c>
@@ -1787,7 +1789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>125</v>
       </c>
@@ -1798,7 +1800,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>125</v>
       </c>
@@ -1809,7 +1811,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>125</v>
       </c>
@@ -1820,7 +1822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A41" s="1" t="s">
         <v>125</v>
       </c>
@@ -1831,7 +1833,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A42" s="1" t="s">
         <v>125</v>
       </c>
@@ -1842,7 +1844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A43" s="1" t="s">
         <v>125</v>
       </c>
@@ -1853,7 +1855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="1" t="s">
         <v>125</v>
       </c>
@@ -1864,7 +1866,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A45" s="1" t="s">
         <v>125</v>
       </c>
@@ -1875,7 +1877,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
         <v>125</v>
       </c>
@@ -1886,7 +1888,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
         <v>125</v>
       </c>
@@ -1897,7 +1899,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
         <v>125</v>
       </c>
@@ -1908,7 +1910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
         <v>125</v>
       </c>
@@ -1919,7 +1921,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A50" s="1" t="s">
         <v>125</v>
       </c>

</xml_diff>

<commit_message>
Update SG350HX-US question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG350/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG350/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14AC34C-8EA8-FE48-A029-E3785A12681F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B14AC34C-8EA8-FE48-A029-E3785A12681F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AAC5E5F-E54D-466B-B058-BF16459C314F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{12464BFD-7489-403B-87AC-4F10CC74C954}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{12464BFD-7489-403B-87AC-4F10CC74C954}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -893,20 +893,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F12D2C-AFB6-4394-849F-EED09355309E}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.5" customWidth="1"/>
-    <col min="2" max="2" width="131.5" customWidth="1"/>
-    <col min="3" max="3" width="44.5" customWidth="1"/>
-    <col min="4" max="4" width="41.5" customWidth="1"/>
-    <col min="5" max="5" width="44.5" customWidth="1"/>
-    <col min="6" max="6" width="27.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" customWidth="1"/>
+    <col min="2" max="2" width="59.453125" customWidth="1"/>
+    <col min="3" max="3" width="44.453125" customWidth="1"/>
+    <col min="4" max="4" width="41.453125" customWidth="1"/>
+    <col min="5" max="5" width="44.453125" customWidth="1"/>
+    <col min="6" max="6" width="27.6328125" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" customWidth="1"/>
+    <col min="8" max="9" width="13.81640625" customWidth="1"/>
+    <col min="10" max="10" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -941,7 +941,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -967,7 +967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -993,7 +993,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -1500,7 +1500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>18</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>18</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>18</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>18</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>18</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
Update SG350HX-US-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/SG350_safety/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/SG350_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A2774B-2192-C640-A3A1-10EE90D70423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{38A2774B-2192-C640-A3A1-10EE90D70423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED0EC481-24DF-41DC-8E93-BA7BE881C176}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{D88B995F-255D-AC4D-BBF8-CDAE9D204577}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D88B995F-255D-AC4D-BBF8-CDAE9D204577}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -566,9 +566,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -606,7 +606,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -712,7 +712,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -854,7 +854,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -863,10 +863,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDE9EF6-57F4-9041-8353-DDD0DBD53FBC}">
   <dimension ref="A1:H50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="2" width="151.5" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="19.1640625" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="5" width="43.5" customWidth="1"/>
@@ -874,7 +874,7 @@
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +900,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -926,7 +926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -952,7 +952,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -978,7 +978,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>117</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>117</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>117</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>117</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>117</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>148</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>148</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>148</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>148</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>148</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>148</v>
       </c>

</xml_diff>

<commit_message>
Update PT1.0-CSP question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/PT1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAF7515-CF4A-4749-ABDF-B2A003A2EBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{B24E3656-90D2-564D-A861-48F914D9A3ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13DF6596-1077-4F99-80C5-11F025069823}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="300">
   <si>
     <t>Type</t>
   </si>
@@ -926,6 +926,18 @@
   </si>
   <si>
     <t>According to the General Isolation Procedure (not to be used on site), name in order the testing points for de-energization, and what voltage mode (AC or DC) they need to be tested for. Also list, what are the 3 measurement-related equipment (not PPE) needed to safely test for de-energization.</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>K</t>
   </si>
 </sst>
 </file>
@@ -1396,7 +1408,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72ACF49E-8AF0-4AFE-A18C-12172871276B}">
   <dimension ref="A1:N37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.6640625" style="12" customWidth="1"/>
@@ -1413,7 +1425,7 @@
     <col min="13" max="13" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1438,10 +1450,18 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="I1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>299</v>
+      </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1449,7 +1469,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1475,7 +1495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1501,7 +1521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1527,7 +1547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1553,7 +1573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1579,7 +1599,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1605,7 +1625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1631,7 +1651,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1657,7 +1677,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1683,7 +1703,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1712,7 +1732,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="68" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="66" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1741,7 +1761,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="85" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="82.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1772,7 +1792,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1797,7 +1817,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1822,7 +1842,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -1847,7 +1867,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -1872,7 +1892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
         <v>103</v>
       </c>
@@ -1916,7 +1936,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
         <v>116</v>
       </c>
@@ -1927,7 +1947,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
         <v>116</v>
       </c>
@@ -1944,7 +1964,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="34" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="33" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>116</v>
       </c>
@@ -1960,7 +1980,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="32" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1980,7 +2000,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -2006,7 +2026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -2026,7 +2046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -2052,7 +2072,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
@@ -2072,7 +2092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
@@ -2092,7 +2112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>10</v>
       </c>
@@ -2118,7 +2138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
@@ -2138,7 +2158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="32" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>10</v>
       </c>
@@ -2164,7 +2184,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
@@ -2190,7 +2210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" s="8" t="s">
         <v>20</v>
       </c>
@@ -2216,7 +2236,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>10</v>
       </c>
@@ -2242,7 +2262,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
@@ -2268,7 +2288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="32" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -2294,7 +2314,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.4">
       <c r="A36" s="8" t="s">
         <v>20</v>
       </c>
@@ -2320,7 +2340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>20</v>
       </c>
@@ -2357,7 +2377,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFF6C89-8415-4E7E-B19A-AC03E2D1CEA1}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="251.6640625" bestFit="1" customWidth="1"/>
@@ -2367,7 +2387,7 @@
     <col min="6" max="6" width="42" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2402,7 +2422,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -2428,7 +2448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -2450,7 +2470,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2476,7 +2496,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -2502,7 +2522,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -2528,7 +2548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -2554,7 +2574,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -2580,7 +2600,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -2602,7 +2622,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -2628,7 +2648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -2655,7 +2675,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2680,7 +2700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
@@ -2709,7 +2729,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -2742,7 +2762,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -2770,7 +2790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -2792,7 +2812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -2820,7 +2840,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
@@ -2840,7 +2860,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
@@ -2869,7 +2889,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -2889,7 +2909,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -2915,7 +2935,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2941,7 +2961,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -2967,7 +2987,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -3004,7 +3024,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42415D1-61AD-4746-A067-51E213EE90DC}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="218.1640625" bestFit="1" customWidth="1"/>
@@ -3015,7 +3035,7 @@
     <col min="7" max="7" width="34.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3050,7 +3070,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -3076,7 +3096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -3102,7 +3122,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3128,7 +3148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -3154,7 +3174,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -3174,7 +3194,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -3200,7 +3220,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -3226,7 +3246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -3252,7 +3272,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -3278,7 +3298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -3307,7 +3327,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3342,7 +3362,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -3373,7 +3393,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -3395,7 +3415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -3417,7 +3437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -3439,7 +3459,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -3461,7 +3481,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
@@ -3481,7 +3501,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
         <v>116</v>
       </c>

</xml_diff>

<commit_message>
Update PT2.0-CSP question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/PT2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6520E602-7817-3E42-832D-30A473F46B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{33F911A6-B4F6-8642-B53B-50CABDCC397A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{370959F1-D1E4-4230-84F3-3F9FCB87266F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -245,6 +245,9 @@
     <t>Door Switch</t>
   </si>
   <si>
+    <t>A,B,D,E,F</t>
+  </si>
+  <si>
     <t>Which of the following are functions of the LC300?</t>
   </si>
   <si>
@@ -263,6 +266,9 @@
     <t>SOC Protection Parameter modification</t>
   </si>
   <si>
+    <t>A,B,E</t>
+  </si>
+  <si>
     <t>If the coolant pH falls below 7.3, it is required to replace the coolant</t>
   </si>
   <si>
@@ -489,12 +495,6 @@
   </si>
   <si>
     <t>List the following components in order of communicates. Start with the smallest level of communication: LC, BMU, BSC, CMU, SCADA</t>
-  </si>
-  <si>
-    <t>A, B, D, E, F</t>
-  </si>
-  <si>
-    <t>A, B, E</t>
   </si>
 </sst>
 </file>
@@ -913,19 +913,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42415D1-61AD-4746-A067-51E213EE90DC}">
   <dimension ref="A1:K45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="218.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.4140625" customWidth="1"/>
+    <col min="2" max="2" width="110.9140625" customWidth="1"/>
     <col min="3" max="3" width="53.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="59.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="67.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="126" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="51.08203125" customWidth="1"/>
     <col min="7" max="7" width="34.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -960,7 +959,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -986,7 +985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -1012,7 +1011,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -1064,7 +1063,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -1084,7 +1083,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -1110,7 +1109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -1136,7 +1135,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1162,7 +1161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1188,7 +1187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1217,7 +1216,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -1246,49 +1245,49 @@
         <v>68</v>
       </c>
       <c r="J12" t="s">
-        <v>151</v>
+        <v>69</v>
       </c>
       <c r="K12">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" t="s">
-        <v>152</v>
+        <v>76</v>
       </c>
       <c r="K13">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -1305,7 +1304,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1327,12 +1326,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C16" s="3" t="b">
         <v>1</v>
@@ -1349,12 +1348,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1371,7 +1370,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -1391,35 +1390,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K19">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J20" t="s">
         <v>3</v>
@@ -1428,12 +1427,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A21" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1454,24 +1453,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J22" t="s">
         <v>5</v>
@@ -1480,50 +1479,50 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D23" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E23" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" t="s">
+        <v>97</v>
+      </c>
+      <c r="J23" t="s">
+        <v>3</v>
+      </c>
+      <c r="K23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" t="s">
         <v>94</v>
       </c>
-      <c r="F23" t="s">
+      <c r="D24" t="s">
         <v>95</v>
       </c>
-      <c r="J23" t="s">
-        <v>3</v>
-      </c>
-      <c r="K23">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="E24" t="s">
         <v>96</v>
       </c>
-      <c r="C24" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" t="s">
-        <v>93</v>
-      </c>
-      <c r="E24" t="s">
-        <v>94</v>
-      </c>
       <c r="F24" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J24" t="s">
         <v>2</v>
@@ -1532,50 +1531,50 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" t="s">
+        <v>95</v>
+      </c>
+      <c r="E25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" t="s">
         <v>97</v>
       </c>
-      <c r="C25" t="s">
-        <v>92</v>
-      </c>
-      <c r="D25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="J25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A26" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" t="s">
         <v>94</v>
       </c>
-      <c r="F25" t="s">
+      <c r="D26" t="s">
         <v>95</v>
       </c>
-      <c r="J25" t="s">
-        <v>3</v>
-      </c>
-      <c r="K25">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C26" t="s">
-        <v>92</v>
-      </c>
-      <c r="D26" t="s">
-        <v>93</v>
-      </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J26" t="s">
         <v>5</v>
@@ -1584,24 +1583,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
         <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J27" t="s">
         <v>3</v>
@@ -1610,24 +1609,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F28" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J28" t="s">
         <v>4</v>
@@ -1636,18 +1635,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J29" t="s">
         <v>2</v>
@@ -1656,12 +1655,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1682,12 +1681,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C31">
         <v>6</v>
@@ -1708,12 +1707,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1734,12 +1733,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1754,24 +1753,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E34" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F34" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J34" t="s">
         <v>3</v>
@@ -1780,24 +1779,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D35" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E35" t="s">
         <v>19</v>
       </c>
       <c r="F35" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J35" t="s">
         <v>4</v>
@@ -1806,24 +1805,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D36" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E36" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F36" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J36" t="s">
         <v>3</v>
@@ -1832,12 +1831,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C37">
         <v>3</v>
@@ -1858,12 +1857,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C38">
         <v>12</v>
@@ -1884,24 +1883,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F39" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J39" t="s">
         <v>5</v>
@@ -1910,24 +1909,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D40" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F40" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J40" t="s">
         <v>4</v>
@@ -1936,24 +1935,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C41" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F41" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J41" t="s">
         <v>4</v>
@@ -1962,12 +1961,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C42" t="b">
         <v>1</v>
@@ -1982,15 +1981,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D43" t="s">
         <v>13</v>
@@ -2008,23 +2007,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="K44">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="K45">
         <v>20</v>

</xml_diff>

<commit_message>
Update PT2.0-CSP-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/PT2_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44464A6-E704-3645-974A-87EC8863A2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7808970-0D2E-0B41-B60A-C80F83897062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{E8EEE946-DEB3-4041-95C0-A3908F45A14E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E8EEE946-DEB3-4041-95C0-A3908F45A14E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -515,6 +515,9 @@
     <t>The voltage the lock is preventing from being turned on</t>
   </si>
   <si>
+    <t>A,B</t>
+  </si>
+  <si>
     <t>Can a lock be removed without contacting the person who placed the lock.</t>
   </si>
   <si>
@@ -525,9 +528,6 @@
   </si>
   <si>
     <t>If you are standing outside the arc flash boundary you can stil receive a 2nd degree burn in the event of an arc.</t>
-  </si>
-  <si>
-    <t>A, B</t>
   </si>
 </sst>
 </file>
@@ -918,12 +918,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FDD113C-2248-8C4A-9AEA-78392E6FAF4A}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -984,7 +981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -1006,7 +1003,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1032,7 +1029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -1058,7 +1055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -1084,7 +1081,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -1110,7 +1107,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -1136,7 +1133,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1158,7 +1155,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1184,7 +1181,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>45</v>
       </c>
@@ -1211,7 +1208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -1236,7 +1233,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1265,7 +1262,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
@@ -1298,7 +1295,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1326,7 +1323,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
@@ -1348,7 +1345,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -1376,7 +1373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -1396,7 +1393,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -1425,7 +1422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -1445,7 +1442,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -1471,7 +1468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>45</v>
       </c>
@@ -1497,7 +1494,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -1523,7 +1520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
@@ -1552,7 +1549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
         <v>11</v>
       </c>
@@ -1578,7 +1575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
@@ -1604,7 +1601,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
         <v>11</v>
       </c>
@@ -1630,7 +1627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
         <v>11</v>
       </c>
@@ -1650,7 +1647,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
         <v>11</v>
       </c>
@@ -1676,7 +1673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
         <v>11</v>
       </c>
@@ -1702,7 +1699,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
         <v>11</v>
       </c>
@@ -1722,7 +1719,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
         <v>11</v>
       </c>
@@ -1748,7 +1745,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
         <v>11</v>
       </c>
@@ -1768,7 +1765,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
         <v>11</v>
       </c>
@@ -1794,7 +1791,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
         <v>11</v>
       </c>
@@ -1820,7 +1817,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
         <v>11</v>
       </c>
@@ -1846,7 +1843,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
         <v>11</v>
       </c>
@@ -1866,7 +1863,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
         <v>11</v>
       </c>
@@ -1892,7 +1889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
         <v>11</v>
       </c>
@@ -1918,7 +1915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
         <v>11</v>
       </c>
@@ -1944,7 +1941,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
         <v>11</v>
       </c>
@@ -1964,7 +1961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
         <v>11</v>
       </c>
@@ -1984,7 +1981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
         <v>11</v>
       </c>
@@ -2004,7 +2001,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
         <v>11</v>
       </c>
@@ -2024,7 +2021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
         <v>11</v>
       </c>
@@ -2050,7 +2047,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A46" s="5" t="s">
         <v>11</v>
       </c>
@@ -2070,7 +2067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A47" s="5" t="s">
         <v>11</v>
       </c>
@@ -2090,7 +2087,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A48" s="5" t="s">
         <v>45</v>
       </c>
@@ -2110,24 +2107,24 @@
         <v>158</v>
       </c>
       <c r="J48" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="K48">
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A49" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C49" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D49" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J49" t="s">
         <v>3</v>
@@ -2136,12 +2133,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A50" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C50" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update Transformer question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/Transformer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9754BA-18EB-4B46-93C8-25A3FE39D259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{36587B1F-BC4E-8B48-8CCC-5F5E0A119A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFC4D75B-19D1-47DB-9DE7-A921639E7B2E}"/>
   <bookViews>
-    <workbookView xWindow="-28020" yWindow="1980" windowWidth="25500" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -543,7 +543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -554,6 +554,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -836,22 +842,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="124.6640625" customWidth="1"/>
-    <col min="3" max="3" width="63.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="124.6328125" customWidth="1"/>
+    <col min="3" max="3" width="63.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.1796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.36328125" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -883,7 +889,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -909,36 +915,36 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:11" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="5">
         <v>14253</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="5">
         <v>15243</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="5">
         <v>41523</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="5">
         <v>45213</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2" t="s">
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+      <c r="K3" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -967,7 +973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -996,7 +1002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1025,7 +1031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1054,7 +1060,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1083,7 +1089,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1112,7 +1118,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -1141,7 +1147,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -1199,7 +1205,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
@@ -1228,7 +1234,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1253,7 +1259,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1278,7 +1284,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1303,7 +1309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1328,7 +1334,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1353,7 +1359,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -1378,7 +1384,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -1403,7 +1409,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -1428,7 +1434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -1453,7 +1459,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -1478,7 +1484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>79</v>
       </c>
@@ -1497,7 +1503,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>79</v>
       </c>
@@ -1516,7 +1522,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1529,7 +1535,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>8</v>
       </c>
@@ -1562,7 +1568,7 @@
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
     </row>
-    <row r="28" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>8</v>
       </c>
@@ -1595,7 +1601,7 @@
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
     </row>
-    <row r="29" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>8</v>
       </c>
@@ -1628,7 +1634,7 @@
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
     </row>
-    <row r="30" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>8</v>
       </c>
@@ -1661,7 +1667,7 @@
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
     </row>
-    <row r="31" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>8</v>
       </c>
@@ -1694,7 +1700,7 @@
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
     </row>
-    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>8</v>
       </c>
@@ -1727,7 +1733,7 @@
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
     </row>
-    <row r="33" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>8</v>
       </c>
@@ -1760,7 +1766,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
     </row>
-    <row r="34" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>8</v>
       </c>
@@ -1793,7 +1799,7 @@
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
     </row>
-    <row r="35" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>8</v>
       </c>
@@ -1826,7 +1832,7 @@
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
     </row>
-    <row r="36" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
         <v>8</v>
       </c>
@@ -1859,7 +1865,7 @@
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
     </row>
-    <row r="37" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>8</v>
       </c>
@@ -1892,7 +1898,7 @@
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
     </row>
-    <row r="38" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>8</v>
       </c>
@@ -1925,7 +1931,7 @@
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
     </row>
-    <row r="39" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>8</v>
       </c>
@@ -1958,7 +1964,7 @@
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
     </row>
-    <row r="40" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>8</v>
       </c>
@@ -1991,7 +1997,7 @@
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
     </row>
-    <row r="41" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
         <v>8</v>
       </c>
@@ -2020,7 +2026,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="4"/>
     </row>
-    <row r="42" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="s">
         <v>8</v>
       </c>
@@ -2049,7 +2055,7 @@
       <c r="N42" s="4"/>
       <c r="O42" s="4"/>
     </row>
-    <row r="43" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>8</v>
       </c>
@@ -2078,7 +2084,7 @@
       <c r="N43" s="4"/>
       <c r="O43" s="4"/>
     </row>
-    <row r="44" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>8</v>
       </c>
@@ -2107,7 +2113,7 @@
       <c r="N44" s="4"/>
       <c r="O44" s="4"/>
     </row>
-    <row r="45" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>8</v>
       </c>
@@ -2136,7 +2142,7 @@
       <c r="N45" s="4"/>
       <c r="O45" s="4"/>
     </row>
-    <row r="46" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Update Transformer-Safety question pool from testpool2
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hebowen/Desktop/QuizSystem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/Transformer_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83867A-897A-274A-A53E-0C0454A78D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{196BE576-945B-438E-9011-CA3EC6259116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78674001-4117-4880-AB51-F4383FF44F4D}"/>
   <bookViews>
-    <workbookView xWindow="-33560" yWindow="600" windowWidth="26060" windowHeight="18220" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -215,6 +215,9 @@
     <t>Does flipping the oil switch (MVT load switch) isolate the entire HV room?</t>
   </si>
   <si>
+    <t>A,C,D,F</t>
+  </si>
+  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -389,6 +392,9 @@
     <t>Moisture</t>
   </si>
   <si>
+    <t>A,B,C</t>
+  </si>
+  <si>
     <t>What is the primary function of a four position oil switch?</t>
   </si>
   <si>
@@ -404,13 +410,7 @@
     <t>Isolate H1A from H2A</t>
   </si>
   <si>
-    <t>A, C, D, F</t>
-  </si>
-  <si>
-    <t>A, B, C</t>
-  </si>
-  <si>
-    <t>A, B, D</t>
+    <t>A,B,D</t>
   </si>
 </sst>
 </file>
@@ -825,22 +825,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E0A9B9-0213-449D-9599-DFD4E1E1084D}">
   <dimension ref="A1:O35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="124.6640625" customWidth="1"/>
-    <col min="3" max="3" width="63.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="109.81640625" customWidth="1"/>
+    <col min="3" max="3" width="63.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.1796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.33203125" customWidth="1"/>
+    <col min="7" max="7" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.26953125" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -872,7 +872,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -901,7 +901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -928,7 +928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -957,7 +957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -986,7 +986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1013,13 +1013,13 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2" t="s">
-        <v>122</v>
+        <v>59</v>
       </c>
       <c r="K6">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1243,10 +1243,10 @@
         <v>58</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -1260,24 +1260,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
@@ -1293,12 +1293,12 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
     </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17" s="4">
         <v>90</v>
@@ -1326,24 +1326,24 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -1359,24 +1359,24 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
     </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
@@ -1392,24 +1392,24 @@
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
     </row>
-    <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
@@ -1425,24 +1425,24 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
     </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
@@ -1458,24 +1458,24 @@
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
     </row>
-    <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
@@ -1491,24 +1491,24 @@
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
@@ -1524,24 +1524,24 @@
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
     </row>
-    <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
@@ -1557,12 +1557,12 @@
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
     </row>
-    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C25" s="4" t="b">
         <v>1</v>
@@ -1586,12 +1586,12 @@
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
     </row>
-    <row r="26" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C26" s="4" t="b">
         <v>1</v>
@@ -1615,12 +1615,12 @@
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
     </row>
-    <row r="27" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C27" s="4" t="b">
         <v>1</v>
@@ -1644,12 +1644,12 @@
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
     </row>
-    <row r="28" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C28" s="4" t="b">
         <v>1</v>
@@ -1673,12 +1673,12 @@
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
     </row>
-    <row r="29" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C29" s="4" t="b">
         <v>1</v>
@@ -1702,12 +1702,12 @@
       <c r="N29" s="6"/>
       <c r="O29" s="6"/>
     </row>
-    <row r="30" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C30" s="4" t="b">
         <v>1</v>
@@ -1731,12 +1731,12 @@
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
     </row>
-    <row r="31" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C31" s="4" t="b">
         <v>1</v>
@@ -1760,12 +1760,12 @@
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
     </row>
-    <row r="32" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C32" s="4" t="b">
         <v>1</v>
@@ -1789,12 +1789,12 @@
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
     </row>
-    <row r="33" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C33" s="4" t="b">
         <v>1</v>
@@ -1818,30 +1818,30 @@
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
     </row>
-    <row r="34" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K34" s="4">
         <v>5</v>
@@ -1851,24 +1851,24 @@
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
     </row>
-    <row r="35" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
@@ -1876,9 +1876,7 @@
       <c r="J35" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="K35" s="4">
-        <v>5</v>
-      </c>
+      <c r="K35" s="4"/>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
       <c r="N35" s="6"/>

</xml_diff>

<commit_message>
Update SC5000UD-MV-P3-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_49596ABF9570A0CEEB3B98154B6F6EBFA8A7ED47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E79F1BC6-F2D1-4AA1-BEE1-3EC6398CE6BC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8DE6AEC-6FEC-F949-9758-AAC64CED554F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quiz" sheetId="1" r:id="rId1"/>
@@ -25,9 +25,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>Question</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>Portable tester</t>
+  </si>
+  <si>
+    <t>Question Text</t>
   </si>
 </sst>
 </file>
@@ -543,295 +543,295 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="124.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="124.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="I2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="I2" t="s">
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" t="s">
         <v>3</v>
       </c>
-      <c r="J2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="J7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" t="s">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
-      <c r="I4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" t="s">
         <v>2</v>
       </c>
-      <c r="J6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" t="s">
-        <v>43</v>
-      </c>
-      <c r="I8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="J10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>55</v>
       </c>
-      <c r="I10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J10">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>56</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>57</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>58</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>59</v>
       </c>
-      <c r="F11" t="s">
-        <v>60</v>
-      </c>
       <c r="I11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>10</v>

</xml_diff>

<commit_message>
Update PT1.0-CSP question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/PT1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{B24E3656-90D2-564D-A861-48F914D9A3ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13DF6596-1077-4F99-80C5-11F025069823}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{B24E3656-90D2-564D-A861-48F914D9A3ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E1D8907-92B1-4C2F-BE74-822391CDFB85}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{23197B31-F529-7149-878B-230427789C59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -238,9 +238,6 @@
     <t>20 min</t>
   </si>
   <si>
-    <t>Which parameter on the LC webpage can be used to configure the IP addresses of PCS and BSC?</t>
-  </si>
-  <si>
     <t>System Parameters</t>
   </si>
   <si>
@@ -259,18 +256,12 @@
     <t>Change from Local/Remote --&gt; Local Mode</t>
   </si>
   <si>
-    <t>What is the kind of communication between BSC and CMU</t>
-  </si>
-  <si>
     <t>Daisy chain</t>
   </si>
   <si>
     <t>CAN</t>
   </si>
   <si>
-    <t>What is the default password to enter the advanced settings web interface of BSC?</t>
-  </si>
-  <si>
     <t>dp@ems100</t>
   </si>
   <si>
@@ -283,9 +274,6 @@
     <t>dp@ems400</t>
   </si>
   <si>
-    <t>Which fuses do you test when confirming zero voltage from the DC capacitors?</t>
-  </si>
-  <si>
     <t>FU1</t>
   </si>
   <si>
@@ -328,9 +316,6 @@
     <t>ECO Mode: Low power consumption mode</t>
   </si>
   <si>
-    <t>SOC parameters: LC200 will send SOC minimum protection value and SOC maximum protection value to BSC synchronously</t>
-  </si>
-  <si>
     <t>Power and grid-connection operation parameter setting</t>
   </si>
   <si>
@@ -343,12 +328,6 @@
     <t>Each powerstack must be connected to a PA board.</t>
   </si>
   <si>
-    <t>DC.DC switch two isolates maintenance power for the DC/DC itself. DC/DC Switch one isolates output power going into the Battery Collection Panel (BCP).</t>
-  </si>
-  <si>
-    <t>The LC200 inside the LC1000 can upgrade the firmware in the PT board of the PCS and the BSC.</t>
-  </si>
-  <si>
     <t>Order</t>
   </si>
   <si>
@@ -385,9 +364,6 @@
     <t>MVT Low Voltage Bushings</t>
   </si>
   <si>
-    <t>A, B, C, D, E, F, G, H, I, J, K, L</t>
-  </si>
-  <si>
     <t>Text</t>
   </si>
   <si>
@@ -928,6 +904,30 @@
     <t>According to the General Isolation Procedure (not to be used on site), name in order the testing points for de-energization, and what voltage mode (AC or DC) they need to be tested for. Also list, what are the 3 measurement-related equipment (not PPE) needed to safely test for de-energization.</t>
   </si>
   <si>
+    <t>Which parameter setting tab on the LC webpage can be used to configure the IP addresses of PCS and BSC?</t>
+  </si>
+  <si>
+    <t>What is the communication type between BSC and CMU?</t>
+  </si>
+  <si>
+    <t>What is the default password for the admin account to login to BSC?</t>
+  </si>
+  <si>
+    <t>Which fuses do you test when confirming de-energized for the DC capacitors?</t>
+  </si>
+  <si>
+    <t>SOC peotection parameters</t>
+  </si>
+  <si>
+    <t>A, C</t>
+  </si>
+  <si>
+    <t>DC.DC aux power switch isolates maintenance power for the DC/DC itself. DC Switch isolates output power going into the Battery Collection Panel (BCP).</t>
+  </si>
+  <si>
+    <t>The LC can upgrade the firmware for PCS and BSC.</t>
+  </si>
+  <si>
     <t>H</t>
   </si>
   <si>
@@ -937,7 +937,7 @@
     <t>J</t>
   </si>
   <si>
-    <t>K</t>
+    <t>E, B, D, F, J. H, I, A, C, G</t>
   </si>
 </sst>
 </file>
@@ -1408,24 +1408,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72ACF49E-8AF0-4AFE-A18C-12172871276B}">
   <dimension ref="A1:N37"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.6640625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="31.33203125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="32.1640625" style="12" customWidth="1"/>
-    <col min="5" max="5" width="26.1640625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="7.75" customWidth="1"/>
+    <col min="2" max="2" width="107.625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="31.25" style="12" customWidth="1"/>
+    <col min="4" max="4" width="32.25" style="12" customWidth="1"/>
+    <col min="5" max="5" width="26.25" style="12" customWidth="1"/>
     <col min="6" max="6" width="31.5" style="12" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.75" style="12" customWidth="1"/>
+    <col min="8" max="8" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.75" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.75" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1451,16 +1451,16 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>298</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>299</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
@@ -1469,7 +1469,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1599,44 +1599,44 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="M7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N7" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="33" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>70</v>
-      </c>
-      <c r="M7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N7" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="33" x14ac:dyDescent="0.45">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>71</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>12</v>
@@ -1651,12 +1651,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>73</v>
+        <v>289</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>51</v>
@@ -1665,36 +1665,36 @@
         <v>52</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" t="s">
+        <v>5</v>
+      </c>
+      <c r="N9" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="M9" t="s">
-        <v>5</v>
-      </c>
-      <c r="N9" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="33" x14ac:dyDescent="0.45">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="10" t="s">
+      <c r="E10" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>80</v>
       </c>
       <c r="M10" t="s">
         <v>3</v>
@@ -1703,56 +1703,56 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="M11" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="M11" t="s">
-        <v>87</v>
-      </c>
       <c r="N11">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="66" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="66" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>38</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="M12" t="s">
         <v>26</v>
@@ -1761,24 +1761,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="82.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>96</v>
+        <v>292</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -1786,18 +1786,18 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="3" t="s">
-        <v>98</v>
+        <v>293</v>
       </c>
       <c r="N13">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C14" s="14" t="b">
         <v>1</v>
@@ -1817,12 +1817,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C15" s="14" t="b">
         <v>1</v>
@@ -1842,12 +1842,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="49.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="33" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>101</v>
+        <v>294</v>
       </c>
       <c r="C16" s="14" t="b">
         <v>1</v>
@@ -1867,12 +1867,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>102</v>
+        <v>295</v>
       </c>
       <c r="C17" s="14" t="b">
         <v>1</v>
@@ -1892,67 +1892,67 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="J18" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="K18" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C18" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>114</v>
+      <c r="L18" s="11" t="s">
+        <v>102</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>115</v>
+        <v>299</v>
       </c>
       <c r="N18">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="N19">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
@@ -1964,9 +1964,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="33" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>21</v>
@@ -1980,12 +1980,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="32" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C22" s="12" t="b">
         <v>1</v>
@@ -2000,24 +2000,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="M23" t="s">
         <v>3</v>
@@ -2026,12 +2026,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C24" s="12" t="b">
         <v>1</v>
@@ -2046,21 +2046,21 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>51</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>52</v>
@@ -2072,12 +2072,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C26" s="12" t="b">
         <v>1</v>
@@ -2092,18 +2092,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="M27" t="s">
         <v>3</v>
@@ -2112,12 +2112,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C28" s="12">
         <v>4</v>
@@ -2138,12 +2138,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C29" s="12" t="b">
         <v>1</v>
@@ -2158,24 +2158,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="32" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="M30" t="s">
         <v>5</v>
@@ -2184,24 +2184,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="M31" t="s">
         <v>4</v>
@@ -2210,24 +2210,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="E32" s="12" t="s">
         <v>51</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="M32" t="s">
         <v>27</v>
@@ -2236,50 +2236,50 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
-        <v>10</v>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="M33" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="N33">
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="M34" t="s">
         <v>2</v>
@@ -2288,24 +2288,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="32" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M35" t="s">
         <v>5</v>
@@ -2314,53 +2314,53 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>49</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="M36" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="N36">
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>49</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="M37" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="N37">
         <v>5</v>
@@ -2377,17 +2377,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AFF6C89-8415-4E7E-B19A-AC03E2D1CEA1}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="251.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="251.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -2422,24 +2422,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>2</v>
@@ -2448,12 +2448,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C3" s="3" t="b">
         <v>1</v>
@@ -2470,24 +2470,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="J4" t="s">
         <v>5</v>
@@ -2496,15 +2496,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>14</v>
@@ -2522,15 +2522,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>14</v>
@@ -2548,24 +2548,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="J7" t="s">
         <v>3</v>
@@ -2574,24 +2574,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="J8" t="s">
         <v>3</v>
@@ -2600,12 +2600,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C9" s="3" t="b">
         <v>1</v>
@@ -2622,24 +2622,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="J10" t="s">
         <v>2</v>
@@ -2648,39 +2648,39 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C12" s="3" t="b">
         <v>1</v>
@@ -2700,24 +2700,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="2"/>
@@ -2729,45 +2729,45 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>36</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="K14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C15" s="3">
         <v>3</v>
@@ -2790,12 +2790,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C16" s="3" t="b">
         <v>1</v>
@@ -2812,7 +2812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -2840,12 +2840,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C18" s="3" t="b">
         <v>1</v>
@@ -2860,41 +2860,41 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="K19">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C20" s="3" t="b">
         <v>1</v>
@@ -2909,24 +2909,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="J21" t="s">
         <v>2</v>
@@ -2935,12 +2935,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>42</v>
@@ -2949,36 +2949,36 @@
         <v>40</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>41</v>
       </c>
       <c r="J22" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="K22">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="J23" t="s">
         <v>4</v>
@@ -2987,12 +2987,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>16</v>
@@ -3007,7 +3007,7 @@
         <v>19</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>3</v>
@@ -3024,18 +3024,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42415D1-61AD-4746-A067-51E213EE90DC}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="218.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="59.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="67.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="218.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="126" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -3070,24 +3070,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>3</v>
@@ -3096,21 +3096,21 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>50</v>
@@ -3122,24 +3122,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J4" t="s">
         <v>4</v>
@@ -3148,24 +3148,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="J5" t="s">
         <v>4</v>
@@ -3174,12 +3174,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="C6" s="3" t="b">
         <v>1</v>
@@ -3194,24 +3194,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="J7" t="s">
         <v>2</v>
@@ -3220,12 +3220,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="C8" s="3">
         <v>645</v>
@@ -3234,7 +3234,7 @@
         <v>690</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="F8" s="3">
         <v>480</v>
@@ -3246,24 +3246,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="J9" t="s">
         <v>3</v>
@@ -3272,24 +3272,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="J10" t="s">
         <v>2</v>
@@ -3298,27 +3298,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="J11" t="s">
         <v>48</v>
@@ -3327,78 +3327,78 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="J12" t="s">
         <v>276</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="J12" t="s">
-        <v>284</v>
       </c>
       <c r="K12">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="K13">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -3415,12 +3415,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C15" s="3" t="b">
         <v>1</v>
@@ -3437,12 +3437,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="C16" s="3" t="b">
         <v>1</v>
@@ -3459,12 +3459,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -3481,12 +3481,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C18" s="3" t="b">
         <v>1</v>
@@ -3501,12 +3501,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="K19">
         <v>20</v>

</xml_diff>

<commit_message>
Update PT1.0-CSP-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jannessa/Desktop/testpool/PT1_safety/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/lily_xu_sungrow-na_com/Documents/Desktop/testpool/testpool/PT1_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D611F50-88D7-1249-B512-799D06946B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9D611F50-88D7-1249-B512-799D06946B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB52FA90-7AED-4BAA-83D9-BF630D175126}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{F6BB879B-BAA8-D548-B6AE-4A8E8CC9CCF6}"/>
+    <workbookView xWindow="90" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BB879B-BAA8-D548-B6AE-4A8E8CC9CCF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -609,9 +609,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -649,7 +649,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -755,7 +755,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -897,7 +897,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -906,17 +906,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B7BEAE-809A-6B44-81E1-03BCF0676C22}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="1" max="1" width="7.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.796875" customWidth="1"/>
+    <col min="3" max="3" width="21.296875" customWidth="1"/>
+    <col min="4" max="4" width="21.69921875" customWidth="1"/>
+    <col min="5" max="5" width="23.69921875" customWidth="1"/>
     <col min="6" max="6" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -948,7 +948,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -970,7 +970,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -996,7 +996,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>10</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>10</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>10</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>10</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>10</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>10</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>10</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>10</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>10</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>10</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update Transformer-Safety question pool
</commit_message>
<xml_diff>
--- a/question_pool.xlsx
+++ b/question_pool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sungrowamer-my.sharepoint.com/personal/nora_guo_sungrow-na_com/Documents/Desktop/testpool/Transformer_safety/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{196BE576-945B-438E-9011-CA3EC6259116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78674001-4117-4880-AB51-F4383FF44F4D}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{196BE576-945B-438E-9011-CA3EC6259116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5132136-D944-4C23-8345-0DE4B8D5692F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{146F5E3C-24C2-4F78-B333-02FCD6E6EAB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -825,22 +825,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E0A9B9-0213-449D-9599-DFD4E1E1084D}">
   <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="109.81640625" customWidth="1"/>
-    <col min="3" max="3" width="63.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.1796875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="109.85546875" customWidth="1"/>
+    <col min="3" max="3" width="63.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.26953125" customWidth="1"/>
+    <col min="7" max="7" width="36.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" customWidth="1"/>
     <col min="10" max="10" width="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -872,7 +872,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -901,7 +901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -928,7 +928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -957,7 +957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -986,7 +986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1106,9 +1106,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>49</v>
@@ -1135,7 +1135,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
@@ -1293,7 +1293,7 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
     </row>
-    <row r="17" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
@@ -1326,7 +1326,7 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
@@ -1359,7 +1359,7 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
     </row>
-    <row r="19" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>10</v>
       </c>
@@ -1392,7 +1392,7 @@
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
     </row>
-    <row r="20" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
@@ -1425,7 +1425,7 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
     </row>
-    <row r="21" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>10</v>
       </c>
@@ -1458,7 +1458,7 @@
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
     </row>
-    <row r="22" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>10</v>
       </c>
@@ -1491,7 +1491,7 @@
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>10</v>
       </c>
@@ -1524,7 +1524,7 @@
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
     </row>
-    <row r="24" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>10</v>
       </c>
@@ -1557,7 +1557,7 @@
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
     </row>
-    <row r="25" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>10</v>
       </c>
@@ -1586,7 +1586,7 @@
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
     </row>
-    <row r="26" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>10</v>
       </c>
@@ -1615,7 +1615,7 @@
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
     </row>
-    <row r="27" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>10</v>
       </c>
@@ -1644,7 +1644,7 @@
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
     </row>
-    <row r="28" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>10</v>
       </c>
@@ -1673,7 +1673,7 @@
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
     </row>
-    <row r="29" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
@@ -1702,7 +1702,7 @@
       <c r="N29" s="6"/>
       <c r="O29" s="6"/>
     </row>
-    <row r="30" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>10</v>
       </c>
@@ -1731,7 +1731,7 @@
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
     </row>
-    <row r="31" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
     </row>
-    <row r="32" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>10</v>
       </c>
@@ -1789,7 +1789,7 @@
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
     </row>
-    <row r="33" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>10</v>
       </c>
@@ -1818,7 +1818,7 @@
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
     </row>
-    <row r="34" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>112</v>
       </c>
@@ -1851,7 +1851,7 @@
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
     </row>
-    <row r="35" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>112</v>
       </c>

</xml_diff>